<commit_message>
Added N_theta_peaks for tropical climates. Some functions for calibrating parameters. Still updating scenario details.
</commit_message>
<xml_diff>
--- a/Data/scenarios.xlsx
+++ b/Data/scenarios.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rober\Documents\GitHub Repos\merging_SFW_decomposition_models\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0685E326-0245-4A01-A949-7E17A69D6D69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B7CEA3F-8D20-45F7-B46F-555C949545E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" xr2:uid="{7C97690C-9E7B-4D0E-86C0-16835BCB4BB0}"/>
+    <workbookView xWindow="15264" yWindow="0" windowWidth="15552" windowHeight="18576" xr2:uid="{7C97690C-9E7B-4D0E-86C0-16835BCB4BB0}"/>
   </bookViews>
   <sheets>
     <sheet name="scenarios" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="765" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="787" uniqueCount="142">
   <si>
     <t>Parameter</t>
   </si>
@@ -409,9 +409,6 @@
     <t>MIMICS</t>
   </si>
   <si>
-    <t>Earthworm-Temperate</t>
-  </si>
-  <si>
     <t>LIT_1</t>
   </si>
   <si>
@@ -452,6 +449,18 @@
   </si>
   <si>
     <t>Inclusion</t>
+  </si>
+  <si>
+    <t>Voigtlaender et al.(2012) https://doi.org/10.1007/s11104-011-0982-9</t>
+  </si>
+  <si>
+    <t>Only soil feeding worm</t>
+  </si>
+  <si>
+    <t>(Laclau et al., 2010); SD is a guess</t>
+  </si>
+  <si>
+    <t>(Campoe et al., 2012)</t>
   </si>
 </sst>
 </file>
@@ -947,7 +956,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -957,6 +966,9 @@
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1057,7 +1069,13 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1759F6D4-436C-4273-8592-6F473E4E1FC6}" name="Table1" displayName="Table1" ref="A1:K120" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
-  <autoFilter ref="A1:K120" xr:uid="{1759F6D4-436C-4273-8592-6F473E4E1FC6}"/>
+  <autoFilter ref="A1:K120" xr:uid="{1759F6D4-436C-4273-8592-6F473E4E1FC6}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="Earthworm"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{9C63AD24-02BE-4FC6-8589-25FEAC9E29E1}" name="Parameter" dataDxfId="10"/>
     <tableColumn id="2" xr3:uid="{6FFFFAD3-CDDD-4A47-9019-7C5E6785F73D}" name="Scenario" dataDxfId="9"/>
@@ -1066,10 +1084,10 @@
     <tableColumn id="5" xr3:uid="{C2652975-ACD3-4499-9A4F-55E61AF86737}" name="Min" dataDxfId="6"/>
     <tableColumn id="6" xr3:uid="{9D50F876-8F5B-4BBE-BE99-655FCFAB6B55}" name="Max" dataDxfId="5"/>
     <tableColumn id="7" xr3:uid="{E3199168-8B68-4130-96B7-37F35FEADAB4}" name="Reference" dataDxfId="4"/>
-    <tableColumn id="10" xr3:uid="{7383E6E0-56E5-496B-9287-EE6E2AA3B268}" name="Help needed" dataDxfId="1"/>
-    <tableColumn id="9" xr3:uid="{5A5E5207-A16E-4A54-BB54-6D4FB1E75949}" name="Category" dataDxfId="3"/>
-    <tableColumn id="11" xr3:uid="{D48D6FAC-CC1D-441E-ACFF-3C1405C9376B}" name="Status (Case study group)" dataDxfId="0"/>
-    <tableColumn id="8" xr3:uid="{F2E55EFF-159B-4FD3-B12E-2E3149126C35}" name="Status (Rob)" dataDxfId="2"/>
+    <tableColumn id="10" xr3:uid="{7383E6E0-56E5-496B-9287-EE6E2AA3B268}" name="Help needed" dataDxfId="3"/>
+    <tableColumn id="9" xr3:uid="{5A5E5207-A16E-4A54-BB54-6D4FB1E75949}" name="Category" dataDxfId="2"/>
+    <tableColumn id="11" xr3:uid="{D48D6FAC-CC1D-441E-ACFF-3C1405C9376B}" name="Status (Case study group)" dataDxfId="1"/>
+    <tableColumn id="8" xr3:uid="{F2E55EFF-159B-4FD3-B12E-2E3149126C35}" name="Status (Rob)" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1398,7 +1416,8 @@
     <col min="1" max="1" width="17.21875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="22.77734375" customWidth="1"/>
     <col min="3" max="4" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="23" customWidth="1"/>
+    <col min="7" max="7" width="52.21875" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="23" customWidth="1"/>
     <col min="10" max="10" width="13.33203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1431,13 +1450,13 @@
         <v>79</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>12</v>
       </c>
@@ -1460,7 +1479,7 @@
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>13</v>
       </c>
@@ -1483,7 +1502,7 @@
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>14</v>
       </c>
@@ -1506,7 +1525,7 @@
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
@@ -1529,7 +1548,7 @@
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>16</v>
       </c>
@@ -1552,7 +1571,7 @@
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>17</v>
       </c>
@@ -1575,7 +1594,7 @@
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>18</v>
       </c>
@@ -1598,7 +1617,7 @@
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>19</v>
       </c>
@@ -1621,7 +1640,7 @@
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>20</v>
       </c>
@@ -1644,7 +1663,7 @@
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>21</v>
       </c>
@@ -1667,7 +1686,7 @@
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>22</v>
       </c>
@@ -1690,7 +1709,7 @@
       <c r="J12" s="1"/>
       <c r="K12" s="1"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>23</v>
       </c>
@@ -1717,7 +1736,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>25</v>
       </c>
@@ -1744,7 +1763,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>27</v>
       </c>
@@ -1771,7 +1790,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>29</v>
       </c>
@@ -1798,7 +1817,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>31</v>
       </c>
@@ -1823,7 +1842,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>32</v>
       </c>
@@ -1846,7 +1865,7 @@
       <c r="J18" s="1"/>
       <c r="K18" s="1"/>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>33</v>
       </c>
@@ -1869,7 +1888,7 @@
       <c r="J19" s="1"/>
       <c r="K19" s="1"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>35</v>
       </c>
@@ -1892,7 +1911,7 @@
       <c r="J20" s="1"/>
       <c r="K20" s="1"/>
     </row>
-    <row r="21" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>36</v>
       </c>
@@ -1915,7 +1934,7 @@
       <c r="J21" s="1"/>
       <c r="K21" s="1"/>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>37</v>
       </c>
@@ -1938,7 +1957,7 @@
       <c r="J22" s="1"/>
       <c r="K22" s="1"/>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>12</v>
       </c>
@@ -1946,22 +1965,26 @@
         <v>38</v>
       </c>
       <c r="C23" s="1">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="D23" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E23" s="1"/>
       <c r="F23" s="1"/>
-      <c r="G23" s="1"/>
+      <c r="G23" s="1" t="s">
+        <v>138</v>
+      </c>
       <c r="H23" s="1"/>
       <c r="I23" s="1" t="s">
         <v>80</v>
       </c>
       <c r="J23" s="1"/>
-      <c r="K23" s="1"/>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="K23" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>13</v>
       </c>
@@ -1969,20 +1992,24 @@
         <v>38</v>
       </c>
       <c r="C24" s="1">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="D24" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E24" s="1"/>
       <c r="F24" s="1"/>
-      <c r="G24" s="1"/>
+      <c r="G24" s="1" t="s">
+        <v>138</v>
+      </c>
       <c r="H24" s="1"/>
       <c r="I24" s="1" t="s">
         <v>80</v>
       </c>
       <c r="J24" s="1"/>
-      <c r="K24" s="1"/>
+      <c r="K24" s="1" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
@@ -1992,20 +2019,24 @@
         <v>38</v>
       </c>
       <c r="C25" s="1">
-        <v>0.3</v>
+        <v>0.18</v>
       </c>
       <c r="D25" s="1">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="E25" s="1"/>
       <c r="F25" s="1"/>
-      <c r="G25" s="1"/>
+      <c r="G25" t="s">
+        <v>140</v>
+      </c>
       <c r="H25" s="1"/>
       <c r="I25" s="1" t="s">
         <v>80</v>
       </c>
       <c r="J25" s="1"/>
-      <c r="K25" s="1"/>
+      <c r="K25" s="1" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
@@ -2015,22 +2046,26 @@
         <v>38</v>
       </c>
       <c r="C26" s="1">
-        <v>0.15</v>
+        <v>0.06</v>
       </c>
       <c r="D26" s="1">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="E26" s="1"/>
       <c r="F26" s="1"/>
-      <c r="G26" s="1"/>
+      <c r="G26" t="s">
+        <v>140</v>
+      </c>
       <c r="H26" s="1"/>
       <c r="I26" s="1" t="s">
         <v>80</v>
       </c>
       <c r="J26" s="1"/>
-      <c r="K26" s="1"/>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="K26" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>16</v>
       </c>
@@ -2038,22 +2073,26 @@
         <v>38</v>
       </c>
       <c r="C27" s="1">
-        <v>70</v>
+        <v>15</v>
       </c>
       <c r="D27" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
-      <c r="G27" s="1"/>
+      <c r="G27" s="1" t="s">
+        <v>138</v>
+      </c>
       <c r="H27" s="1"/>
       <c r="I27" s="1" t="s">
         <v>80</v>
       </c>
       <c r="J27" s="1"/>
-      <c r="K27" s="1"/>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="K27" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>17</v>
       </c>
@@ -2061,20 +2100,24 @@
         <v>38</v>
       </c>
       <c r="C28" s="1">
-        <v>0.4</v>
+        <v>0.12</v>
       </c>
       <c r="D28" s="1">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="E28" s="1"/>
       <c r="F28" s="1"/>
-      <c r="G28" s="1"/>
+      <c r="G28" s="1" t="s">
+        <v>138</v>
+      </c>
       <c r="H28" s="1"/>
       <c r="I28" s="1" t="s">
         <v>80</v>
       </c>
       <c r="J28" s="1"/>
-      <c r="K28" s="1"/>
+      <c r="K28" s="1" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
@@ -2130,20 +2173,28 @@
         <v>38</v>
       </c>
       <c r="C31" s="1">
-        <v>1270</v>
+        <v>1930</v>
       </c>
       <c r="D31" s="1">
-        <v>0</v>
-      </c>
-      <c r="E31" s="1"/>
-      <c r="F31" s="1"/>
-      <c r="G31" s="1"/>
+        <v>232</v>
+      </c>
+      <c r="E31" s="1">
+        <v>1222</v>
+      </c>
+      <c r="F31" s="1">
+        <v>1642</v>
+      </c>
+      <c r="G31" t="s">
+        <v>141</v>
+      </c>
       <c r="H31" s="1"/>
       <c r="I31" s="1" t="s">
         <v>81</v>
       </c>
       <c r="J31" s="1"/>
-      <c r="K31" s="1"/>
+      <c r="K31" s="1" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
@@ -2339,13 +2390,17 @@
       </c>
       <c r="E39" s="1"/>
       <c r="F39" s="1"/>
-      <c r="G39" s="1"/>
+      <c r="G39" s="1" t="s">
+        <v>139</v>
+      </c>
       <c r="H39" s="1"/>
       <c r="I39" s="1" t="s">
         <v>82</v>
       </c>
       <c r="J39" s="1"/>
-      <c r="K39" s="1"/>
+      <c r="K39" s="1" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
@@ -2354,8 +2409,8 @@
       <c r="B40" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C40" s="2" t="s">
-        <v>34</v>
+      <c r="C40" s="5">
+        <v>1.89202E-4</v>
       </c>
       <c r="D40" s="1">
         <v>0</v>
@@ -2385,13 +2440,17 @@
       </c>
       <c r="E41" s="1"/>
       <c r="F41" s="1"/>
-      <c r="G41" s="1"/>
+      <c r="G41" s="1" t="s">
+        <v>139</v>
+      </c>
       <c r="H41" s="1"/>
       <c r="I41" s="1" t="s">
         <v>82</v>
       </c>
       <c r="J41" s="1"/>
-      <c r="K41" s="1"/>
+      <c r="K41" s="1" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="42" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
@@ -2439,7 +2498,7 @@
       <c r="J43" s="1"/>
       <c r="K43" s="1"/>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
         <v>12</v>
       </c>
@@ -2462,7 +2521,7 @@
       <c r="J44" s="1"/>
       <c r="K44" s="1"/>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
         <v>13</v>
       </c>
@@ -2485,7 +2544,7 @@
       <c r="J45" s="1"/>
       <c r="K45" s="1"/>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
         <v>14</v>
       </c>
@@ -2508,7 +2567,7 @@
       <c r="J46" s="1"/>
       <c r="K46" s="1"/>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
         <v>15</v>
       </c>
@@ -2531,7 +2590,7 @@
       <c r="J47" s="1"/>
       <c r="K47" s="1"/>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
         <v>16</v>
       </c>
@@ -2554,7 +2613,7 @@
       <c r="J48" s="1"/>
       <c r="K48" s="1"/>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
         <v>17</v>
       </c>
@@ -2577,7 +2636,7 @@
       <c r="J49" s="1"/>
       <c r="K49" s="1"/>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
         <v>18</v>
       </c>
@@ -2600,7 +2659,7 @@
       <c r="J50" s="1"/>
       <c r="K50" s="1"/>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
         <v>19</v>
       </c>
@@ -2623,7 +2682,7 @@
       <c r="J51" s="1"/>
       <c r="K51" s="1"/>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
         <v>20</v>
       </c>
@@ -2646,7 +2705,7 @@
       <c r="J52" s="1"/>
       <c r="K52" s="1"/>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
         <v>21</v>
       </c>
@@ -2669,7 +2728,7 @@
       <c r="J53" s="1"/>
       <c r="K53" s="1"/>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
         <v>22</v>
       </c>
@@ -2692,7 +2751,7 @@
       <c r="J54" s="1"/>
       <c r="K54" s="1"/>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
         <v>42</v>
       </c>
@@ -2715,7 +2774,7 @@
       <c r="J55" s="1"/>
       <c r="K55" s="1"/>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
         <v>43</v>
       </c>
@@ -2738,7 +2797,7 @@
       <c r="J56" s="1"/>
       <c r="K56" s="1"/>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
         <v>44</v>
       </c>
@@ -2761,7 +2820,7 @@
       <c r="J57" s="1"/>
       <c r="K57" s="1"/>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58" s="1" t="s">
         <v>45</v>
       </c>
@@ -2784,7 +2843,7 @@
       <c r="J58" s="1"/>
       <c r="K58" s="1"/>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
         <v>46</v>
       </c>
@@ -2807,7 +2866,7 @@
       <c r="J59" s="1"/>
       <c r="K59" s="1"/>
     </row>
-    <row r="60" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
         <v>48</v>
       </c>
@@ -2830,7 +2889,7 @@
       <c r="J60" s="1"/>
       <c r="K60" s="1"/>
     </row>
-    <row r="61" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61" s="1" t="s">
         <v>49</v>
       </c>
@@ -2853,7 +2912,7 @@
       <c r="J61" s="1"/>
       <c r="K61" s="1"/>
     </row>
-    <row r="62" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
         <v>12</v>
       </c>
@@ -2880,7 +2939,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="63" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" s="1" t="s">
         <v>13</v>
       </c>
@@ -2907,7 +2966,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="64" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:11" ht="86.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64" s="1" t="s">
         <v>14</v>
       </c>
@@ -2934,7 +2993,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="65" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:11" ht="86.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65" s="1" t="s">
         <v>15</v>
       </c>
@@ -2961,7 +3020,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="66" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66" s="1" t="s">
         <v>16</v>
       </c>
@@ -2988,7 +3047,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="67" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67" s="1" t="s">
         <v>17</v>
       </c>
@@ -3015,7 +3074,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="68" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68" s="1" t="s">
         <v>18</v>
       </c>
@@ -3043,7 +3102,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69" s="1" t="s">
         <v>19</v>
       </c>
@@ -3074,7 +3133,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70" s="1" t="s">
         <v>20</v>
       </c>
@@ -3105,7 +3164,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71" s="1" t="s">
         <v>21</v>
       </c>
@@ -3132,7 +3191,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72" s="1" t="s">
         <v>22</v>
       </c>
@@ -3163,7 +3222,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="73" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:11" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73" s="1" t="s">
         <v>42</v>
       </c>
@@ -3190,7 +3249,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="74" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:11" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A74" s="1" t="s">
         <v>43</v>
       </c>
@@ -3217,7 +3276,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="75" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:11" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A75" s="1" t="s">
         <v>44</v>
       </c>
@@ -3244,7 +3303,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A76" s="1" t="s">
         <v>45</v>
       </c>
@@ -3269,7 +3328,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="77" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:11" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A77" s="1" t="s">
         <v>46</v>
       </c>
@@ -3296,7 +3355,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="78" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:11" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A78" s="1" t="s">
         <v>48</v>
       </c>
@@ -3323,7 +3382,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="79" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79" s="1" t="s">
         <v>49</v>
       </c>
@@ -3339,10 +3398,10 @@
       <c r="E79" s="1"/>
       <c r="F79" s="1"/>
       <c r="G79" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="H79" s="1" t="s">
         <v>135</v>
-      </c>
-      <c r="H79" s="1" t="s">
-        <v>136</v>
       </c>
       <c r="I79" s="1" t="s">
         <v>83</v>
@@ -3352,7 +3411,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="80" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A80" s="1" t="s">
         <v>12</v>
       </c>
@@ -3379,7 +3438,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="81" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81" s="1" t="s">
         <v>13</v>
       </c>
@@ -3406,7 +3465,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="82" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:11" ht="86.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A82" s="1" t="s">
         <v>14</v>
       </c>
@@ -3433,7 +3492,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="83" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:11" ht="86.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A83" s="1" t="s">
         <v>15</v>
       </c>
@@ -3460,7 +3519,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="84" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A84" s="1" t="s">
         <v>16</v>
       </c>
@@ -3487,7 +3546,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="85" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A85" s="1" t="s">
         <v>17</v>
       </c>
@@ -3514,7 +3573,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="86" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A86" s="1" t="s">
         <v>18</v>
       </c>
@@ -3542,7 +3601,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A87" s="1" t="s">
         <v>19</v>
       </c>
@@ -3573,7 +3632,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A88" s="1" t="s">
         <v>20</v>
       </c>
@@ -3604,7 +3663,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A89" s="1" t="s">
         <v>21</v>
       </c>
@@ -3631,7 +3690,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A90" s="1" t="s">
         <v>22</v>
       </c>
@@ -3662,7 +3721,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="91" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:11" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A91" s="1" t="s">
         <v>42</v>
       </c>
@@ -3689,7 +3748,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="92" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:11" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A92" s="1" t="s">
         <v>43</v>
       </c>
@@ -3716,7 +3775,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="93" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:11" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A93" s="1" t="s">
         <v>44</v>
       </c>
@@ -3743,7 +3802,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A94" s="1" t="s">
         <v>45</v>
       </c>
@@ -3768,7 +3827,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="95" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:11" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A95" s="1" t="s">
         <v>46</v>
       </c>
@@ -3795,7 +3854,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="96" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A96" s="1" t="s">
         <v>48</v>
       </c>
@@ -3820,7 +3879,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="97" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A97" s="1" t="s">
         <v>49</v>
       </c>
@@ -3836,10 +3895,10 @@
       <c r="E97" s="1"/>
       <c r="F97" s="1"/>
       <c r="G97" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="H97" s="1" t="s">
         <v>135</v>
-      </c>
-      <c r="H97" s="1" t="s">
-        <v>136</v>
       </c>
       <c r="I97" s="1" t="s">
         <v>83</v>
@@ -3849,7 +3908,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="98" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:11" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A98" s="1" t="s">
         <v>59</v>
       </c>
@@ -3876,7 +3935,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="99" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:11" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A99" s="1" t="s">
         <v>60</v>
       </c>
@@ -3903,7 +3962,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="100" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:11" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A100" s="1" t="s">
         <v>61</v>
       </c>
@@ -3930,7 +3989,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="101" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A101" s="1" t="s">
         <v>62</v>
       </c>
@@ -3955,7 +4014,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="102" spans="1:11" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:11" ht="100.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A102" s="1" t="s">
         <v>63</v>
       </c>
@@ -3982,7 +4041,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="103" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A103" s="1" t="s">
         <v>12</v>
       </c>
@@ -4012,7 +4071,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A104" s="1" t="s">
         <v>13</v>
       </c>
@@ -4042,7 +4101,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="105" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A105" s="1" t="s">
         <v>14</v>
       </c>
@@ -4072,7 +4131,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="106" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A106" s="1" t="s">
         <v>15</v>
       </c>
@@ -4102,7 +4161,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A107" s="1" t="s">
         <v>16</v>
       </c>
@@ -4132,7 +4191,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="108" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A108" s="1" t="s">
         <v>17</v>
       </c>
@@ -4162,7 +4221,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="109" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A109" s="1" t="s">
         <v>18</v>
       </c>
@@ -4192,7 +4251,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="110" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A110" s="1" t="s">
         <v>19</v>
       </c>
@@ -4222,7 +4281,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="111" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A111" s="1" t="s">
         <v>20</v>
       </c>
@@ -4252,7 +4311,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="112" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A112" s="1" t="s">
         <v>21</v>
       </c>
@@ -4282,7 +4341,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A113" s="1" t="s">
         <v>22</v>
       </c>
@@ -4312,7 +4371,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A114" s="1" t="s">
         <v>66</v>
       </c>
@@ -4342,7 +4401,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="115" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A115" s="1" t="s">
         <v>67</v>
       </c>
@@ -4373,7 +4432,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A116" s="1" t="s">
         <v>68</v>
       </c>
@@ -4403,7 +4462,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A117" s="1" t="s">
         <v>69</v>
       </c>
@@ -4433,7 +4492,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A118" s="1" t="s">
         <v>70</v>
       </c>
@@ -4458,7 +4517,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A119" s="1" t="s">
         <v>71</v>
       </c>
@@ -4488,7 +4547,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A120" s="1" t="s">
         <v>73</v>
       </c>
@@ -4528,7 +4587,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA0710C0-AB94-4FBF-AB29-E5085BC4F559}">
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.77734375" customWidth="1"/>
@@ -4563,7 +4622,7 @@
         <v>100</v>
       </c>
       <c r="B2" t="s">
-        <v>124</v>
+        <v>6</v>
       </c>
       <c r="C2" t="s">
         <v>38</v>
@@ -4605,7 +4664,7 @@
         <v>0.1</v>
       </c>
       <c r="E5" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F5" t="s">
         <v>78</v>
@@ -4619,13 +4678,13 @@
         <v>58</v>
       </c>
       <c r="C6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D6">
         <v>0.1</v>
       </c>
       <c r="E6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F6" t="s">
         <v>78</v>
@@ -4636,10 +4695,10 @@
         <v>100</v>
       </c>
       <c r="B7" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="C7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D7">
         <v>0.1</v>
@@ -4656,13 +4715,13 @@
         <v>100</v>
       </c>
       <c r="B8" t="s">
-        <v>100</v>
+        <v>65</v>
       </c>
       <c r="C8" t="s">
-        <v>114</v>
+        <v>9</v>
       </c>
       <c r="D8">
-        <v>200</v>
+        <v>0.1</v>
       </c>
       <c r="E8" t="s">
         <v>132</v>
@@ -4679,13 +4738,13 @@
         <v>100</v>
       </c>
       <c r="C9" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D9">
         <v>200</v>
       </c>
       <c r="E9" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F9" t="s">
         <v>78</v>
@@ -4699,13 +4758,13 @@
         <v>100</v>
       </c>
       <c r="C10" t="s">
-        <v>101</v>
+        <v>115</v>
       </c>
       <c r="D10">
-        <v>750</v>
+        <v>200</v>
       </c>
       <c r="E10" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F10" t="s">
         <v>78</v>
@@ -4719,13 +4778,13 @@
         <v>100</v>
       </c>
       <c r="C11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D11">
-        <v>6750</v>
+        <v>750</v>
       </c>
       <c r="E11" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F11" t="s">
         <v>78</v>
@@ -4739,13 +4798,13 @@
         <v>100</v>
       </c>
       <c r="C12" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D12">
-        <v>2500</v>
+        <v>6750</v>
       </c>
       <c r="E12" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F12" t="s">
         <v>78</v>
@@ -4753,19 +4812,19 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>116</v>
+        <v>100</v>
       </c>
       <c r="B13" t="s">
         <v>100</v>
       </c>
       <c r="C13" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D13">
-        <v>200</v>
+        <v>2500</v>
       </c>
       <c r="E13" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F13" t="s">
         <v>78</v>
@@ -4779,13 +4838,13 @@
         <v>100</v>
       </c>
       <c r="C14" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D14">
-        <v>1000</v>
+        <v>200</v>
       </c>
       <c r="E14" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F14" t="s">
         <v>78</v>
@@ -4799,13 +4858,13 @@
         <v>100</v>
       </c>
       <c r="C15" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D15">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="E15" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F15" t="s">
         <v>78</v>
@@ -4819,13 +4878,13 @@
         <v>100</v>
       </c>
       <c r="C16" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D16">
-        <v>10</v>
+        <v>2000</v>
       </c>
       <c r="E16" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F16" t="s">
         <v>78</v>
@@ -4839,13 +4898,13 @@
         <v>100</v>
       </c>
       <c r="C17" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D17">
-        <v>0.1</v>
+        <v>10</v>
       </c>
       <c r="E17" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F17" t="s">
         <v>78</v>
@@ -4859,13 +4918,13 @@
         <v>100</v>
       </c>
       <c r="C18" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D18">
-        <v>400</v>
+        <v>0.1</v>
       </c>
       <c r="E18" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F18" t="s">
         <v>78</v>
@@ -4879,13 +4938,13 @@
         <v>100</v>
       </c>
       <c r="C19" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D19">
-        <v>10</v>
+        <v>400</v>
       </c>
       <c r="E19" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F19" t="s">
         <v>78</v>
@@ -4899,13 +4958,13 @@
         <v>100</v>
       </c>
       <c r="C20" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D20">
-        <v>1000</v>
+        <v>10</v>
       </c>
       <c r="E20" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F20" t="s">
         <v>78</v>
@@ -4919,13 +4978,13 @@
         <v>100</v>
       </c>
       <c r="C21" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D21">
-        <v>3000</v>
+        <v>1000</v>
       </c>
       <c r="E21" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F21" t="s">
         <v>78</v>
@@ -4939,13 +4998,13 @@
         <v>100</v>
       </c>
       <c r="C22" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D22">
-        <v>40</v>
+        <v>3000</v>
       </c>
       <c r="E22" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F22" t="s">
         <v>78</v>
@@ -4953,19 +5012,19 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="B23" t="s">
         <v>100</v>
       </c>
       <c r="C23" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="D23">
-        <v>1000</v>
+        <v>40</v>
       </c>
       <c r="E23" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F23" t="s">
         <v>78</v>
@@ -4979,13 +5038,13 @@
         <v>100</v>
       </c>
       <c r="C24" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D24">
-        <v>210.1</v>
+        <v>1000</v>
       </c>
       <c r="E24" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F24" t="s">
         <v>78</v>
@@ -4999,13 +5058,13 @@
         <v>100</v>
       </c>
       <c r="C25" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="D25">
-        <v>2450</v>
+        <v>210.1</v>
       </c>
       <c r="E25" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F25" t="s">
         <v>78</v>
@@ -5019,13 +5078,13 @@
         <v>100</v>
       </c>
       <c r="C26" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D26">
-        <v>3000</v>
+        <v>2450</v>
       </c>
       <c r="E26" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F26" t="s">
         <v>78</v>
@@ -5039,13 +5098,13 @@
         <v>100</v>
       </c>
       <c r="C27" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D27">
-        <v>1000</v>
+        <v>3000</v>
       </c>
       <c r="E27" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F27" t="s">
         <v>78</v>
@@ -5053,19 +5112,19 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B28" t="s">
         <v>100</v>
       </c>
       <c r="C28" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="D28">
-        <v>200</v>
+        <v>1000</v>
       </c>
       <c r="E28" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F28" t="s">
         <v>78</v>
@@ -5079,13 +5138,13 @@
         <v>100</v>
       </c>
       <c r="C29" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D29">
-        <v>3000</v>
+        <v>200</v>
       </c>
       <c r="E29" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F29" t="s">
         <v>78</v>
@@ -5099,13 +5158,13 @@
         <v>100</v>
       </c>
       <c r="C30" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="D30">
-        <v>20</v>
+        <v>3000</v>
       </c>
       <c r="E30" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F30" t="s">
         <v>78</v>
@@ -5119,13 +5178,13 @@
         <v>100</v>
       </c>
       <c r="C31" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="D31">
         <v>20</v>
       </c>
       <c r="E31" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F31" t="s">
         <v>78</v>
@@ -5139,13 +5198,13 @@
         <v>100</v>
       </c>
       <c r="C32" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D32">
-        <v>400</v>
+        <v>20</v>
       </c>
       <c r="E32" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F32" t="s">
         <v>78</v>
@@ -5159,13 +5218,13 @@
         <v>100</v>
       </c>
       <c r="C33" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D33">
-        <v>1000</v>
+        <v>400</v>
       </c>
       <c r="E33" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F33" t="s">
         <v>78</v>
@@ -5179,15 +5238,35 @@
         <v>100</v>
       </c>
       <c r="C34" t="s">
+        <v>129</v>
+      </c>
+      <c r="D34">
+        <v>1000</v>
+      </c>
+      <c r="E34" t="s">
         <v>131</v>
       </c>
-      <c r="D34">
+      <c r="F34" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>123</v>
+      </c>
+      <c r="B35" t="s">
+        <v>100</v>
+      </c>
+      <c r="C35" t="s">
+        <v>130</v>
+      </c>
+      <c r="D35">
         <v>3000</v>
       </c>
-      <c r="E34" t="s">
-        <v>132</v>
-      </c>
-      <c r="F34" t="s">
+      <c r="E35" t="s">
+        <v>131</v>
+      </c>
+      <c r="F35" t="s">
         <v>78</v>
       </c>
     </row>
@@ -5213,7 +5292,7 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Cleaning up the directory.
</commit_message>
<xml_diff>
--- a/Data/scenarios.xlsx
+++ b/Data/scenarios.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rober\Documents\GitHub Repos\merging_SFW_decomposition_models\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B7CEA3F-8D20-45F7-B46F-555C949545E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD298E47-FD00-48D1-8D6C-3DDDD486F975}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" activeTab="1" xr2:uid="{7C97690C-9E7B-4D0E-86C0-16835BCB4BB0}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" activeTab="2" xr2:uid="{7C97690C-9E7B-4D0E-86C0-16835BCB4BB0}"/>
   </bookViews>
   <sheets>
     <sheet name="scenarios" sheetId="1" r:id="rId1"/>
@@ -55,9 +55,6 @@
     <t>Tree</t>
   </si>
   <si>
-    <t>Earthworm - Temperate</t>
-  </si>
-  <si>
     <t>Herb</t>
   </si>
   <si>
@@ -461,6 +458,9 @@
   </si>
   <si>
     <t>(Campoe et al., 2012)</t>
+  </si>
+  <si>
+    <t>EarthwormTemperate</t>
   </si>
 </sst>
 </file>
@@ -1069,13 +1069,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1759F6D4-436C-4273-8592-6F473E4E1FC6}" name="Table1" displayName="Table1" ref="A1:K120" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
-  <autoFilter ref="A1:K120" xr:uid="{1759F6D4-436C-4273-8592-6F473E4E1FC6}">
-    <filterColumn colId="1">
-      <filters>
-        <filter val="Earthworm"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:K120" xr:uid="{1759F6D4-436C-4273-8592-6F473E4E1FC6}"/>
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{9C63AD24-02BE-4FC6-8589-25FEAC9E29E1}" name="Parameter" dataDxfId="10"/>
     <tableColumn id="2" xr3:uid="{6FFFFAD3-CDDD-4A47-9019-7C5E6785F73D}" name="Scenario" dataDxfId="9"/>
@@ -1435,33 +1429,33 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>75</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>76</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>6</v>
+        <v>141</v>
       </c>
       <c r="C2" s="1">
         <v>6</v>
@@ -1474,17 +1468,17 @@
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
       <c r="I2" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
     </row>
-    <row r="3" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>6</v>
+        <v>141</v>
       </c>
       <c r="C3" s="1">
         <v>26</v>
@@ -1497,17 +1491,17 @@
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
       <c r="I3" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
     </row>
-    <row r="4" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>6</v>
+        <v>141</v>
       </c>
       <c r="C4" s="1">
         <v>0.3</v>
@@ -1520,17 +1514,17 @@
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
       <c r="I4" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
     </row>
-    <row r="5" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>6</v>
+        <v>141</v>
       </c>
       <c r="C5" s="1">
         <v>0.15</v>
@@ -1543,17 +1537,17 @@
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
       <c r="I5" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
     </row>
-    <row r="6" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>6</v>
+        <v>141</v>
       </c>
       <c r="C6" s="1">
         <v>70</v>
@@ -1566,17 +1560,17 @@
       <c r="G6" s="1"/>
       <c r="H6" s="1"/>
       <c r="I6" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
     </row>
-    <row r="7" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>6</v>
+        <v>141</v>
       </c>
       <c r="C7" s="1">
         <v>0.4</v>
@@ -1589,17 +1583,17 @@
       <c r="G7" s="1"/>
       <c r="H7" s="1"/>
       <c r="I7" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
     </row>
-    <row r="8" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>6</v>
+        <v>141</v>
       </c>
       <c r="C8" s="1">
         <v>0.2</v>
@@ -1612,17 +1606,17 @@
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
       <c r="I8" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
     </row>
-    <row r="9" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>6</v>
+        <v>141</v>
       </c>
       <c r="C9" s="1">
         <v>50</v>
@@ -1635,17 +1629,17 @@
       <c r="G9" s="1"/>
       <c r="H9" s="1"/>
       <c r="I9" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
     </row>
-    <row r="10" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>6</v>
+        <v>141</v>
       </c>
       <c r="C10" s="1">
         <v>1270</v>
@@ -1658,17 +1652,17 @@
       <c r="G10" s="1"/>
       <c r="H10" s="1"/>
       <c r="I10" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
     </row>
-    <row r="11" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>6</v>
+        <v>141</v>
       </c>
       <c r="C11" s="1">
         <v>6</v>
@@ -1681,17 +1675,17 @@
       <c r="G11" s="1"/>
       <c r="H11" s="1"/>
       <c r="I11" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
     </row>
-    <row r="12" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>6</v>
+        <v>141</v>
       </c>
       <c r="C12" s="1">
         <v>1300</v>
@@ -1704,17 +1698,17 @@
       <c r="G12" s="1"/>
       <c r="H12" s="1"/>
       <c r="I12" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J12" s="1"/>
       <c r="K12" s="1"/>
     </row>
-    <row r="13" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>6</v>
+        <v>141</v>
       </c>
       <c r="C13" s="1">
         <v>1.1000000000000001E-3</v>
@@ -1725,23 +1719,23 @@
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
       <c r="G13" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H13" s="1"/>
       <c r="I13" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J13" s="1"/>
       <c r="K13" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>6</v>
+        <v>141</v>
       </c>
       <c r="C14" s="1">
         <v>0.53</v>
@@ -1752,23 +1746,23 @@
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
       <c r="G14" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H14" s="1"/>
       <c r="I14" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J14" s="1"/>
       <c r="K14" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>6</v>
+        <v>141</v>
       </c>
       <c r="C15" s="1">
         <v>0.09</v>
@@ -1779,23 +1773,23 @@
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
       <c r="G15" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H15" s="1"/>
       <c r="I15" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J15" s="1"/>
       <c r="K15" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>6</v>
+        <v>141</v>
       </c>
       <c r="C16" s="1">
         <v>0.22</v>
@@ -1806,23 +1800,23 @@
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
       <c r="G16" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H16" s="1"/>
       <c r="I16" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J16" s="1"/>
       <c r="K16" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>6</v>
+        <v>141</v>
       </c>
       <c r="C17" s="1">
         <v>0</v>
@@ -1835,19 +1829,19 @@
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
       <c r="I17" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J17" s="1"/>
       <c r="K17" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>6</v>
+        <v>141</v>
       </c>
       <c r="C18" s="1">
         <v>0</v>
@@ -1860,20 +1854,20 @@
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
       <c r="I18" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J18" s="1"/>
       <c r="K18" s="1"/>
     </row>
-    <row r="19" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>33</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>34</v>
       </c>
       <c r="D19" s="1">
         <v>0</v>
@@ -1883,17 +1877,17 @@
       <c r="G19" s="1"/>
       <c r="H19" s="1"/>
       <c r="I19" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J19" s="1"/>
       <c r="K19" s="1"/>
     </row>
-    <row r="20" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>6</v>
+        <v>141</v>
       </c>
       <c r="C20" s="1">
         <v>0</v>
@@ -1906,17 +1900,17 @@
       <c r="G20" s="1"/>
       <c r="H20" s="1"/>
       <c r="I20" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J20" s="1"/>
       <c r="K20" s="1"/>
     </row>
-    <row r="21" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>6</v>
+        <v>141</v>
       </c>
       <c r="C21" s="1">
         <v>0</v>
@@ -1929,17 +1923,17 @@
       <c r="G21" s="1"/>
       <c r="H21" s="1"/>
       <c r="I21" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J21" s="1"/>
       <c r="K21" s="1"/>
     </row>
-    <row r="22" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>6</v>
+        <v>141</v>
       </c>
       <c r="C22" s="1">
         <v>-0.02</v>
@@ -1952,17 +1946,17 @@
       <c r="G22" s="1"/>
       <c r="H22" s="1"/>
       <c r="I22" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J22" s="1"/>
       <c r="K22" s="1"/>
     </row>
-    <row r="23" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C23" s="1">
         <v>19</v>
@@ -1973,23 +1967,23 @@
       <c r="E23" s="1"/>
       <c r="F23" s="1"/>
       <c r="G23" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H23" s="1"/>
       <c r="I23" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J23" s="1"/>
       <c r="K23" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C24" s="1">
         <v>15</v>
@@ -2000,23 +1994,23 @@
       <c r="E24" s="1"/>
       <c r="F24" s="1"/>
       <c r="G24" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H24" s="1"/>
       <c r="I24" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J24" s="1"/>
       <c r="K24" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C25" s="1">
         <v>0.18</v>
@@ -2027,23 +2021,23 @@
       <c r="E25" s="1"/>
       <c r="F25" s="1"/>
       <c r="G25" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="H25" s="1"/>
       <c r="I25" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J25" s="1"/>
       <c r="K25" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C26" s="1">
         <v>0.06</v>
@@ -2054,23 +2048,23 @@
       <c r="E26" s="1"/>
       <c r="F26" s="1"/>
       <c r="G26" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="H26" s="1"/>
       <c r="I26" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J26" s="1"/>
       <c r="K26" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="27" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C27" s="1">
         <v>15</v>
@@ -2081,23 +2075,23 @@
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
       <c r="G27" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H27" s="1"/>
       <c r="I27" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J27" s="1"/>
       <c r="K27" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C28" s="1">
         <v>0.12</v>
@@ -2108,23 +2102,23 @@
       <c r="E28" s="1"/>
       <c r="F28" s="1"/>
       <c r="G28" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H28" s="1"/>
       <c r="I28" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J28" s="1"/>
       <c r="K28" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C29" s="1">
         <v>0.2</v>
@@ -2137,17 +2131,17 @@
       <c r="G29" s="1"/>
       <c r="H29" s="1"/>
       <c r="I29" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J29" s="1"/>
       <c r="K29" s="1"/>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C30" s="1">
         <v>50</v>
@@ -2160,17 +2154,17 @@
       <c r="G30" s="1"/>
       <c r="H30" s="1"/>
       <c r="I30" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="J30" s="1"/>
       <c r="K30" s="1"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C31" s="1">
         <v>1930</v>
@@ -2185,23 +2179,23 @@
         <v>1642</v>
       </c>
       <c r="G31" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="H31" s="1"/>
       <c r="I31" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="J31" s="1"/>
       <c r="K31" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C32" s="1">
         <v>6</v>
@@ -2214,17 +2208,17 @@
       <c r="G32" s="1"/>
       <c r="H32" s="1"/>
       <c r="I32" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J32" s="1"/>
       <c r="K32" s="1"/>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C33" s="1">
         <v>1300</v>
@@ -2237,17 +2231,17 @@
       <c r="G33" s="1"/>
       <c r="H33" s="1"/>
       <c r="I33" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J33" s="1"/>
       <c r="K33" s="1"/>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C34" s="1">
         <v>1.5598291E-2</v>
@@ -2258,23 +2252,23 @@
       <c r="E34" s="1"/>
       <c r="F34" s="1"/>
       <c r="G34" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H34" s="1"/>
       <c r="I34" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J34" s="1"/>
       <c r="K34" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C35" s="1">
         <v>0.53</v>
@@ -2285,23 +2279,23 @@
       <c r="E35" s="1"/>
       <c r="F35" s="1"/>
       <c r="G35" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H35" s="1"/>
       <c r="I35" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J35" s="1"/>
       <c r="K35" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C36" s="1">
         <v>0.09</v>
@@ -2312,23 +2306,23 @@
       <c r="E36" s="1"/>
       <c r="F36" s="1"/>
       <c r="G36" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H36" s="1"/>
       <c r="I36" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J36" s="1"/>
       <c r="K36" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C37" s="1">
         <v>5.2999999999999999E-2</v>
@@ -2339,23 +2333,23 @@
       <c r="E37" s="1"/>
       <c r="F37" s="1"/>
       <c r="G37" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H37" s="1"/>
       <c r="I37" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J37" s="1"/>
       <c r="K37" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C38" s="1">
         <v>0</v>
@@ -2368,19 +2362,19 @@
       <c r="G38" s="1"/>
       <c r="H38" s="1"/>
       <c r="I38" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J38" s="1"/>
       <c r="K38" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C39" s="1">
         <v>0</v>
@@ -2391,23 +2385,23 @@
       <c r="E39" s="1"/>
       <c r="F39" s="1"/>
       <c r="G39" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="H39" s="1"/>
       <c r="I39" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J39" s="1"/>
       <c r="K39" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C40" s="5">
         <v>1.89202E-4</v>
@@ -2420,17 +2414,17 @@
       <c r="G40" s="1"/>
       <c r="H40" s="1"/>
       <c r="I40" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J40" s="1"/>
       <c r="K40" s="1"/>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C41" s="1">
         <v>0</v>
@@ -2441,23 +2435,23 @@
       <c r="E41" s="1"/>
       <c r="F41" s="1"/>
       <c r="G41" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="H41" s="1"/>
       <c r="I41" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J41" s="1"/>
       <c r="K41" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="42" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C42" s="1">
         <v>0</v>
@@ -2470,17 +2464,17 @@
       <c r="G42" s="1"/>
       <c r="H42" s="1"/>
       <c r="I42" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J42" s="1"/>
       <c r="K42" s="1"/>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B43" s="1" t="s">
         <v>37</v>
-      </c>
-      <c r="B43" s="1" t="s">
-        <v>38</v>
       </c>
       <c r="C43" s="1">
         <v>-0.02</v>
@@ -2493,17 +2487,17 @@
       <c r="G43" s="1"/>
       <c r="H43" s="1"/>
       <c r="I43" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J43" s="1"/>
       <c r="K43" s="1"/>
     </row>
-    <row r="44" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C44" s="1">
         <v>6</v>
@@ -2516,17 +2510,17 @@
       <c r="G44" s="1"/>
       <c r="H44" s="1"/>
       <c r="I44" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J44" s="1"/>
       <c r="K44" s="1"/>
     </row>
-    <row r="45" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C45" s="1">
         <v>26</v>
@@ -2539,17 +2533,17 @@
       <c r="G45" s="1"/>
       <c r="H45" s="1"/>
       <c r="I45" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J45" s="1"/>
       <c r="K45" s="1"/>
     </row>
-    <row r="46" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C46" s="1">
         <v>0.3</v>
@@ -2562,17 +2556,17 @@
       <c r="G46" s="1"/>
       <c r="H46" s="1"/>
       <c r="I46" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J46" s="1"/>
       <c r="K46" s="1"/>
     </row>
-    <row r="47" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C47" s="1">
         <v>0.15</v>
@@ -2585,17 +2579,17 @@
       <c r="G47" s="1"/>
       <c r="H47" s="1"/>
       <c r="I47" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J47" s="1"/>
       <c r="K47" s="1"/>
     </row>
-    <row r="48" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C48" s="1">
         <v>70</v>
@@ -2608,17 +2602,17 @@
       <c r="G48" s="1"/>
       <c r="H48" s="1"/>
       <c r="I48" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J48" s="1"/>
       <c r="K48" s="1"/>
     </row>
-    <row r="49" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C49" s="1">
         <v>0.4</v>
@@ -2631,17 +2625,17 @@
       <c r="G49" s="1"/>
       <c r="H49" s="1"/>
       <c r="I49" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J49" s="1"/>
       <c r="K49" s="1"/>
     </row>
-    <row r="50" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C50" s="1">
         <v>0.2</v>
@@ -2654,17 +2648,17 @@
       <c r="G50" s="1"/>
       <c r="H50" s="1"/>
       <c r="I50" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J50" s="1"/>
       <c r="K50" s="1"/>
     </row>
-    <row r="51" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C51" s="1">
         <v>50</v>
@@ -2677,17 +2671,17 @@
       <c r="G51" s="1"/>
       <c r="H51" s="1"/>
       <c r="I51" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="J51" s="1"/>
       <c r="K51" s="1"/>
     </row>
-    <row r="52" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C52" s="1">
         <v>1270</v>
@@ -2700,17 +2694,17 @@
       <c r="G52" s="1"/>
       <c r="H52" s="1"/>
       <c r="I52" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="J52" s="1"/>
       <c r="K52" s="1"/>
     </row>
-    <row r="53" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C53" s="1">
         <v>6</v>
@@ -2723,17 +2717,17 @@
       <c r="G53" s="1"/>
       <c r="H53" s="1"/>
       <c r="I53" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J53" s="1"/>
       <c r="K53" s="1"/>
     </row>
-    <row r="54" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C54" s="1">
         <v>1300</v>
@@ -2746,17 +2740,17 @@
       <c r="G54" s="1"/>
       <c r="H54" s="1"/>
       <c r="I54" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J54" s="1"/>
       <c r="K54" s="1"/>
     </row>
-    <row r="55" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C55" s="1">
         <v>0.1</v>
@@ -2769,17 +2763,17 @@
       <c r="G55" s="1"/>
       <c r="H55" s="1"/>
       <c r="I55" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J55" s="1"/>
       <c r="K55" s="1"/>
     </row>
-    <row r="56" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C56" s="1">
         <v>0.5</v>
@@ -2792,17 +2786,17 @@
       <c r="G56" s="1"/>
       <c r="H56" s="1"/>
       <c r="I56" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J56" s="1"/>
       <c r="K56" s="1"/>
     </row>
-    <row r="57" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C57" s="1">
         <v>0.35</v>
@@ -2815,17 +2809,17 @@
       <c r="G57" s="1"/>
       <c r="H57" s="1"/>
       <c r="I57" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J57" s="1"/>
       <c r="K57" s="1"/>
     </row>
-    <row r="58" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A58" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C58" s="1">
         <v>0</v>
@@ -2838,20 +2832,20 @@
       <c r="G58" s="1"/>
       <c r="H58" s="1"/>
       <c r="I58" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J58" s="1"/>
       <c r="K58" s="1"/>
     </row>
-    <row r="59" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C59" s="2" t="s">
         <v>46</v>
-      </c>
-      <c r="B59" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C59" s="2" t="s">
-        <v>47</v>
       </c>
       <c r="D59" s="1">
         <v>0</v>
@@ -2861,17 +2855,17 @@
       <c r="G59" s="1"/>
       <c r="H59" s="1"/>
       <c r="I59" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J59" s="1"/>
       <c r="K59" s="1"/>
     </row>
-    <row r="60" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C60" s="1">
         <v>6.0100000000000001E-2</v>
@@ -2884,17 +2878,17 @@
       <c r="G60" s="1"/>
       <c r="H60" s="1"/>
       <c r="I60" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J60" s="1"/>
       <c r="K60" s="1"/>
     </row>
-    <row r="61" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A61" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C61" s="1">
         <v>0</v>
@@ -2907,17 +2901,17 @@
       <c r="G61" s="1"/>
       <c r="H61" s="1"/>
       <c r="I61" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J61" s="1"/>
       <c r="K61" s="1"/>
     </row>
-    <row r="62" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C62" s="1">
         <v>12</v>
@@ -2928,23 +2922,23 @@
       <c r="E62" s="1"/>
       <c r="F62" s="1"/>
       <c r="G62" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H62" s="1"/>
       <c r="I62" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J62" s="1"/>
       <c r="K62" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="63" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A63" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C63" s="1">
         <v>20</v>
@@ -2955,23 +2949,23 @@
       <c r="E63" s="1"/>
       <c r="F63" s="1"/>
       <c r="G63" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H63" s="1"/>
       <c r="I63" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J63" s="1"/>
       <c r="K63" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="64" spans="1:11" ht="86.4" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A64" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C64" s="1">
         <v>0.2</v>
@@ -2982,23 +2976,23 @@
       <c r="E64" s="1"/>
       <c r="F64" s="1"/>
       <c r="G64" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H64" s="1"/>
       <c r="I64" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J64" s="1"/>
       <c r="K64" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="65" spans="1:11" ht="86.4" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A65" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C65" s="1">
         <v>0.1</v>
@@ -3009,23 +3003,23 @@
       <c r="E65" s="1"/>
       <c r="F65" s="1"/>
       <c r="G65" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H65" s="1"/>
       <c r="I65" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J65" s="1"/>
       <c r="K65" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="66" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A66" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C66" s="1">
         <v>0.45</v>
@@ -3036,23 +3030,23 @@
       <c r="E66" s="1"/>
       <c r="F66" s="1"/>
       <c r="G66" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H66" s="1"/>
       <c r="I66" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J66" s="1"/>
       <c r="K66" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="67" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A67" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C67" s="1">
         <v>0.22</v>
@@ -3063,23 +3057,23 @@
       <c r="E67" s="1"/>
       <c r="F67" s="1"/>
       <c r="G67" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H67" s="1"/>
       <c r="I67" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J67" s="1"/>
       <c r="K67" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="68" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A68" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C68" s="1">
         <v>0.21</v>
@@ -3091,23 +3085,23 @@
       <c r="E68" s="1"/>
       <c r="F68" s="1"/>
       <c r="G68" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H68" s="1"/>
       <c r="I68" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J68" s="1"/>
       <c r="K68" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="69" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A69" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C69" s="1">
         <v>212</v>
@@ -3122,23 +3116,23 @@
         <v>290</v>
       </c>
       <c r="G69" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H69" s="1"/>
       <c r="I69" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="J69" s="1"/>
       <c r="K69" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="70" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A70" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C70" s="1">
         <v>1428</v>
@@ -3153,23 +3147,23 @@
         <v>1481</v>
       </c>
       <c r="G70" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H70" s="1"/>
       <c r="I70" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="J70" s="1"/>
       <c r="K70" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="71" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A71" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C71" s="1">
         <v>6</v>
@@ -3180,23 +3174,23 @@
       <c r="E71" s="1"/>
       <c r="F71" s="1"/>
       <c r="G71" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H71" s="3"/>
       <c r="I71" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J71" s="1"/>
       <c r="K71" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="72" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A72" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C72" s="1">
         <v>880</v>
@@ -3211,23 +3205,23 @@
         <v>960</v>
       </c>
       <c r="G72" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H72" s="3"/>
       <c r="I72" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J72" s="1"/>
       <c r="K72" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="73" spans="1:11" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A73" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C73" s="1">
         <v>5.7999999999999996E-3</v>
@@ -3238,23 +3232,23 @@
       <c r="E73" s="1"/>
       <c r="F73" s="1"/>
       <c r="G73" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H73" s="1"/>
       <c r="I73" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J73" s="1"/>
       <c r="K73" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="74" spans="1:11" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A74" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C74" s="1">
         <v>0.50930200000000003</v>
@@ -3265,23 +3259,23 @@
       <c r="E74" s="1"/>
       <c r="F74" s="1"/>
       <c r="G74" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H74" s="1"/>
       <c r="I74" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J74" s="1"/>
       <c r="K74" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="75" spans="1:11" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A75" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C75" s="1">
         <v>0.35</v>
@@ -3292,23 +3286,23 @@
       <c r="E75" s="1"/>
       <c r="F75" s="1"/>
       <c r="G75" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H75" s="1"/>
       <c r="I75" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J75" s="1"/>
       <c r="K75" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="76" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A76" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C76" s="1">
         <v>0</v>
@@ -3321,22 +3315,22 @@
       <c r="G76" s="1"/>
       <c r="H76" s="1"/>
       <c r="I76" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J76" s="1"/>
       <c r="K76" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="77" spans="1:11" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A77" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D77" s="1">
         <v>0</v>
@@ -3344,23 +3338,23 @@
       <c r="E77" s="1"/>
       <c r="F77" s="1"/>
       <c r="G77" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H77" s="1"/>
       <c r="I77" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J77" s="1"/>
       <c r="K77" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="78" spans="1:11" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A78" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C78" s="1">
         <v>6.0100000000000001E-2</v>
@@ -3371,23 +3365,23 @@
       <c r="E78" s="1"/>
       <c r="F78" s="1"/>
       <c r="G78" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="H78" s="1"/>
       <c r="I78" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J78" s="1"/>
       <c r="K78" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="79" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A79" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B79" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="B79" s="1" t="s">
-        <v>50</v>
       </c>
       <c r="C79" s="1">
         <v>6.0100000000000001E-2</v>
@@ -3398,25 +3392,25 @@
       <c r="E79" s="1"/>
       <c r="F79" s="1"/>
       <c r="G79" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="H79" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="H79" s="1" t="s">
-        <v>135</v>
-      </c>
       <c r="I79" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J79" s="1"/>
       <c r="K79" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="80" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A80" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C80" s="1">
         <v>12</v>
@@ -3427,23 +3421,23 @@
       <c r="E80" s="1"/>
       <c r="F80" s="1"/>
       <c r="G80" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H80" s="1"/>
       <c r="I80" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J80" s="1"/>
       <c r="K80" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="81" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A81" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C81" s="1">
         <v>20</v>
@@ -3454,23 +3448,23 @@
       <c r="E81" s="1"/>
       <c r="F81" s="1"/>
       <c r="G81" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H81" s="1"/>
       <c r="I81" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J81" s="1"/>
       <c r="K81" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="82" spans="1:11" ht="86.4" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A82" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C82" s="1">
         <v>0.2</v>
@@ -3481,23 +3475,23 @@
       <c r="E82" s="1"/>
       <c r="F82" s="1"/>
       <c r="G82" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H82" s="1"/>
       <c r="I82" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J82" s="1"/>
       <c r="K82" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="83" spans="1:11" ht="86.4" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A83" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C83" s="1">
         <v>0.1</v>
@@ -3508,23 +3502,23 @@
       <c r="E83" s="1"/>
       <c r="F83" s="1"/>
       <c r="G83" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H83" s="1"/>
       <c r="I83" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J83" s="1"/>
       <c r="K83" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="84" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="84" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A84" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C84" s="1">
         <v>0.45</v>
@@ -3535,23 +3529,23 @@
       <c r="E84" s="1"/>
       <c r="F84" s="1"/>
       <c r="G84" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H84" s="1"/>
       <c r="I84" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J84" s="1"/>
       <c r="K84" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="85" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="85" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A85" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C85" s="1">
         <v>0.22</v>
@@ -3562,23 +3556,23 @@
       <c r="E85" s="1"/>
       <c r="F85" s="1"/>
       <c r="G85" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H85" s="1"/>
       <c r="I85" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J85" s="1"/>
       <c r="K85" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="86" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="86" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A86" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C86" s="1">
         <v>0.21</v>
@@ -3590,23 +3584,23 @@
       <c r="E86" s="1"/>
       <c r="F86" s="1"/>
       <c r="G86" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H86" s="1"/>
       <c r="I86" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J86" s="1"/>
       <c r="K86" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="87" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="87" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A87" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C87" s="1">
         <v>212</v>
@@ -3621,23 +3615,23 @@
         <v>290</v>
       </c>
       <c r="G87" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H87" s="1"/>
       <c r="I87" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="J87" s="1"/>
       <c r="K87" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="88" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="88" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A88" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C88" s="1">
         <v>1428</v>
@@ -3652,23 +3646,23 @@
         <v>1481</v>
       </c>
       <c r="G88" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H88" s="1"/>
       <c r="I88" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="J88" s="1"/>
       <c r="K88" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="89" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="89" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A89" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C89" s="1">
         <v>6</v>
@@ -3679,23 +3673,23 @@
       <c r="E89" s="1"/>
       <c r="F89" s="1"/>
       <c r="G89" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H89" s="3"/>
       <c r="I89" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J89" s="1"/>
       <c r="K89" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="90" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="90" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A90" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C90" s="1">
         <v>880</v>
@@ -3710,23 +3704,23 @@
         <v>960</v>
       </c>
       <c r="G90" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H90" s="3"/>
       <c r="I90" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J90" s="1"/>
       <c r="K90" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="91" spans="1:11" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="91" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A91" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C91" s="1">
         <v>5.7999999999999996E-3</v>
@@ -3737,23 +3731,23 @@
       <c r="E91" s="1"/>
       <c r="F91" s="1"/>
       <c r="G91" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H91" s="1"/>
       <c r="I91" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J91" s="1"/>
       <c r="K91" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="92" spans="1:11" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="92" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A92" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C92" s="1">
         <v>0.50930200000000003</v>
@@ -3764,23 +3758,23 @@
       <c r="E92" s="1"/>
       <c r="F92" s="1"/>
       <c r="G92" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H92" s="1"/>
       <c r="I92" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J92" s="1"/>
       <c r="K92" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="93" spans="1:11" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="93" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A93" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C93" s="1">
         <v>0.35</v>
@@ -3791,23 +3785,23 @@
       <c r="E93" s="1"/>
       <c r="F93" s="1"/>
       <c r="G93" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H93" s="1"/>
       <c r="I93" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J93" s="1"/>
       <c r="K93" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="94" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="94" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A94" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C94" s="1">
         <v>0</v>
@@ -3820,22 +3814,22 @@
       <c r="G94" s="1"/>
       <c r="H94" s="1"/>
       <c r="I94" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J94" s="1"/>
       <c r="K94" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="95" spans="1:11" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="95" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A95" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D95" s="1">
         <v>0</v>
@@ -3843,23 +3837,23 @@
       <c r="E95" s="1"/>
       <c r="F95" s="1"/>
       <c r="G95" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H95" s="1"/>
       <c r="I95" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J95" s="1"/>
       <c r="K95" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="96" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="96" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A96" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C96" s="1">
         <v>6.0100000000000001E-2</v>
@@ -3872,19 +3866,19 @@
       <c r="G96" s="1"/>
       <c r="H96" s="1"/>
       <c r="I96" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J96" s="1"/>
       <c r="K96" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="97" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="97" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A97" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C97" s="1">
         <v>6.0100000000000001E-2</v>
@@ -3895,25 +3889,25 @@
       <c r="E97" s="1"/>
       <c r="F97" s="1"/>
       <c r="G97" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="H97" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="H97" s="1" t="s">
-        <v>135</v>
-      </c>
       <c r="I97" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J97" s="1"/>
       <c r="K97" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="98" spans="1:11" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="98" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A98" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C98" s="1">
         <v>5.1000000000000004E-3</v>
@@ -3924,23 +3918,23 @@
       <c r="E98" s="1"/>
       <c r="F98" s="1"/>
       <c r="G98" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H98" s="1"/>
       <c r="I98" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J98" s="1"/>
       <c r="K98" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="99" spans="1:11" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="99" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A99" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C99" s="1">
         <v>0.6</v>
@@ -3951,23 +3945,23 @@
       <c r="E99" s="1"/>
       <c r="F99" s="1"/>
       <c r="G99" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H99" s="1"/>
       <c r="I99" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J99" s="1"/>
       <c r="K99" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="100" spans="1:11" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="100" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A100" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C100" s="1">
         <v>0.35</v>
@@ -3978,23 +3972,23 @@
       <c r="E100" s="1"/>
       <c r="F100" s="1"/>
       <c r="G100" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H100" s="1"/>
       <c r="I100" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J100" s="1"/>
       <c r="K100" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="101" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="101" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A101" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C101" s="1">
         <v>0</v>
@@ -4007,19 +4001,19 @@
       <c r="G101" s="1"/>
       <c r="H101" s="1"/>
       <c r="I101" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J101" s="1"/>
       <c r="K101" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="102" spans="1:11" ht="100.8" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="102" spans="1:11" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A102" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C102" s="1">
         <v>1.6799999999999999E-2</v>
@@ -4030,23 +4024,23 @@
       <c r="E102" s="1"/>
       <c r="F102" s="1"/>
       <c r="G102" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H102" s="1"/>
       <c r="I102" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J102" s="1"/>
       <c r="K102" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="103" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="103" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A103" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C103" s="1">
         <v>10</v>
@@ -4058,25 +4052,25 @@
       <c r="E103" s="1"/>
       <c r="F103" s="1"/>
       <c r="G103" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="H103" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="H103" s="1" t="s">
-        <v>95</v>
-      </c>
       <c r="I103" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J103" s="1"/>
       <c r="K103" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="104" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="104" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A104" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C104" s="1">
         <v>26</v>
@@ -4088,25 +4082,25 @@
       <c r="E104" s="1"/>
       <c r="F104" s="1"/>
       <c r="G104" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="H104" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="H104" s="1" t="s">
-        <v>95</v>
-      </c>
       <c r="I104" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J104" s="1"/>
       <c r="K104" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="105" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="105" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A105" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C105" s="1">
         <v>0.3</v>
@@ -4118,25 +4112,25 @@
       <c r="E105" s="1"/>
       <c r="F105" s="1"/>
       <c r="G105" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="H105" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="H105" s="1" t="s">
-        <v>95</v>
-      </c>
       <c r="I105" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J105" s="1"/>
       <c r="K105" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="106" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="106" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A106" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C106" s="1">
         <v>0.15</v>
@@ -4148,25 +4142,25 @@
       <c r="E106" s="1"/>
       <c r="F106" s="1"/>
       <c r="G106" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="H106" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="H106" s="1" t="s">
-        <v>95</v>
-      </c>
       <c r="I106" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J106" s="1"/>
       <c r="K106" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="107" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="107" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A107" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C107" s="1">
         <v>70</v>
@@ -4178,25 +4172,25 @@
       <c r="E107" s="1"/>
       <c r="F107" s="1"/>
       <c r="G107" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="H107" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="H107" s="1" t="s">
-        <v>95</v>
-      </c>
       <c r="I107" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J107" s="1"/>
       <c r="K107" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="108" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="108" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A108" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C108" s="1">
         <v>0.4</v>
@@ -4208,25 +4202,25 @@
       <c r="E108" s="1"/>
       <c r="F108" s="1"/>
       <c r="G108" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="H108" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="H108" s="1" t="s">
-        <v>95</v>
-      </c>
       <c r="I108" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J108" s="1"/>
       <c r="K108" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="109" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="109" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A109" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C109" s="1">
         <v>0.2</v>
@@ -4238,25 +4232,25 @@
       <c r="E109" s="1"/>
       <c r="F109" s="1"/>
       <c r="G109" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="H109" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="H109" s="1" t="s">
-        <v>95</v>
-      </c>
       <c r="I109" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J109" s="1"/>
       <c r="K109" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="110" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="110" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A110" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C110" s="1">
         <v>433</v>
@@ -4268,25 +4262,25 @@
       <c r="E110" s="1"/>
       <c r="F110" s="1"/>
       <c r="G110" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="H110" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="H110" s="1" t="s">
-        <v>95</v>
-      </c>
       <c r="I110" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="J110" s="1"/>
       <c r="K110" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="111" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="111" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A111" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C111" s="1">
         <v>0</v>
@@ -4298,25 +4292,25 @@
       <c r="E111" s="1"/>
       <c r="F111" s="1"/>
       <c r="G111" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="H111" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="H111" s="1" t="s">
-        <v>95</v>
-      </c>
       <c r="I111" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="J111" s="1"/>
       <c r="K111" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="112" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="112" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A112" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C112" s="1">
         <v>6</v>
@@ -4328,25 +4322,25 @@
       <c r="E112" s="1"/>
       <c r="F112" s="1"/>
       <c r="G112" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="H112" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="H112" s="1" t="s">
-        <v>95</v>
-      </c>
       <c r="I112" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J112" s="1"/>
       <c r="K112" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="113" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="113" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A113" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C113" s="1">
         <v>1300</v>
@@ -4358,25 +4352,25 @@
       <c r="E113" s="1"/>
       <c r="F113" s="1"/>
       <c r="G113" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="H113" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="H113" s="1" t="s">
-        <v>95</v>
-      </c>
       <c r="I113" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J113" s="1"/>
       <c r="K113" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="114" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="114" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A114" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C114" s="1">
         <v>0.02</v>
@@ -4388,25 +4382,25 @@
       <c r="E114" s="1"/>
       <c r="F114" s="1"/>
       <c r="G114" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="H114" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="H114" s="1" t="s">
-        <v>95</v>
-      </c>
       <c r="I114" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J114" s="1"/>
       <c r="K114" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="115" spans="1:11" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="115" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A115" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C115" s="1">
         <f>1/36</f>
@@ -4419,25 +4413,25 @@
       <c r="E115" s="1"/>
       <c r="F115" s="1"/>
       <c r="G115" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="H115" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="H115" s="1" t="s">
-        <v>93</v>
-      </c>
       <c r="I115" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J115" s="1"/>
       <c r="K115" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="116" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="116" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A116" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C116" s="1">
         <v>0.5</v>
@@ -4449,25 +4443,25 @@
       <c r="E116" s="1"/>
       <c r="F116" s="1"/>
       <c r="G116" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="H116" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I116" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J116" s="1"/>
       <c r="K116" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="117" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="117" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A117" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C117" s="1">
         <v>0.37</v>
@@ -4479,25 +4473,25 @@
       <c r="E117" s="1"/>
       <c r="F117" s="1"/>
       <c r="G117" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="H117" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I117" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J117" s="1"/>
       <c r="K117" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="118" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="118" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A118" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B118" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C118" s="1">
         <v>0</v>
@@ -4510,22 +4504,22 @@
       <c r="G118" s="1"/>
       <c r="H118" s="1"/>
       <c r="I118" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J118" s="1"/>
       <c r="K118" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="119" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="119" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A119" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B119" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C119" s="2" t="s">
         <v>71</v>
-      </c>
-      <c r="B119" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="C119" s="2" t="s">
-        <v>72</v>
       </c>
       <c r="D119" s="1">
         <f>Table1[[#This Row],[Value]]*2</f>
@@ -4534,28 +4528,28 @@
       <c r="E119" s="1"/>
       <c r="F119" s="1"/>
       <c r="G119" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H119" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I119" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J119" s="1"/>
       <c r="K119" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="120" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="120" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A120" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B120" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C120" s="2" t="s">
         <v>73</v>
-      </c>
-      <c r="B120" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="C120" s="2" t="s">
-        <v>74</v>
       </c>
       <c r="D120" s="1">
         <f>Table1[[#This Row],[Value]]*2</f>
@@ -4564,17 +4558,17 @@
       <c r="E120" s="1"/>
       <c r="F120" s="1"/>
       <c r="G120" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H120" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I120" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J120" s="1"/>
       <c r="K120" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -4599,675 +4593,675 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1" t="s">
         <v>98</v>
-      </c>
-      <c r="D1" t="s">
-        <v>99</v>
       </c>
       <c r="E1" t="s">
         <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>141</v>
       </c>
       <c r="C2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D5">
         <v>0.1</v>
       </c>
       <c r="E5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D6">
         <v>0.1</v>
       </c>
       <c r="E6" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D7">
         <v>0.1</v>
       </c>
       <c r="E7" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D8">
         <v>0.1</v>
       </c>
       <c r="E8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C9" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D9">
         <v>200</v>
       </c>
       <c r="E9" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B10" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D10">
         <v>200</v>
       </c>
       <c r="E10" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
+        <v>99</v>
+      </c>
+      <c r="B11" t="s">
+        <v>99</v>
+      </c>
+      <c r="C11" t="s">
         <v>100</v>
-      </c>
-      <c r="B11" t="s">
-        <v>100</v>
-      </c>
-      <c r="C11" t="s">
-        <v>101</v>
       </c>
       <c r="D11">
         <v>750</v>
       </c>
       <c r="E11" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F11" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B12" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C12" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D12">
         <v>6750</v>
       </c>
       <c r="E12" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F12" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B13" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C13" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D13">
         <v>2500</v>
       </c>
       <c r="E13" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F13" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B14" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C14" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D14">
         <v>200</v>
       </c>
       <c r="E14" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C15" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D15">
         <v>1000</v>
       </c>
       <c r="E15" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F15" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C16" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D16">
         <v>2000</v>
       </c>
       <c r="E16" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F16" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B17" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C17" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D17">
         <v>10</v>
       </c>
       <c r="E17" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F17" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B18" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C18" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D18">
         <v>0.1</v>
       </c>
       <c r="E18" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F18" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C19" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D19">
         <v>400</v>
       </c>
       <c r="E19" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F19" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B20" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C20" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D20">
         <v>10</v>
       </c>
       <c r="E20" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F20" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B21" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C21" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D21">
         <v>1000</v>
       </c>
       <c r="E21" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F21" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B22" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C22" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D22">
         <v>3000</v>
       </c>
       <c r="E22" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F22" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B23" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C23" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D23">
         <v>40</v>
       </c>
       <c r="E23" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F23" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B24" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C24" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D24">
         <v>1000</v>
       </c>
       <c r="E24" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F24" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B25" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C25" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D25">
         <v>210.1</v>
       </c>
       <c r="E25" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F25" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B26" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C26" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D26">
         <v>2450</v>
       </c>
       <c r="E26" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F26" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B27" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C27" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D27">
         <v>3000</v>
       </c>
       <c r="E27" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F27" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B28" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C28" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D28">
         <v>1000</v>
       </c>
       <c r="E28" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F28" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
+        <v>122</v>
+      </c>
+      <c r="B29" t="s">
+        <v>99</v>
+      </c>
+      <c r="C29" t="s">
         <v>123</v>
-      </c>
-      <c r="B29" t="s">
-        <v>100</v>
-      </c>
-      <c r="C29" t="s">
-        <v>124</v>
       </c>
       <c r="D29">
         <v>200</v>
       </c>
       <c r="E29" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F29" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B30" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C30" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D30">
         <v>3000</v>
       </c>
       <c r="E30" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F30" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B31" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C31" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D31">
         <v>20</v>
       </c>
       <c r="E31" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F31" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B32" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C32" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D32">
         <v>20</v>
       </c>
       <c r="E32" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F32" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B33" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C33" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D33">
         <v>400</v>
       </c>
       <c r="E33" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F33" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B34" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C34" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D34">
         <v>1000</v>
       </c>
       <c r="E34" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F34" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B35" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C35" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D35">
         <v>3000</v>
       </c>
       <c r="E35" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F35" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -5286,13 +5280,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
@@ -5300,7 +5294,7 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>141</v>
       </c>
       <c r="C2">
         <v>1</v>
@@ -5308,10 +5302,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>6</v>
+        <v>141</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -5319,10 +5313,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>6</v>
+        <v>141</v>
       </c>
       <c r="C4">
         <v>1</v>
@@ -5330,10 +5324,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>6</v>
+        <v>141</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -5341,10 +5335,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>6</v>
+        <v>141</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -5352,10 +5346,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>6</v>
+        <v>141</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -5366,7 +5360,7 @@
         <v>5</v>
       </c>
       <c r="B8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -5374,10 +5368,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C9">
         <v>1</v>
@@ -5385,10 +5379,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C10">
         <v>1</v>
@@ -5396,10 +5390,10 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -5407,10 +5401,10 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C12">
         <v>0</v>
@@ -5418,10 +5412,10 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B13" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C13">
         <v>0</v>
@@ -5432,7 +5426,7 @@
         <v>5</v>
       </c>
       <c r="B14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C14">
         <v>1</v>
@@ -5440,10 +5434,10 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B15" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C15">
         <v>1</v>
@@ -5451,10 +5445,10 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B16" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C16">
         <v>0</v>
@@ -5462,10 +5456,10 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B17" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C17">
         <v>0</v>
@@ -5473,10 +5467,10 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B18" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C18">
         <v>1</v>
@@ -5484,10 +5478,10 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B19" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C19">
         <v>0</v>
@@ -5498,7 +5492,7 @@
         <v>5</v>
       </c>
       <c r="B20" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C20">
         <v>1</v>
@@ -5506,10 +5500,10 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B21" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C21">
         <v>1</v>
@@ -5517,10 +5511,10 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B22" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C22">
         <v>0</v>
@@ -5528,10 +5522,10 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B23" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C23">
         <v>0</v>
@@ -5539,10 +5533,10 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B24" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C24">
         <v>1</v>
@@ -5550,10 +5544,10 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B25" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C25">
         <v>0</v>
@@ -5564,7 +5558,7 @@
         <v>5</v>
       </c>
       <c r="B26" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C26">
         <v>1</v>
@@ -5572,10 +5566,10 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B27" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C27">
         <v>1</v>
@@ -5583,10 +5577,10 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B28" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C28">
         <v>0</v>
@@ -5594,10 +5588,10 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B29" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C29">
         <v>0</v>
@@ -5605,10 +5599,10 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B30" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C30">
         <v>1</v>
@@ -5616,10 +5610,10 @@
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B31" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C31">
         <v>1</v>
@@ -5630,7 +5624,7 @@
         <v>5</v>
       </c>
       <c r="B32" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C32">
         <v>0</v>
@@ -5638,10 +5632,10 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B33" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C33">
         <v>1</v>
@@ -5649,10 +5643,10 @@
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B34" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C34">
         <v>0</v>
@@ -5660,10 +5654,10 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B35" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C35">
         <v>1</v>
@@ -5671,10 +5665,10 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B36" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C36">
         <v>0</v>
@@ -5682,10 +5676,10 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B37" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C37">
         <v>0</v>

</xml_diff>

<commit_message>
Modifed the code so only the Millennial model remains.
</commit_message>
<xml_diff>
--- a/Data/scenarios.xlsx
+++ b/Data/scenarios.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rober\Documents\GitHub Repos\merging_SFW_decomposition_models\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FCF02A8-253E-41F9-9202-8FD3180CAAB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AFDE102-210E-46A1-A2D8-E12311C08128}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" xr2:uid="{7C97690C-9E7B-4D0E-86C0-16835BCB4BB0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" xr2:uid="{7C97690C-9E7B-4D0E-86C0-16835BCB4BB0}"/>
   </bookViews>
   <sheets>
     <sheet name="scenarios" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="808" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="748" uniqueCount="135">
   <si>
     <t>Parameter</t>
   </si>
@@ -377,48 +377,6 @@
   </si>
   <si>
     <t>Millennial</t>
-  </si>
-  <si>
-    <t>ACTIVE</t>
-  </si>
-  <si>
-    <t>SLOW</t>
-  </si>
-  <si>
-    <t>PASSIVE</t>
-  </si>
-  <si>
-    <t>StrLitter</t>
-  </si>
-  <si>
-    <t>MetLitter</t>
-  </si>
-  <si>
-    <t>Century</t>
-  </si>
-  <si>
-    <t>MIMICS</t>
-  </si>
-  <si>
-    <t>LIT_1</t>
-  </si>
-  <si>
-    <t>LIT_2</t>
-  </si>
-  <si>
-    <t>MIC_1</t>
-  </si>
-  <si>
-    <t>MIC_2</t>
-  </si>
-  <si>
-    <t>SOM_1</t>
-  </si>
-  <si>
-    <t>SOM_2</t>
-  </si>
-  <si>
-    <t>SOM_3</t>
   </si>
   <si>
     <t>Just to start spin-up</t>
@@ -1429,18 +1387,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD4418A0-EB93-4361-AE80-4D25DF544368}">
   <dimension ref="A1:K120"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.77734375" customWidth="1"/>
-    <col min="3" max="3" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="52.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="3" max="3" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="52.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="9" width="23" customWidth="1"/>
-    <col min="10" max="10" width="13.33203125" customWidth="1"/>
+    <col min="10" max="10" width="13.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1469,18 +1427,18 @@
         <v>76</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>133</v>
+        <v>119</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="C2" s="1">
         <v>6</v>
@@ -1491,7 +1449,7 @@
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1" t="s">
-        <v>141</v>
+        <v>127</v>
       </c>
       <c r="H2" s="1"/>
       <c r="I2" s="1" t="s">
@@ -1502,12 +1460,12 @@
         <v>75</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="C3" s="1">
         <v>26</v>
@@ -1527,12 +1485,12 @@
         <v>75</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="C4" s="1">
         <v>0.3</v>
@@ -1552,12 +1510,12 @@
         <v>75</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="C5" s="1">
         <v>0.15</v>
@@ -1577,12 +1535,12 @@
         <v>75</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="C6" s="1">
         <v>73</v>
@@ -1597,7 +1555,7 @@
         <v>78</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>142</v>
+        <v>128</v>
       </c>
       <c r="H6" s="1"/>
       <c r="I6" s="1" t="s">
@@ -1608,12 +1566,12 @@
         <v>75</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="C7" s="1">
         <v>0.28000000000000003</v>
@@ -1628,7 +1586,7 @@
         <v>0.33</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>142</v>
+        <v>128</v>
       </c>
       <c r="H7" s="1"/>
       <c r="I7" s="1" t="s">
@@ -1639,12 +1597,12 @@
         <v>75</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="C8" s="1">
         <v>0.2</v>
@@ -1659,10 +1617,10 @@
         <v>0.3</v>
       </c>
       <c r="G8" t="s">
-        <v>146</v>
+        <v>132</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>147</v>
+        <v>133</v>
       </c>
       <c r="I8" s="1" t="s">
         <v>77</v>
@@ -1672,12 +1630,12 @@
         <v>75</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>18</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="C9" s="6">
         <f>C10*0.03</f>
@@ -1696,7 +1654,7 @@
         <v>17.920000000000002</v>
       </c>
       <c r="G9" t="s">
-        <v>145</v>
+        <v>131</v>
       </c>
       <c r="H9" s="1"/>
       <c r="I9" s="1" t="s">
@@ -1707,12 +1665,12 @@
         <v>75</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>19</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="C10" s="1">
         <f>336/0.75</f>
@@ -1731,7 +1689,7 @@
         <v>448</v>
       </c>
       <c r="G10" t="s">
-        <v>144</v>
+        <v>130</v>
       </c>
       <c r="H10" s="1"/>
       <c r="I10" s="1" t="s">
@@ -1742,12 +1700,12 @@
         <v>75</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="C11" s="1">
         <v>7.7</v>
@@ -1762,7 +1720,7 @@
         <v>8</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>142</v>
+        <v>128</v>
       </c>
       <c r="H11" s="1"/>
       <c r="I11" s="1" t="s">
@@ -1773,12 +1731,12 @@
         <v>75</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>21</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="C12" s="1">
         <v>700</v>
@@ -1793,7 +1751,7 @@
         <v>1160</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>143</v>
+        <v>129</v>
       </c>
       <c r="H12" s="1"/>
       <c r="I12" s="1" t="s">
@@ -1804,12 +1762,12 @@
         <v>75</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>22</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="C13" s="1">
         <v>1.5873020000000002E-2</v>
@@ -1822,7 +1780,7 @@
       </c>
       <c r="F13" s="1"/>
       <c r="G13" s="1" t="s">
-        <v>140</v>
+        <v>126</v>
       </c>
       <c r="H13" s="1"/>
       <c r="I13" s="1" t="s">
@@ -1833,12 +1791,12 @@
         <v>75</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>23</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="C14" s="1">
         <v>0.53</v>
@@ -1860,12 +1818,12 @@
         <v>75</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>25</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="C15" s="1">
         <v>0.09</v>
@@ -1887,12 +1845,12 @@
         <v>75</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>27</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="C16" s="1">
         <v>0.22</v>
@@ -1914,12 +1872,12 @@
         <v>75</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>29</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="C17" s="1">
         <v>0</v>
@@ -1939,12 +1897,12 @@
         <v>75</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="C18" s="1">
         <v>0</v>
@@ -1962,12 +1920,12 @@
       <c r="J18" s="1"/>
       <c r="K18" s="1"/>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>31</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="C19" s="5">
         <v>1.89202E-4</v>
@@ -1985,12 +1943,12 @@
       <c r="J19" s="1"/>
       <c r="K19" s="1"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>32</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="C20" s="1">
         <v>0</v>
@@ -2008,12 +1966,12 @@
       <c r="J20" s="1"/>
       <c r="K20" s="1"/>
     </row>
-    <row r="21" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>33</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="C21" s="1">
         <v>0</v>
@@ -2025,7 +1983,7 @@
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
       <c r="H21" s="1" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="I21" s="1" t="s">
         <v>79</v>
@@ -2033,12 +1991,12 @@
       <c r="J21" s="1"/>
       <c r="K21" s="1"/>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>34</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="C22" s="1">
         <v>-0.02</v>
@@ -2056,7 +2014,7 @@
       <c r="J22" s="1"/>
       <c r="K22" s="1"/>
     </row>
-    <row r="23" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>11</v>
       </c>
@@ -2072,7 +2030,7 @@
       <c r="E23" s="1"/>
       <c r="F23" s="1"/>
       <c r="G23" s="1" t="s">
-        <v>135</v>
+        <v>121</v>
       </c>
       <c r="H23" s="1"/>
       <c r="I23" s="1" t="s">
@@ -2083,7 +2041,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>12</v>
       </c>
@@ -2099,7 +2057,7 @@
       <c r="E24" s="1"/>
       <c r="F24" s="1"/>
       <c r="G24" s="1" t="s">
-        <v>135</v>
+        <v>121</v>
       </c>
       <c r="H24" s="1"/>
       <c r="I24" s="1" t="s">
@@ -2110,7 +2068,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>13</v>
       </c>
@@ -2126,7 +2084,7 @@
       <c r="E25" s="1"/>
       <c r="F25" s="1"/>
       <c r="G25" t="s">
-        <v>137</v>
+        <v>123</v>
       </c>
       <c r="H25" s="1"/>
       <c r="I25" s="1" t="s">
@@ -2137,7 +2095,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>14</v>
       </c>
@@ -2153,7 +2111,7 @@
       <c r="E26" s="1"/>
       <c r="F26" s="1"/>
       <c r="G26" t="s">
-        <v>137</v>
+        <v>123</v>
       </c>
       <c r="H26" s="1"/>
       <c r="I26" s="1" t="s">
@@ -2164,7 +2122,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>15</v>
       </c>
@@ -2180,7 +2138,7 @@
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
       <c r="G27" s="1" t="s">
-        <v>135</v>
+        <v>121</v>
       </c>
       <c r="H27" s="1"/>
       <c r="I27" s="1" t="s">
@@ -2191,7 +2149,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>16</v>
       </c>
@@ -2207,7 +2165,7 @@
       <c r="E28" s="1"/>
       <c r="F28" s="1"/>
       <c r="G28" s="1" t="s">
-        <v>135</v>
+        <v>121</v>
       </c>
       <c r="H28" s="1"/>
       <c r="I28" s="1" t="s">
@@ -2218,7 +2176,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>17</v>
       </c>
@@ -2241,7 +2199,7 @@
       <c r="J29" s="1"/>
       <c r="K29" s="1"/>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>18</v>
       </c>
@@ -2264,7 +2222,7 @@
       <c r="J30" s="1"/>
       <c r="K30" s="1"/>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>19</v>
       </c>
@@ -2284,7 +2242,7 @@
         <v>1642</v>
       </c>
       <c r="G31" t="s">
-        <v>138</v>
+        <v>124</v>
       </c>
       <c r="H31" s="1"/>
       <c r="I31" s="1" t="s">
@@ -2295,7 +2253,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>20</v>
       </c>
@@ -2318,7 +2276,7 @@
       <c r="J32" s="1"/>
       <c r="K32" s="1"/>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>21</v>
       </c>
@@ -2341,7 +2299,7 @@
       <c r="J33" s="1"/>
       <c r="K33" s="1"/>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>22</v>
       </c>
@@ -2368,7 +2326,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>23</v>
       </c>
@@ -2395,7 +2353,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>25</v>
       </c>
@@ -2422,7 +2380,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>27</v>
       </c>
@@ -2449,7 +2407,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>29</v>
       </c>
@@ -2474,7 +2432,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>30</v>
       </c>
@@ -2490,7 +2448,7 @@
       <c r="E39" s="1"/>
       <c r="F39" s="1"/>
       <c r="G39" s="1" t="s">
-        <v>136</v>
+        <v>122</v>
       </c>
       <c r="H39" s="1"/>
       <c r="I39" s="1" t="s">
@@ -2501,7 +2459,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>31</v>
       </c>
@@ -2524,7 +2482,7 @@
       <c r="J40" s="1"/>
       <c r="K40" s="1"/>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>32</v>
       </c>
@@ -2540,7 +2498,7 @@
       <c r="E41" s="1"/>
       <c r="F41" s="1"/>
       <c r="G41" s="1" t="s">
-        <v>136</v>
+        <v>122</v>
       </c>
       <c r="H41" s="1"/>
       <c r="I41" s="1" t="s">
@@ -2551,7 +2509,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="42" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>33</v>
       </c>
@@ -2568,7 +2526,7 @@
       <c r="F42" s="1"/>
       <c r="G42" s="1"/>
       <c r="H42" s="1" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="I42" s="1" t="s">
         <v>79</v>
@@ -2576,7 +2534,7 @@
       <c r="J42" s="1"/>
       <c r="K42" s="1"/>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>34</v>
       </c>
@@ -2599,7 +2557,7 @@
       <c r="J43" s="1"/>
       <c r="K43" s="1"/>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>11</v>
       </c>
@@ -2622,7 +2580,7 @@
       <c r="J44" s="1"/>
       <c r="K44" s="1"/>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>12</v>
       </c>
@@ -2645,7 +2603,7 @@
       <c r="J45" s="1"/>
       <c r="K45" s="1"/>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>13</v>
       </c>
@@ -2668,7 +2626,7 @@
       <c r="J46" s="1"/>
       <c r="K46" s="1"/>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>14</v>
       </c>
@@ -2691,7 +2649,7 @@
       <c r="J47" s="1"/>
       <c r="K47" s="1"/>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>15</v>
       </c>
@@ -2714,7 +2672,7 @@
       <c r="J48" s="1"/>
       <c r="K48" s="1"/>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>16</v>
       </c>
@@ -2737,7 +2695,7 @@
       <c r="J49" s="1"/>
       <c r="K49" s="1"/>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>17</v>
       </c>
@@ -2760,7 +2718,7 @@
       <c r="J50" s="1"/>
       <c r="K50" s="1"/>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>18</v>
       </c>
@@ -2783,7 +2741,7 @@
       <c r="J51" s="1"/>
       <c r="K51" s="1"/>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>19</v>
       </c>
@@ -2806,7 +2764,7 @@
       <c r="J52" s="1"/>
       <c r="K52" s="1"/>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>20</v>
       </c>
@@ -2829,7 +2787,7 @@
       <c r="J53" s="1"/>
       <c r="K53" s="1"/>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>21</v>
       </c>
@@ -2852,7 +2810,7 @@
       <c r="J54" s="1"/>
       <c r="K54" s="1"/>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>39</v>
       </c>
@@ -2875,7 +2833,7 @@
       <c r="J55" s="1"/>
       <c r="K55" s="1"/>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>40</v>
       </c>
@@ -2898,7 +2856,7 @@
       <c r="J56" s="1"/>
       <c r="K56" s="1"/>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>41</v>
       </c>
@@ -2921,7 +2879,7 @@
       <c r="J57" s="1"/>
       <c r="K57" s="1"/>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>42</v>
       </c>
@@ -2944,7 +2902,7 @@
       <c r="J58" s="1"/>
       <c r="K58" s="1"/>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>43</v>
       </c>
@@ -2967,7 +2925,7 @@
       <c r="J59" s="1"/>
       <c r="K59" s="1"/>
     </row>
-    <row r="60" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>45</v>
       </c>
@@ -2990,7 +2948,7 @@
       <c r="J60" s="1"/>
       <c r="K60" s="1"/>
     </row>
-    <row r="61" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>46</v>
       </c>
@@ -3013,7 +2971,7 @@
       <c r="J61" s="1"/>
       <c r="K61" s="1"/>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>11</v>
       </c>
@@ -3040,7 +2998,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>12</v>
       </c>
@@ -3067,7 +3025,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="64" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>13</v>
       </c>
@@ -3094,7 +3052,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="65" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>14</v>
       </c>
@@ -3121,7 +3079,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>15</v>
       </c>
@@ -3148,7 +3106,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>16</v>
       </c>
@@ -3175,7 +3133,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>17</v>
       </c>
@@ -3203,7 +3161,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>18</v>
       </c>
@@ -3234,7 +3192,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>19</v>
       </c>
@@ -3265,7 +3223,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>20</v>
       </c>
@@ -3292,7 +3250,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>21</v>
       </c>
@@ -3323,7 +3281,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="73" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>39</v>
       </c>
@@ -3350,7 +3308,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="74" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
         <v>40</v>
       </c>
@@ -3377,7 +3335,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="75" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
         <v>41</v>
       </c>
@@ -3404,7 +3362,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
         <v>42</v>
       </c>
@@ -3429,7 +3387,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="77" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
         <v>43</v>
       </c>
@@ -3456,7 +3414,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="78" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
         <v>45</v>
       </c>
@@ -3483,7 +3441,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="79" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
         <v>46</v>
       </c>
@@ -3499,10 +3457,10 @@
       <c r="E79" s="1"/>
       <c r="F79" s="1"/>
       <c r="G79" s="1" t="s">
-        <v>131</v>
+        <v>117</v>
       </c>
       <c r="H79" s="1" t="s">
-        <v>132</v>
+        <v>118</v>
       </c>
       <c r="I79" s="1" t="s">
         <v>80</v>
@@ -3512,7 +3470,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
         <v>11</v>
       </c>
@@ -3539,7 +3497,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
         <v>12</v>
       </c>
@@ -3566,7 +3524,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="82" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
         <v>13</v>
       </c>
@@ -3593,7 +3551,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="83" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
         <v>14</v>
       </c>
@@ -3620,7 +3578,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
         <v>15</v>
       </c>
@@ -3647,7 +3605,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
         <v>16</v>
       </c>
@@ -3674,7 +3632,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
         <v>17</v>
       </c>
@@ -3702,7 +3660,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
         <v>18</v>
       </c>
@@ -3733,7 +3691,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
         <v>19</v>
       </c>
@@ -3764,7 +3722,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
         <v>20</v>
       </c>
@@ -3791,7 +3749,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
         <v>21</v>
       </c>
@@ -3822,7 +3780,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="91" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
         <v>39</v>
       </c>
@@ -3849,7 +3807,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="92" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
         <v>40</v>
       </c>
@@ -3876,7 +3834,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="93" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
         <v>41</v>
       </c>
@@ -3903,7 +3861,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
         <v>42</v>
       </c>
@@ -3928,7 +3886,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="95" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
         <v>43</v>
       </c>
@@ -3955,7 +3913,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="96" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
         <v>45</v>
       </c>
@@ -3980,7 +3938,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="97" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A97" s="1" t="s">
         <v>46</v>
       </c>
@@ -3996,10 +3954,10 @@
       <c r="E97" s="1"/>
       <c r="F97" s="1"/>
       <c r="G97" s="1" t="s">
-        <v>131</v>
+        <v>117</v>
       </c>
       <c r="H97" s="1" t="s">
-        <v>132</v>
+        <v>118</v>
       </c>
       <c r="I97" s="1" t="s">
         <v>80</v>
@@ -4009,7 +3967,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="98" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A98" s="1" t="s">
         <v>56</v>
       </c>
@@ -4036,7 +3994,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="99" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
         <v>57</v>
       </c>
@@ -4063,7 +4021,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="100" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A100" s="1" t="s">
         <v>58</v>
       </c>
@@ -4090,7 +4048,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="101" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A101" s="1" t="s">
         <v>59</v>
       </c>
@@ -4115,7 +4073,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="102" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A102" s="1" t="s">
         <v>60</v>
       </c>
@@ -4142,7 +4100,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="103" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A103" s="1" t="s">
         <v>11</v>
       </c>
@@ -4172,7 +4130,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A104" s="1" t="s">
         <v>12</v>
       </c>
@@ -4202,7 +4160,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="105" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A105" s="1" t="s">
         <v>13</v>
       </c>
@@ -4232,7 +4190,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="106" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A106" s="1" t="s">
         <v>14</v>
       </c>
@@ -4262,7 +4220,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A107" s="1" t="s">
         <v>15</v>
       </c>
@@ -4292,7 +4250,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="108" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A108" s="1" t="s">
         <v>16</v>
       </c>
@@ -4322,7 +4280,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="109" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A109" s="1" t="s">
         <v>17</v>
       </c>
@@ -4352,7 +4310,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="110" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A110" s="1" t="s">
         <v>18</v>
       </c>
@@ -4382,7 +4340,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="111" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A111" s="1" t="s">
         <v>19</v>
       </c>
@@ -4412,7 +4370,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="112" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A112" s="1" t="s">
         <v>20</v>
       </c>
@@ -4442,7 +4400,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A113" s="1" t="s">
         <v>21</v>
       </c>
@@ -4472,7 +4430,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A114" s="1" t="s">
         <v>63</v>
       </c>
@@ -4502,7 +4460,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="115" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A115" s="1" t="s">
         <v>64</v>
       </c>
@@ -4533,7 +4491,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A116" s="1" t="s">
         <v>65</v>
       </c>
@@ -4563,7 +4521,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A117" s="1" t="s">
         <v>66</v>
       </c>
@@ -4593,7 +4551,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A118" s="1" t="s">
         <v>67</v>
       </c>
@@ -4618,7 +4576,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A119" s="1" t="s">
         <v>68</v>
       </c>
@@ -4648,7 +4606,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A120" s="1" t="s">
         <v>70</v>
       </c>
@@ -4688,17 +4646,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA0710C0-AB94-4FBF-AB29-E5085BC4F559}">
-  <dimension ref="A1:F35"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:F23"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.77734375" customWidth="1"/>
+    <col min="1" max="1" width="11.7109375" customWidth="1"/>
     <col min="2" max="2" width="20" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.88671875" customWidth="1"/>
+    <col min="3" max="3" width="13.85546875" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="35.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="35.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>94</v>
       </c>
@@ -4718,18 +4676,18 @@
         <v>74</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>97</v>
       </c>
       <c r="B2" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="C2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>97</v>
       </c>
@@ -4740,7 +4698,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>97</v>
       </c>
@@ -4751,7 +4709,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>97</v>
       </c>
@@ -4765,13 +4723,13 @@
         <v>0.1</v>
       </c>
       <c r="E5" t="s">
-        <v>130</v>
+        <v>116</v>
       </c>
       <c r="F5" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>97</v>
       </c>
@@ -4785,13 +4743,13 @@
         <v>0.1</v>
       </c>
       <c r="E6" t="s">
-        <v>130</v>
+        <v>116</v>
       </c>
       <c r="F6" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>97</v>
       </c>
@@ -4805,13 +4763,13 @@
         <v>0.1</v>
       </c>
       <c r="E7" t="s">
-        <v>130</v>
+        <v>116</v>
       </c>
       <c r="F7" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>97</v>
       </c>
@@ -4825,13 +4783,13 @@
         <v>0.1</v>
       </c>
       <c r="E8" t="s">
-        <v>129</v>
+        <v>115</v>
       </c>
       <c r="F8" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>97</v>
       </c>
@@ -4845,13 +4803,13 @@
         <v>200</v>
       </c>
       <c r="E9" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="F9" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>97</v>
       </c>
@@ -4865,13 +4823,13 @@
         <v>200</v>
       </c>
       <c r="E10" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="F10" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>97</v>
       </c>
@@ -4885,13 +4843,13 @@
         <v>750</v>
       </c>
       <c r="E11" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="F11" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>97</v>
       </c>
@@ -4905,13 +4863,13 @@
         <v>6750</v>
       </c>
       <c r="E12" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="F12" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>97</v>
       </c>
@@ -4925,13 +4883,13 @@
         <v>2500</v>
       </c>
       <c r="E13" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="F13" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>113</v>
       </c>
@@ -4945,13 +4903,13 @@
         <v>200</v>
       </c>
       <c r="E14" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="F14" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>113</v>
       </c>
@@ -4965,13 +4923,13 @@
         <v>1000</v>
       </c>
       <c r="E15" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="F15" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>113</v>
       </c>
@@ -4985,13 +4943,13 @@
         <v>2000</v>
       </c>
       <c r="E16" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="F16" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>113</v>
       </c>
@@ -5005,13 +4963,13 @@
         <v>10</v>
       </c>
       <c r="E17" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="F17" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>113</v>
       </c>
@@ -5025,13 +4983,13 @@
         <v>0.1</v>
       </c>
       <c r="E18" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="F18" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>113</v>
       </c>
@@ -5045,13 +5003,13 @@
         <v>400</v>
       </c>
       <c r="E19" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="F19" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>113</v>
       </c>
@@ -5065,13 +5023,13 @@
         <v>10</v>
       </c>
       <c r="E20" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="F20" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>113</v>
       </c>
@@ -5085,13 +5043,13 @@
         <v>1000</v>
       </c>
       <c r="E21" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="F21" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>113</v>
       </c>
@@ -5105,13 +5063,13 @@
         <v>3000</v>
       </c>
       <c r="E22" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="F22" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>113</v>
       </c>
@@ -5125,249 +5083,9 @@
         <v>40</v>
       </c>
       <c r="E23" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="F23" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>119</v>
-      </c>
-      <c r="B24" t="s">
-        <v>97</v>
-      </c>
-      <c r="C24" t="s">
-        <v>117</v>
-      </c>
-      <c r="D24">
-        <v>1000</v>
-      </c>
-      <c r="E24" t="s">
-        <v>128</v>
-      </c>
-      <c r="F24" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>119</v>
-      </c>
-      <c r="B25" t="s">
-        <v>97</v>
-      </c>
-      <c r="C25" t="s">
-        <v>118</v>
-      </c>
-      <c r="D25">
-        <v>210.1</v>
-      </c>
-      <c r="E25" t="s">
-        <v>128</v>
-      </c>
-      <c r="F25" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
-        <v>119</v>
-      </c>
-      <c r="B26" t="s">
-        <v>97</v>
-      </c>
-      <c r="C26" t="s">
-        <v>114</v>
-      </c>
-      <c r="D26">
-        <v>2450</v>
-      </c>
-      <c r="E26" t="s">
-        <v>128</v>
-      </c>
-      <c r="F26" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>119</v>
-      </c>
-      <c r="B27" t="s">
-        <v>97</v>
-      </c>
-      <c r="C27" t="s">
-        <v>115</v>
-      </c>
-      <c r="D27">
-        <v>3000</v>
-      </c>
-      <c r="E27" t="s">
-        <v>128</v>
-      </c>
-      <c r="F27" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
-        <v>119</v>
-      </c>
-      <c r="B28" t="s">
-        <v>97</v>
-      </c>
-      <c r="C28" t="s">
-        <v>116</v>
-      </c>
-      <c r="D28">
-        <v>1000</v>
-      </c>
-      <c r="E28" t="s">
-        <v>128</v>
-      </c>
-      <c r="F28" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
-        <v>120</v>
-      </c>
-      <c r="B29" t="s">
-        <v>97</v>
-      </c>
-      <c r="C29" t="s">
-        <v>121</v>
-      </c>
-      <c r="D29">
-        <v>200</v>
-      </c>
-      <c r="E29" t="s">
-        <v>128</v>
-      </c>
-      <c r="F29" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
-        <v>120</v>
-      </c>
-      <c r="B30" t="s">
-        <v>97</v>
-      </c>
-      <c r="C30" t="s">
-        <v>122</v>
-      </c>
-      <c r="D30">
-        <v>3000</v>
-      </c>
-      <c r="E30" t="s">
-        <v>128</v>
-      </c>
-      <c r="F30" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
-        <v>120</v>
-      </c>
-      <c r="B31" t="s">
-        <v>97</v>
-      </c>
-      <c r="C31" t="s">
-        <v>123</v>
-      </c>
-      <c r="D31">
-        <v>20</v>
-      </c>
-      <c r="E31" t="s">
-        <v>128</v>
-      </c>
-      <c r="F31" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
-        <v>120</v>
-      </c>
-      <c r="B32" t="s">
-        <v>97</v>
-      </c>
-      <c r="C32" t="s">
-        <v>124</v>
-      </c>
-      <c r="D32">
-        <v>20</v>
-      </c>
-      <c r="E32" t="s">
-        <v>128</v>
-      </c>
-      <c r="F32" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
-        <v>120</v>
-      </c>
-      <c r="B33" t="s">
-        <v>97</v>
-      </c>
-      <c r="C33" t="s">
-        <v>125</v>
-      </c>
-      <c r="D33">
-        <v>400</v>
-      </c>
-      <c r="E33" t="s">
-        <v>128</v>
-      </c>
-      <c r="F33" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A34" t="s">
-        <v>120</v>
-      </c>
-      <c r="B34" t="s">
-        <v>97</v>
-      </c>
-      <c r="C34" t="s">
-        <v>126</v>
-      </c>
-      <c r="D34">
-        <v>1000</v>
-      </c>
-      <c r="E34" t="s">
-        <v>128</v>
-      </c>
-      <c r="F34" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
-        <v>120</v>
-      </c>
-      <c r="B35" t="s">
-        <v>97</v>
-      </c>
-      <c r="C35" t="s">
-        <v>127</v>
-      </c>
-      <c r="D35">
-        <v>3000</v>
-      </c>
-      <c r="E35" t="s">
-        <v>128</v>
-      </c>
-      <c r="F35" t="s">
         <v>75</v>
       </c>
     </row>
@@ -5379,13 +5097,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC182590-26D0-4168-8E7C-B448CD67FE47}">
   <dimension ref="A1:C37"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>95</v>
       </c>
@@ -5393,76 +5111,76 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="C3">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="C4">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="C5">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="C6">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="C7">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -5473,7 +5191,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>6</v>
       </c>
@@ -5484,7 +5202,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>7</v>
       </c>
@@ -5495,7 +5213,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -5506,7 +5224,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -5517,7 +5235,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>10</v>
       </c>
@@ -5528,7 +5246,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>5</v>
       </c>
@@ -5539,7 +5257,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>6</v>
       </c>
@@ -5550,7 +5268,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>7</v>
       </c>
@@ -5561,7 +5279,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>8</v>
       </c>
@@ -5572,7 +5290,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>9</v>
       </c>
@@ -5583,7 +5301,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>10</v>
       </c>
@@ -5594,7 +5312,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>5</v>
       </c>
@@ -5605,7 +5323,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>6</v>
       </c>
@@ -5616,7 +5334,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>7</v>
       </c>
@@ -5627,7 +5345,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>8</v>
       </c>
@@ -5638,7 +5356,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>9</v>
       </c>
@@ -5649,7 +5367,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>10</v>
       </c>
@@ -5660,7 +5378,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>5</v>
       </c>
@@ -5671,7 +5389,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>6</v>
       </c>
@@ -5682,7 +5400,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>7</v>
       </c>
@@ -5693,7 +5411,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>8</v>
       </c>
@@ -5704,7 +5422,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>9</v>
       </c>
@@ -5715,7 +5433,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>10</v>
       </c>
@@ -5726,7 +5444,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>5</v>
       </c>
@@ -5737,7 +5455,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>6</v>
       </c>
@@ -5748,7 +5466,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>7</v>
       </c>
@@ -5759,7 +5477,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>8</v>
       </c>
@@ -5770,7 +5488,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>9</v>
       </c>
@@ -5781,7 +5499,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Working on the scenario file.
</commit_message>
<xml_diff>
--- a/Data/scenarios.xlsx
+++ b/Data/scenarios.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rober\Documents\GitHub Repos\merging_SFW_decomposition_models\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C4127D7-FD44-4073-B8BA-C4C21D531FA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{552E65D8-5B48-4470-86CA-61AB06316E5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" xr2:uid="{7C97690C-9E7B-4D0E-86C0-16835BCB4BB0}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{7C97690C-9E7B-4D0E-86C0-16835BCB4BB0}"/>
   </bookViews>
   <sheets>
     <sheet name="scenarios" sheetId="1" r:id="rId1"/>
     <sheet name="state_variables_value" sheetId="2" r:id="rId2"/>
-    <sheet name="state_variable_include" sheetId="4" r:id="rId3"/>
+    <sheet name="effect_of_animals" sheetId="5" r:id="rId3"/>
+    <sheet name="state_variable_include" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="644" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="688" uniqueCount="131">
   <si>
     <t>Parameter</t>
   </si>
@@ -238,15 +239,9 @@
     <t>k_exudate_intercept</t>
   </si>
   <si>
-    <t>2.74e-5</t>
-  </si>
-  <si>
     <t>k_exudate_slope</t>
   </si>
   <si>
-    <t>1.3e-5</t>
-  </si>
-  <si>
     <t>Min</t>
   </si>
   <si>
@@ -422,6 +417,18 @@
   </si>
   <si>
     <t>Buchkowski et al. 2024; Buchkowski and Schmitz 2023 for average weight from WE plots; 25% dry weight, 50% carbon</t>
+  </si>
+  <si>
+    <t>EffectPool</t>
+  </si>
+  <si>
+    <t>EffectParameter</t>
+  </si>
+  <si>
+    <t>LWMC</t>
+  </si>
+  <si>
+    <t>EffectSize</t>
   </si>
 </sst>
 </file>
@@ -1369,18 +1376,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD4418A0-EB93-4361-AE80-4D25DF544368}">
   <dimension ref="A1:K99"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
-    <col min="3" max="3" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="52.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.7265625" customWidth="1"/>
+    <col min="3" max="3" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="52.26953125" bestFit="1" customWidth="1"/>
     <col min="8" max="9" width="23" customWidth="1"/>
-    <col min="10" max="10" width="13.28515625" customWidth="1"/>
+    <col min="10" max="10" width="13.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1394,28 +1401,28 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
@@ -1431,18 +1438,18 @@
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="H2" s="1"/>
       <c r="I2" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J2" s="1"/>
       <c r="K2" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
@@ -1460,14 +1467,14 @@
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
       <c r="I3" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J3" s="1"/>
       <c r="K3" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>13</v>
       </c>
@@ -1485,14 +1492,14 @@
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
       <c r="I4" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J4" s="1"/>
       <c r="K4" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>14</v>
       </c>
@@ -1510,14 +1517,14 @@
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
       <c r="I5" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J5" s="1"/>
       <c r="K5" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
@@ -1537,18 +1544,18 @@
         <v>78</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="H6" s="1"/>
       <c r="I6" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J6" s="1"/>
       <c r="K6" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>16</v>
       </c>
@@ -1568,18 +1575,18 @@
         <v>0.33</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="H7" s="1"/>
       <c r="I7" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J7" s="1"/>
       <c r="K7" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>17</v>
       </c>
@@ -1599,20 +1606,20 @@
         <v>0.3</v>
       </c>
       <c r="G8" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J8" s="1"/>
       <c r="K8" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>18</v>
       </c>
@@ -1636,18 +1643,18 @@
         <v>17.920000000000002</v>
       </c>
       <c r="G9" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="H9" s="1"/>
       <c r="I9" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="J9" s="1"/>
       <c r="K9" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>19</v>
       </c>
@@ -1671,18 +1678,18 @@
         <v>448</v>
       </c>
       <c r="G10" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H10" s="1"/>
       <c r="I10" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="J10" s="1"/>
       <c r="K10" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
@@ -1702,18 +1709,18 @@
         <v>8</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="H11" s="1"/>
       <c r="I11" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J11" s="1"/>
       <c r="K11" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>21</v>
       </c>
@@ -1733,18 +1740,18 @@
         <v>1160</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="H12" s="1"/>
       <c r="I12" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J12" s="1"/>
       <c r="K12" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>22</v>
       </c>
@@ -1762,18 +1769,18 @@
       </c>
       <c r="F13" s="1"/>
       <c r="G13" s="1" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="H13" s="1"/>
       <c r="I13" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J13" s="1"/>
       <c r="K13" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>23</v>
       </c>
@@ -1793,14 +1800,14 @@
       </c>
       <c r="H14" s="1"/>
       <c r="I14" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J14" s="1"/>
       <c r="K14" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>25</v>
       </c>
@@ -1820,14 +1827,14 @@
       </c>
       <c r="H15" s="1"/>
       <c r="I15" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J15" s="1"/>
       <c r="K15" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>27</v>
       </c>
@@ -1847,14 +1854,14 @@
       </c>
       <c r="H16" s="1"/>
       <c r="I16" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J16" s="1"/>
       <c r="K16" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>29</v>
       </c>
@@ -1872,22 +1879,22 @@
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
       <c r="I17" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J17" s="1"/>
       <c r="K17" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C18" s="1">
-        <v>0</v>
+      <c r="C18" s="5">
+        <v>1.89202E-4</v>
       </c>
       <c r="D18" s="1">
         <v>0</v>
@@ -1897,12 +1904,12 @@
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
       <c r="I18" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J18" s="1"/>
       <c r="K18" s="1"/>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>31</v>
       </c>
@@ -1920,20 +1927,20 @@
       <c r="G19" s="1"/>
       <c r="H19" s="1"/>
       <c r="I19" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J19" s="1"/>
       <c r="K19" s="1"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>32</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C20" s="1">
-        <v>0</v>
+      <c r="C20" s="5">
+        <v>1.89202E-4</v>
       </c>
       <c r="D20" s="1">
         <v>0</v>
@@ -1943,12 +1950,12 @@
       <c r="G20" s="1"/>
       <c r="H20" s="1"/>
       <c r="I20" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J20" s="1"/>
       <c r="K20" s="1"/>
     </row>
-    <row r="21" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>33</v>
       </c>
@@ -1965,15 +1972,15 @@
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
       <c r="H21" s="1" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J21" s="1"/>
       <c r="K21" s="1"/>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>34</v>
       </c>
@@ -1991,12 +1998,12 @@
       <c r="G22" s="1"/>
       <c r="H22" s="1"/>
       <c r="I22" s="1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="J22" s="1"/>
       <c r="K22" s="1"/>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>11</v>
       </c>
@@ -2014,12 +2021,12 @@
       <c r="G23" s="1"/>
       <c r="H23" s="1"/>
       <c r="I23" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J23" s="1"/>
       <c r="K23" s="1"/>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>12</v>
       </c>
@@ -2037,12 +2044,12 @@
       <c r="G24" s="1"/>
       <c r="H24" s="1"/>
       <c r="I24" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J24" s="1"/>
       <c r="K24" s="1"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>13</v>
       </c>
@@ -2060,12 +2067,12 @@
       <c r="G25" s="1"/>
       <c r="H25" s="1"/>
       <c r="I25" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J25" s="1"/>
       <c r="K25" s="1"/>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>14</v>
       </c>
@@ -2083,12 +2090,12 @@
       <c r="G26" s="1"/>
       <c r="H26" s="1"/>
       <c r="I26" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J26" s="1"/>
       <c r="K26" s="1"/>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>15</v>
       </c>
@@ -2106,12 +2113,12 @@
       <c r="G27" s="1"/>
       <c r="H27" s="1"/>
       <c r="I27" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J27" s="1"/>
       <c r="K27" s="1"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>16</v>
       </c>
@@ -2129,12 +2136,12 @@
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
       <c r="I28" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J28" s="1"/>
       <c r="K28" s="1"/>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>17</v>
       </c>
@@ -2152,12 +2159,12 @@
       <c r="G29" s="1"/>
       <c r="H29" s="1"/>
       <c r="I29" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J29" s="1"/>
       <c r="K29" s="1"/>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>18</v>
       </c>
@@ -2175,12 +2182,12 @@
       <c r="G30" s="1"/>
       <c r="H30" s="1"/>
       <c r="I30" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="J30" s="1"/>
       <c r="K30" s="1"/>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>19</v>
       </c>
@@ -2198,12 +2205,12 @@
       <c r="G31" s="1"/>
       <c r="H31" s="1"/>
       <c r="I31" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="J31" s="1"/>
       <c r="K31" s="1"/>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>20</v>
       </c>
@@ -2221,12 +2228,12 @@
       <c r="G32" s="1"/>
       <c r="H32" s="1"/>
       <c r="I32" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J32" s="1"/>
       <c r="K32" s="1"/>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>21</v>
       </c>
@@ -2244,12 +2251,12 @@
       <c r="G33" s="1"/>
       <c r="H33" s="1"/>
       <c r="I33" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J33" s="1"/>
       <c r="K33" s="1"/>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>37</v>
       </c>
@@ -2267,12 +2274,12 @@
       <c r="G34" s="1"/>
       <c r="H34" s="1"/>
       <c r="I34" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J34" s="1"/>
       <c r="K34" s="1"/>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>38</v>
       </c>
@@ -2290,12 +2297,12 @@
       <c r="G35" s="1"/>
       <c r="H35" s="1"/>
       <c r="I35" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J35" s="1"/>
       <c r="K35" s="1"/>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>39</v>
       </c>
@@ -2313,12 +2320,12 @@
       <c r="G36" s="1"/>
       <c r="H36" s="1"/>
       <c r="I36" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J36" s="1"/>
       <c r="K36" s="1"/>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>40</v>
       </c>
@@ -2336,12 +2343,12 @@
       <c r="G37" s="1"/>
       <c r="H37" s="1"/>
       <c r="I37" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J37" s="1"/>
       <c r="K37" s="1"/>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>41</v>
       </c>
@@ -2359,12 +2366,12 @@
       <c r="G38" s="1"/>
       <c r="H38" s="1"/>
       <c r="I38" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J38" s="1"/>
       <c r="K38" s="1"/>
     </row>
-    <row r="39" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>43</v>
       </c>
@@ -2382,12 +2389,12 @@
       <c r="G39" s="1"/>
       <c r="H39" s="1"/>
       <c r="I39" s="1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="J39" s="1"/>
       <c r="K39" s="1"/>
     </row>
-    <row r="40" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
         <v>44</v>
       </c>
@@ -2405,12 +2412,12 @@
       <c r="G40" s="1"/>
       <c r="H40" s="1"/>
       <c r="I40" s="1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="J40" s="1"/>
       <c r="K40" s="1"/>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
         <v>11</v>
       </c>
@@ -2430,14 +2437,14 @@
       </c>
       <c r="H41" s="1"/>
       <c r="I41" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J41" s="1"/>
       <c r="K41" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
         <v>12</v>
       </c>
@@ -2457,14 +2464,14 @@
       </c>
       <c r="H42" s="1"/>
       <c r="I42" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J42" s="1"/>
       <c r="K42" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="43" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
         <v>13</v>
       </c>
@@ -2484,14 +2491,14 @@
       </c>
       <c r="H43" s="1"/>
       <c r="I43" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J43" s="1"/>
       <c r="K43" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="44" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
         <v>14</v>
       </c>
@@ -2511,14 +2518,14 @@
       </c>
       <c r="H44" s="1"/>
       <c r="I44" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J44" s="1"/>
       <c r="K44" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
         <v>15</v>
       </c>
@@ -2538,14 +2545,14 @@
       </c>
       <c r="H45" s="1"/>
       <c r="I45" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J45" s="1"/>
       <c r="K45" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
         <v>16</v>
       </c>
@@ -2565,14 +2572,14 @@
       </c>
       <c r="H46" s="1"/>
       <c r="I46" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J46" s="1"/>
       <c r="K46" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>17</v>
       </c>
@@ -2589,18 +2596,18 @@
       <c r="E47" s="1"/>
       <c r="F47" s="1"/>
       <c r="G47" s="1" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="H47" s="1"/>
       <c r="I47" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J47" s="1"/>
       <c r="K47" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
         <v>18</v>
       </c>
@@ -2620,18 +2627,18 @@
         <v>290</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="H48" s="1"/>
       <c r="I48" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="J48" s="1"/>
       <c r="K48" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>19</v>
       </c>
@@ -2651,18 +2658,18 @@
         <v>1481</v>
       </c>
       <c r="G49" s="1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="H49" s="1"/>
       <c r="I49" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="J49" s="1"/>
       <c r="K49" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
         <v>20</v>
       </c>
@@ -2678,18 +2685,18 @@
       <c r="E50" s="1"/>
       <c r="F50" s="1"/>
       <c r="G50" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="H50" s="3"/>
       <c r="I50" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J50" s="1"/>
       <c r="K50" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A51" s="1" t="s">
         <v>21</v>
       </c>
@@ -2709,18 +2716,18 @@
         <v>960</v>
       </c>
       <c r="G51" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="H51" s="3"/>
       <c r="I51" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J51" s="1"/>
       <c r="K51" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="52" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
         <v>37</v>
       </c>
@@ -2740,14 +2747,14 @@
       </c>
       <c r="H52" s="1"/>
       <c r="I52" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J52" s="1"/>
       <c r="K52" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="53" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A53" s="1" t="s">
         <v>38</v>
       </c>
@@ -2767,14 +2774,14 @@
       </c>
       <c r="H53" s="1"/>
       <c r="I53" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J53" s="1"/>
       <c r="K53" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="54" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
         <v>39</v>
       </c>
@@ -2794,14 +2801,14 @@
       </c>
       <c r="H54" s="1"/>
       <c r="I54" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J54" s="1"/>
       <c r="K54" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A55" s="1" t="s">
         <v>40</v>
       </c>
@@ -2819,14 +2826,14 @@
       <c r="G55" s="1"/>
       <c r="H55" s="1"/>
       <c r="I55" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J55" s="1"/>
       <c r="K55" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="56" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
         <v>41</v>
       </c>
@@ -2846,14 +2853,14 @@
       </c>
       <c r="H56" s="1"/>
       <c r="I56" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J56" s="1"/>
       <c r="K56" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="57" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
         <v>43</v>
       </c>
@@ -2873,14 +2880,14 @@
       </c>
       <c r="H57" s="1"/>
       <c r="I57" s="1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="J57" s="1"/>
       <c r="K57" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="58" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A58" s="1" t="s">
         <v>44</v>
       </c>
@@ -2896,20 +2903,20 @@
       <c r="E58" s="1"/>
       <c r="F58" s="1"/>
       <c r="G58" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H58" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="I58" s="1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="J58" s="1"/>
       <c r="K58" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
         <v>11</v>
       </c>
@@ -2929,14 +2936,14 @@
       </c>
       <c r="H59" s="1"/>
       <c r="I59" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J59" s="1"/>
       <c r="K59" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A60" s="1" t="s">
         <v>12</v>
       </c>
@@ -2956,14 +2963,14 @@
       </c>
       <c r="H60" s="1"/>
       <c r="I60" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J60" s="1"/>
       <c r="K60" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="61" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A61" s="1" t="s">
         <v>13</v>
       </c>
@@ -2983,14 +2990,14 @@
       </c>
       <c r="H61" s="1"/>
       <c r="I61" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J61" s="1"/>
       <c r="K61" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="62" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A62" s="1" t="s">
         <v>14</v>
       </c>
@@ -3010,14 +3017,14 @@
       </c>
       <c r="H62" s="1"/>
       <c r="I62" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J62" s="1"/>
       <c r="K62" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A63" s="1" t="s">
         <v>15</v>
       </c>
@@ -3037,14 +3044,14 @@
       </c>
       <c r="H63" s="1"/>
       <c r="I63" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J63" s="1"/>
       <c r="K63" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A64" s="1" t="s">
         <v>16</v>
       </c>
@@ -3064,14 +3071,14 @@
       </c>
       <c r="H64" s="1"/>
       <c r="I64" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J64" s="1"/>
       <c r="K64" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A65" s="1" t="s">
         <v>17</v>
       </c>
@@ -3088,18 +3095,18 @@
       <c r="E65" s="1"/>
       <c r="F65" s="1"/>
       <c r="G65" s="1" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="H65" s="1"/>
       <c r="I65" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J65" s="1"/>
       <c r="K65" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A66" s="1" t="s">
         <v>18</v>
       </c>
@@ -3119,18 +3126,18 @@
         <v>290</v>
       </c>
       <c r="G66" s="1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="H66" s="1"/>
       <c r="I66" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="J66" s="1"/>
       <c r="K66" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A67" s="1" t="s">
         <v>19</v>
       </c>
@@ -3150,18 +3157,18 @@
         <v>1481</v>
       </c>
       <c r="G67" s="1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="H67" s="1"/>
       <c r="I67" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="J67" s="1"/>
       <c r="K67" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A68" s="1" t="s">
         <v>20</v>
       </c>
@@ -3177,18 +3184,18 @@
       <c r="E68" s="1"/>
       <c r="F68" s="1"/>
       <c r="G68" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="H68" s="3"/>
       <c r="I68" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J68" s="1"/>
       <c r="K68" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A69" s="1" t="s">
         <v>21</v>
       </c>
@@ -3208,18 +3215,18 @@
         <v>960</v>
       </c>
       <c r="G69" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="H69" s="3"/>
       <c r="I69" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J69" s="1"/>
       <c r="K69" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="70" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A70" s="1" t="s">
         <v>37</v>
       </c>
@@ -3239,14 +3246,14 @@
       </c>
       <c r="H70" s="1"/>
       <c r="I70" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J70" s="1"/>
       <c r="K70" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="71" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A71" s="1" t="s">
         <v>38</v>
       </c>
@@ -3266,14 +3273,14 @@
       </c>
       <c r="H71" s="1"/>
       <c r="I71" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J71" s="1"/>
       <c r="K71" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="72" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A72" s="1" t="s">
         <v>39</v>
       </c>
@@ -3293,14 +3300,14 @@
       </c>
       <c r="H72" s="1"/>
       <c r="I72" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J72" s="1"/>
       <c r="K72" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A73" s="1" t="s">
         <v>40</v>
       </c>
@@ -3318,14 +3325,14 @@
       <c r="G73" s="1"/>
       <c r="H73" s="1"/>
       <c r="I73" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J73" s="1"/>
       <c r="K73" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="74" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A74" s="1" t="s">
         <v>41</v>
       </c>
@@ -3345,14 +3352,14 @@
       </c>
       <c r="H74" s="1"/>
       <c r="I74" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J74" s="1"/>
       <c r="K74" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="75" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A75" s="1" t="s">
         <v>43</v>
       </c>
@@ -3370,14 +3377,14 @@
       <c r="G75" s="1"/>
       <c r="H75" s="1"/>
       <c r="I75" s="1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="J75" s="1"/>
       <c r="K75" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="76" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A76" s="1" t="s">
         <v>44</v>
       </c>
@@ -3393,20 +3400,20 @@
       <c r="E76" s="1"/>
       <c r="F76" s="1"/>
       <c r="G76" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H76" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="I76" s="1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="J76" s="1"/>
       <c r="K76" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="77" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A77" s="1" t="s">
         <v>54</v>
       </c>
@@ -3426,14 +3433,14 @@
       </c>
       <c r="H77" s="1"/>
       <c r="I77" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J77" s="1"/>
       <c r="K77" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="78" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A78" s="1" t="s">
         <v>55</v>
       </c>
@@ -3453,14 +3460,14 @@
       </c>
       <c r="H78" s="1"/>
       <c r="I78" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J78" s="1"/>
       <c r="K78" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="79" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A79" s="1" t="s">
         <v>56</v>
       </c>
@@ -3480,14 +3487,14 @@
       </c>
       <c r="H79" s="1"/>
       <c r="I79" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J79" s="1"/>
       <c r="K79" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A80" s="1" t="s">
         <v>57</v>
       </c>
@@ -3505,14 +3512,14 @@
       <c r="G80" s="1"/>
       <c r="H80" s="1"/>
       <c r="I80" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J80" s="1"/>
       <c r="K80" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="81" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A81" s="1" t="s">
         <v>58</v>
       </c>
@@ -3532,14 +3539,14 @@
       </c>
       <c r="H81" s="1"/>
       <c r="I81" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J81" s="1"/>
       <c r="K81" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A82" s="1" t="s">
         <v>11</v>
       </c>
@@ -3556,20 +3563,20 @@
       <c r="E82" s="1"/>
       <c r="F82" s="1"/>
       <c r="G82" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="H82" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="I82" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J82" s="1"/>
       <c r="K82" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A83" s="1" t="s">
         <v>12</v>
       </c>
@@ -3586,20 +3593,20 @@
       <c r="E83" s="1"/>
       <c r="F83" s="1"/>
       <c r="G83" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="H83" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="I83" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J83" s="1"/>
       <c r="K83" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="84" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A84" s="1" t="s">
         <v>13</v>
       </c>
@@ -3616,20 +3623,20 @@
       <c r="E84" s="1"/>
       <c r="F84" s="1"/>
       <c r="G84" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="H84" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="I84" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J84" s="1"/>
       <c r="K84" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="85" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A85" s="1" t="s">
         <v>14</v>
       </c>
@@ -3646,20 +3653,20 @@
       <c r="E85" s="1"/>
       <c r="F85" s="1"/>
       <c r="G85" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="H85" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="I85" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J85" s="1"/>
       <c r="K85" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="86" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A86" s="1" t="s">
         <v>15</v>
       </c>
@@ -3676,20 +3683,20 @@
       <c r="E86" s="1"/>
       <c r="F86" s="1"/>
       <c r="G86" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="H86" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="I86" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J86" s="1"/>
       <c r="K86" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="87" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A87" s="1" t="s">
         <v>16</v>
       </c>
@@ -3706,20 +3713,20 @@
       <c r="E87" s="1"/>
       <c r="F87" s="1"/>
       <c r="G87" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="H87" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="I87" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J87" s="1"/>
       <c r="K87" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="88" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A88" s="1" t="s">
         <v>17</v>
       </c>
@@ -3736,20 +3743,20 @@
       <c r="E88" s="1"/>
       <c r="F88" s="1"/>
       <c r="G88" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="H88" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="I88" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J88" s="1"/>
       <c r="K88" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="89" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A89" s="1" t="s">
         <v>18</v>
       </c>
@@ -3766,20 +3773,20 @@
       <c r="E89" s="1"/>
       <c r="F89" s="1"/>
       <c r="G89" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="H89" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="I89" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="J89" s="1"/>
       <c r="K89" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="90" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A90" s="1" t="s">
         <v>19</v>
       </c>
@@ -3796,20 +3803,20 @@
       <c r="E90" s="1"/>
       <c r="F90" s="1"/>
       <c r="G90" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="H90" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="I90" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="J90" s="1"/>
       <c r="K90" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="91" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A91" s="1" t="s">
         <v>20</v>
       </c>
@@ -3826,20 +3833,20 @@
       <c r="E91" s="1"/>
       <c r="F91" s="1"/>
       <c r="G91" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="H91" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="I91" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J91" s="1"/>
       <c r="K91" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="92" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A92" s="1" t="s">
         <v>21</v>
       </c>
@@ -3856,20 +3863,20 @@
       <c r="E92" s="1"/>
       <c r="F92" s="1"/>
       <c r="G92" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="H92" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="I92" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J92" s="1"/>
       <c r="K92" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="93" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A93" s="1" t="s">
         <v>61</v>
       </c>
@@ -3886,20 +3893,20 @@
       <c r="E93" s="1"/>
       <c r="F93" s="1"/>
       <c r="G93" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="H93" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="I93" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J93" s="1"/>
       <c r="K93" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="94" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="94" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A94" s="1" t="s">
         <v>62</v>
       </c>
@@ -3917,20 +3924,20 @@
       <c r="E94" s="1"/>
       <c r="F94" s="1"/>
       <c r="G94" s="4" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="H94" s="1" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="I94" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J94" s="1"/>
       <c r="K94" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="95" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A95" s="1" t="s">
         <v>63</v>
       </c>
@@ -3947,20 +3954,20 @@
       <c r="E95" s="1"/>
       <c r="F95" s="1"/>
       <c r="G95" s="1" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="H95" s="1" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="I95" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J95" s="1"/>
       <c r="K95" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="96" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A96" s="1" t="s">
         <v>64</v>
       </c>
@@ -3977,20 +3984,20 @@
       <c r="E96" s="1"/>
       <c r="F96" s="1"/>
       <c r="G96" s="1" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="H96" s="1" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="I96" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J96" s="1"/>
       <c r="K96" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="97" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A97" s="1" t="s">
         <v>65</v>
       </c>
@@ -4008,22 +4015,22 @@
       <c r="G97" s="1"/>
       <c r="H97" s="1"/>
       <c r="I97" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J97" s="1"/>
       <c r="K97" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="98" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="98" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A98" s="1" t="s">
         <v>66</v>
       </c>
       <c r="B98" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C98" s="2" t="s">
-        <v>67</v>
+      <c r="C98" s="5">
+        <v>2.7399999999999999E-5</v>
       </c>
       <c r="D98" s="1">
         <f>Table1[[#This Row],[Value]]*2</f>
@@ -4032,28 +4039,28 @@
       <c r="E98" s="1"/>
       <c r="F98" s="1"/>
       <c r="G98" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="H98" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="H98" s="1" t="s">
-        <v>86</v>
-      </c>
       <c r="I98" s="1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="J98" s="1"/>
       <c r="K98" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="99" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A99" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B99" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C99" s="2" t="s">
-        <v>69</v>
+      <c r="C99" s="5">
+        <v>1.2999999999999999E-5</v>
       </c>
       <c r="D99" s="1">
         <f>Table1[[#This Row],[Value]]*2</f>
@@ -4062,17 +4069,17 @@
       <c r="E99" s="1"/>
       <c r="F99" s="1"/>
       <c r="G99" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="H99" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="H99" s="1" t="s">
-        <v>86</v>
-      </c>
       <c r="I99" s="1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="J99" s="1"/>
       <c r="K99" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -4086,38 +4093,38 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA0710C0-AB94-4FBF-AB29-E5085BC4F559}">
   <dimension ref="A1:F22"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.7109375" customWidth="1"/>
+    <col min="1" max="1" width="11.7265625" customWidth="1"/>
     <col min="2" max="2" width="20" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.85546875" customWidth="1"/>
+    <col min="3" max="3" width="13.81640625" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="35.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="35.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D1" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E1" t="s">
         <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B2" t="s">
         <v>35</v>
@@ -4130,15 +4137,15 @@
         <v>6.45</v>
       </c>
       <c r="E2" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F2" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B3" t="s">
         <v>36</v>
@@ -4147,9 +4154,9 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B4" t="s">
         <v>45</v>
@@ -4161,15 +4168,15 @@
         <v>0.1</v>
       </c>
       <c r="E4" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="F4" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B5" t="s">
         <v>53</v>
@@ -4181,15 +4188,15 @@
         <v>0.1</v>
       </c>
       <c r="E5" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="F5" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B6" t="s">
         <v>53</v>
@@ -4201,15 +4208,15 @@
         <v>0.1</v>
       </c>
       <c r="E6" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="F6" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B7" t="s">
         <v>60</v>
@@ -4221,310 +4228,310 @@
         <v>0.1</v>
       </c>
       <c r="E7" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F7" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B8" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C8" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D8">
         <v>200</v>
       </c>
       <c r="E8" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F8" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B9" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C9" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="D9">
         <v>200</v>
       </c>
       <c r="E9" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F9" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B10" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C10" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D10">
         <v>750</v>
       </c>
       <c r="E10" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F10" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
+        <v>93</v>
+      </c>
+      <c r="B11" t="s">
+        <v>93</v>
+      </c>
+      <c r="C11" t="s">
         <v>95</v>
-      </c>
-      <c r="B11" t="s">
-        <v>95</v>
-      </c>
-      <c r="C11" t="s">
-        <v>97</v>
       </c>
       <c r="D11">
         <v>6750</v>
       </c>
       <c r="E11" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F11" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B12" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C12" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D12">
         <v>2500</v>
       </c>
       <c r="E12" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F12" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B13" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C13" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D13">
         <v>200</v>
       </c>
       <c r="E13" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F13" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B14" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C14" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D14">
         <v>1000</v>
       </c>
       <c r="E14" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F14" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B15" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C15" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D15">
         <v>2000</v>
       </c>
       <c r="E15" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F15" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B16" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C16" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D16">
         <v>10</v>
       </c>
       <c r="E16" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F16" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B17" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C17" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D17">
         <v>0.1</v>
       </c>
       <c r="E17" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F17" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B18" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C18" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D18">
         <v>400</v>
       </c>
       <c r="E18" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F18" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B19" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C19" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D19">
         <v>10</v>
       </c>
       <c r="E19" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F19" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B20" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C20" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D20">
         <v>1000</v>
       </c>
       <c r="E20" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F20" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B21" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C21" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D21">
         <v>3000</v>
       </c>
       <c r="E21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F21" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B22" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C22" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="D22">
         <v>40</v>
       </c>
       <c r="E22" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F22" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -4533,26 +4540,199 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFDB7072-D0E7-4AF9-A2DD-825DB900D6FF}">
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="12.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.08984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25.36328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.453125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>91</v>
+      </c>
+      <c r="D1" t="s">
+        <v>127</v>
+      </c>
+      <c r="E1" t="s">
+        <v>128</v>
+      </c>
+      <c r="F1" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D2" t="s">
+        <v>104</v>
+      </c>
+      <c r="E2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>93</v>
+      </c>
+      <c r="B3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" t="s">
+        <v>99</v>
+      </c>
+      <c r="E3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" t="s">
+        <v>97</v>
+      </c>
+      <c r="E4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>93</v>
+      </c>
+      <c r="B5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" t="s">
+        <v>99</v>
+      </c>
+      <c r="E5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>93</v>
+      </c>
+      <c r="B6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" t="s">
+        <v>97</v>
+      </c>
+      <c r="E6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>93</v>
+      </c>
+      <c r="B7" t="s">
+        <v>53</v>
+      </c>
+      <c r="C7" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" t="s">
+        <v>99</v>
+      </c>
+      <c r="E7" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>93</v>
+      </c>
+      <c r="B8" t="s">
+        <v>53</v>
+      </c>
+      <c r="C8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" t="s">
+        <v>97</v>
+      </c>
+      <c r="E8" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>93</v>
+      </c>
+      <c r="B9" t="s">
+        <v>60</v>
+      </c>
+      <c r="C9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" t="s">
+        <v>129</v>
+      </c>
+      <c r="E9" t="s">
+        <v>67</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC182590-26D0-4168-8E7C-B448CD67FE47}">
   <dimension ref="A1:C31"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.7265625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -4563,7 +4743,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -4574,7 +4754,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -4585,7 +4765,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -4596,7 +4776,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -4607,7 +4787,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -4618,7 +4798,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -4629,7 +4809,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>6</v>
       </c>
@@ -4640,7 +4820,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>7</v>
       </c>
@@ -4651,7 +4831,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -4662,7 +4842,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -4673,7 +4853,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>10</v>
       </c>
@@ -4684,7 +4864,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>5</v>
       </c>
@@ -4695,7 +4875,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>6</v>
       </c>
@@ -4706,7 +4886,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>7</v>
       </c>
@@ -4717,7 +4897,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>8</v>
       </c>
@@ -4728,7 +4908,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>9</v>
       </c>
@@ -4739,7 +4919,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>10</v>
       </c>
@@ -4750,7 +4930,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>5</v>
       </c>
@@ -4761,7 +4941,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>6</v>
       </c>
@@ -4772,7 +4952,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>7</v>
       </c>
@@ -4783,7 +4963,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>8</v>
       </c>
@@ -4794,7 +4974,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>9</v>
       </c>
@@ -4805,7 +4985,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>10</v>
       </c>
@@ -4816,7 +4996,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>5</v>
       </c>
@@ -4827,7 +5007,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>6</v>
       </c>
@@ -4838,7 +5018,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>7</v>
       </c>
@@ -4849,7 +5029,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>8</v>
       </c>
@@ -4860,7 +5040,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>9</v>
       </c>
@@ -4871,7 +5051,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Modified the code so that the animal fit doesn't always fit the effect sizes, because this is challenging to work with.
</commit_message>
<xml_diff>
--- a/Data/scenarios.xlsx
+++ b/Data/scenarios.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rober\Documents\GitHub Repos\merging_SFW_decomposition_models\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{489B97FC-7726-481C-A9C3-B0F72E9D162D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A252B0D-9B1D-43E6-9CA2-1EA286133C0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" activeTab="1" xr2:uid="{7C97690C-9E7B-4D0E-86C0-16835BCB4BB0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" activeTab="2" xr2:uid="{7C97690C-9E7B-4D0E-86C0-16835BCB4BB0}"/>
   </bookViews>
   <sheets>
     <sheet name="scenarios" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="730" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="753" uniqueCount="138">
   <si>
     <t>Parameter</t>
   </si>
@@ -124,9 +124,6 @@
     <t>Petersen + Luxton 1982</t>
   </si>
   <si>
-    <t>E_earthworm</t>
-  </si>
-  <si>
     <t>c_earthworm_litter</t>
   </si>
   <si>
@@ -157,9 +154,6 @@
     <t>p_detritivores</t>
   </si>
   <si>
-    <t>E_detritivores</t>
-  </si>
-  <si>
     <t>c_detritivores</t>
   </si>
   <si>
@@ -208,9 +202,6 @@
     <t>p_detpredator</t>
   </si>
   <si>
-    <t>E_detpredator</t>
-  </si>
-  <si>
     <t>c_detpredator</t>
   </si>
   <si>
@@ -232,9 +223,6 @@
     <t>p_rootherb</t>
   </si>
   <si>
-    <t>E_root_herb</t>
-  </si>
-  <si>
     <t>k_exudate_intercept</t>
   </si>
   <si>
@@ -442,7 +430,25 @@
     <t>day-1</t>
   </si>
   <si>
-    <t>Mulder et al. 2007; Buchkowski et al. 2024</t>
+    <t>Buchkowski et al. 2024 converted to per gram earthworm carbon</t>
+  </si>
+  <si>
+    <t>Mulder et al. 2007; Buchkowski et al. 2024; from Lavelle et al. 1987, Hamoui 1981, Brown et al. unpublished, Lavelle 1979</t>
+  </si>
+  <si>
+    <t>Need to explore this more to get a better number</t>
+  </si>
+  <si>
+    <t>Warburg et al. 1984 2.5 year lifespan</t>
+  </si>
+  <si>
+    <t>Topp et al. 2006 SBB</t>
+  </si>
+  <si>
+    <t>Topp et al. 2006 for density, NM&amp;M lab for weight</t>
+  </si>
+  <si>
+    <t>Need to refine</t>
   </si>
 </sst>
 </file>
@@ -1056,21 +1062,21 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1759F6D4-436C-4273-8592-6F473E4E1FC6}" name="Table1" displayName="Table1" ref="A1:L99" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
-  <autoFilter ref="A1:L99" xr:uid="{1759F6D4-436C-4273-8592-6F473E4E1FC6}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1759F6D4-436C-4273-8592-6F473E4E1FC6}" name="Table1" displayName="Table1" ref="A1:L93" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+  <autoFilter ref="A1:L93" xr:uid="{1759F6D4-436C-4273-8592-6F473E4E1FC6}"/>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{9C63AD24-02BE-4FC6-8589-25FEAC9E29E1}" name="Parameter" dataDxfId="11"/>
     <tableColumn id="2" xr3:uid="{6FFFFAD3-CDDD-4A47-9019-7C5E6785F73D}" name="Scenario" dataDxfId="10"/>
-    <tableColumn id="12" xr3:uid="{624CA8D0-C933-480B-99CE-4C2DA98C9671}" name="Units" dataDxfId="0"/>
-    <tableColumn id="3" xr3:uid="{43A09F60-45AF-4366-B3C3-21E470E20743}" name="Value" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{58AE1493-138A-4C0F-B37F-DC15984C1B4D}" name="SD" dataDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{C2652975-ACD3-4499-9A4F-55E61AF86737}" name="Min" dataDxfId="7"/>
-    <tableColumn id="6" xr3:uid="{9D50F876-8F5B-4BBE-BE99-655FCFAB6B55}" name="Max" dataDxfId="6"/>
-    <tableColumn id="7" xr3:uid="{E3199168-8B68-4130-96B7-37F35FEADAB4}" name="Reference" dataDxfId="5"/>
-    <tableColumn id="10" xr3:uid="{7383E6E0-56E5-496B-9287-EE6E2AA3B268}" name="Help needed" dataDxfId="4"/>
-    <tableColumn id="9" xr3:uid="{5A5E5207-A16E-4A54-BB54-6D4FB1E75949}" name="Category" dataDxfId="3"/>
-    <tableColumn id="11" xr3:uid="{D48D6FAC-CC1D-441E-ACFF-3C1405C9376B}" name="Status (Case study group)" dataDxfId="2"/>
-    <tableColumn id="8" xr3:uid="{F2E55EFF-159B-4FD3-B12E-2E3149126C35}" name="Status (Rob)" dataDxfId="1"/>
+    <tableColumn id="12" xr3:uid="{624CA8D0-C933-480B-99CE-4C2DA98C9671}" name="Units" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{43A09F60-45AF-4366-B3C3-21E470E20743}" name="Value" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{58AE1493-138A-4C0F-B37F-DC15984C1B4D}" name="SD" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{C2652975-ACD3-4499-9A4F-55E61AF86737}" name="Min" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{9D50F876-8F5B-4BBE-BE99-655FCFAB6B55}" name="Max" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{E3199168-8B68-4130-96B7-37F35FEADAB4}" name="Reference" dataDxfId="4"/>
+    <tableColumn id="10" xr3:uid="{7383E6E0-56E5-496B-9287-EE6E2AA3B268}" name="Help needed" dataDxfId="3"/>
+    <tableColumn id="9" xr3:uid="{5A5E5207-A16E-4A54-BB54-6D4FB1E75949}" name="Category" dataDxfId="2"/>
+    <tableColumn id="11" xr3:uid="{D48D6FAC-CC1D-441E-ACFF-3C1405C9376B}" name="Status (Case study group)" dataDxfId="1"/>
+    <tableColumn id="8" xr3:uid="{F2E55EFF-159B-4FD3-B12E-2E3149126C35}" name="Status (Rob)" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1393,7 +1399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD4418A0-EB93-4361-AE80-4D25DF544368}">
-  <dimension ref="A1:L99"/>
+  <dimension ref="A1:L93"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.28515625" bestFit="1" customWidth="1"/>
@@ -1414,7 +1420,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>2</v>
@@ -1423,25 +1429,25 @@
         <v>3</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
@@ -1449,10 +1455,10 @@
         <v>11</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="D2" s="1">
         <v>6</v>
@@ -1463,15 +1469,15 @@
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
       <c r="H2" s="1" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="I2" s="1"/>
       <c r="J2" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K2" s="1"/>
       <c r="L2" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
@@ -1479,10 +1485,10 @@
         <v>12</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="D3" s="1">
         <v>26</v>
@@ -1495,11 +1501,11 @@
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K3" s="1"/>
       <c r="L3" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
@@ -1507,10 +1513,10 @@
         <v>13</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="D4" s="1">
         <v>0.3</v>
@@ -1523,11 +1529,11 @@
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K4" s="1"/>
       <c r="L4" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
@@ -1535,10 +1541,10 @@
         <v>14</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="D5" s="1">
         <v>0.15</v>
@@ -1551,11 +1557,11 @@
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
       <c r="J5" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K5" s="1"/>
       <c r="L5" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
@@ -1563,10 +1569,10 @@
         <v>15</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="D6" s="1">
         <v>73</v>
@@ -1581,15 +1587,15 @@
         <v>78</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="I6" s="1"/>
       <c r="J6" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K6" s="1"/>
       <c r="L6" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
@@ -1597,10 +1603,10 @@
         <v>16</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="D7" s="1">
         <v>0.28000000000000003</v>
@@ -1615,15 +1621,15 @@
         <v>0.33</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="I7" s="1"/>
       <c r="J7" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K7" s="1"/>
       <c r="L7" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="30" x14ac:dyDescent="0.25">
@@ -1631,10 +1637,10 @@
         <v>17</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="D8" s="1">
         <v>0.2</v>
@@ -1649,17 +1655,17 @@
         <v>0.3</v>
       </c>
       <c r="H8" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K8" s="1"/>
       <c r="L8" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
@@ -1667,10 +1673,10 @@
         <v>18</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="D9" s="6">
         <f>D10*0.03</f>
@@ -1689,15 +1695,15 @@
         <v>17.920000000000002</v>
       </c>
       <c r="H9" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="I9" s="1"/>
       <c r="J9" s="1" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="K9" s="1"/>
       <c r="L9" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
@@ -1705,10 +1711,10 @@
         <v>19</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="D10" s="1">
         <f>336/0.75</f>
@@ -1727,15 +1733,15 @@
         <v>448</v>
       </c>
       <c r="H10" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="I10" s="1"/>
       <c r="J10" s="1" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="K10" s="1"/>
       <c r="L10" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
@@ -1743,7 +1749,7 @@
         <v>20</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C11" s="1"/>
       <c r="D11" s="1">
@@ -1759,15 +1765,15 @@
         <v>8</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="I11" s="1"/>
       <c r="J11" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K11" s="1"/>
       <c r="L11" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="30" x14ac:dyDescent="0.25">
@@ -1775,10 +1781,10 @@
         <v>21</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="D12" s="1">
         <v>700</v>
@@ -1793,26 +1799,26 @@
         <v>1160</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="I12" s="1"/>
       <c r="J12" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K12" s="1"/>
       <c r="L12" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>22</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="D13" s="1">
         <f>0.217/365/6.45</f>
@@ -1824,19 +1830,19 @@
         <v>9.2173728363597747E-5</v>
       </c>
       <c r="G13" s="1">
-        <f>0.5/365/6.45</f>
-        <v>2.1238186258893489E-4</v>
+        <f>0.0018/6.45</f>
+        <v>2.7906976744186045E-4</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="I13" s="1"/>
       <c r="J13" s="1" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="K13" s="1"/>
       <c r="L13" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
@@ -1844,10 +1850,10 @@
         <v>23</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="D14" s="1">
         <v>0.53</v>
@@ -1862,11 +1868,11 @@
       </c>
       <c r="I14" s="1"/>
       <c r="J14" s="1" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="K14" s="1"/>
       <c r="L14" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
@@ -1874,10 +1880,10 @@
         <v>25</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="D15" s="1">
         <v>0.09</v>
@@ -1892,11 +1898,11 @@
       </c>
       <c r="I15" s="1"/>
       <c r="J15" s="1" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="K15" s="1"/>
       <c r="L15" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
@@ -1904,10 +1910,10 @@
         <v>27</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="D16" s="1">
         <v>0.22</v>
@@ -1922,37 +1928,42 @@
       </c>
       <c r="I16" s="1"/>
       <c r="J16" s="1" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="K16" s="1"/>
       <c r="L16" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>29</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1">
-        <v>0</v>
+        <v>34</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="D17" s="5">
+        <f>0.00207/0.0375</f>
+        <v>5.5199999999999999E-2</v>
       </c>
       <c r="E17" s="1">
         <v>0</v>
       </c>
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
-      <c r="H17" s="1"/>
+      <c r="H17" s="1" t="s">
+        <v>131</v>
+      </c>
       <c r="I17" s="1"/>
       <c r="J17" s="1" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="K17" s="1"/>
       <c r="L17" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="18" spans="1:12" ht="30" x14ac:dyDescent="0.25">
@@ -1960,65 +1971,75 @@
         <v>30</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="D18" s="5">
-        <v>1.89202E-4</v>
+        <f>0.00207/0.0375</f>
+        <v>5.5199999999999999E-2</v>
       </c>
       <c r="E18" s="1">
         <v>0</v>
       </c>
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
-      <c r="H18" s="1"/>
+      <c r="H18" s="1" t="s">
+        <v>131</v>
+      </c>
       <c r="I18" s="1"/>
       <c r="J18" s="1" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="K18" s="1"/>
-      <c r="L18" s="1"/>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L18" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>31</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="D19" s="5">
-        <v>1.89202E-4</v>
+        <f>0.00207/0.0375</f>
+        <v>5.5199999999999999E-2</v>
       </c>
       <c r="E19" s="1">
         <v>0</v>
       </c>
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
-      <c r="H19" s="1"/>
+      <c r="H19" s="1" t="s">
+        <v>131</v>
+      </c>
       <c r="I19" s="1"/>
       <c r="J19" s="1" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="K19" s="1"/>
-      <c r="L19" s="1"/>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L19" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>32</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="D20" s="5">
-        <v>1.89202E-4</v>
+        <v>125</v>
+      </c>
+      <c r="D20" s="1">
+        <v>0</v>
       </c>
       <c r="E20" s="1">
         <v>0</v>
@@ -2026,25 +2047,29 @@
       <c r="F20" s="1"/>
       <c r="G20" s="1"/>
       <c r="H20" s="1"/>
-      <c r="I20" s="1"/>
+      <c r="I20" s="1" t="s">
+        <v>120</v>
+      </c>
       <c r="J20" s="1" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="K20" s="1"/>
-      <c r="L20" s="1"/>
-    </row>
-    <row r="21" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="L20" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>33</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="D21" s="1">
-        <v>0</v>
+        <v>-0.02</v>
       </c>
       <c r="E21" s="1">
         <v>0</v>
@@ -2053,26 +2078,28 @@
       <c r="G21" s="1"/>
       <c r="H21" s="1"/>
       <c r="I21" s="1" t="s">
-        <v>124</v>
+        <v>133</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="K21" s="1"/>
-      <c r="L21" s="1"/>
+      <c r="L21" s="1" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>35</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D22" s="1">
-        <v>-0.02</v>
+        <v>6</v>
       </c>
       <c r="E22" s="1">
         <v>0</v>
@@ -2080,25 +2107,29 @@
       <c r="F22" s="1"/>
       <c r="G22" s="1"/>
       <c r="H22" s="1"/>
-      <c r="I22" s="1"/>
+      <c r="I22" s="1" t="s">
+        <v>137</v>
+      </c>
       <c r="J22" s="1" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="K22" s="1"/>
-      <c r="L22" s="1"/>
+      <c r="L22" s="1" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="D23" s="1">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="E23" s="1">
         <v>0</v>
@@ -2106,25 +2137,29 @@
       <c r="F23" s="1"/>
       <c r="G23" s="1"/>
       <c r="H23" s="1"/>
-      <c r="I23" s="1"/>
+      <c r="I23" s="1" t="s">
+        <v>137</v>
+      </c>
       <c r="J23" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K23" s="1"/>
-      <c r="L23" s="1"/>
+      <c r="L23" s="1" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="D24" s="1">
-        <v>26</v>
+        <v>0.3</v>
       </c>
       <c r="E24" s="1">
         <v>0</v>
@@ -2132,25 +2167,29 @@
       <c r="F24" s="1"/>
       <c r="G24" s="1"/>
       <c r="H24" s="1"/>
-      <c r="I24" s="1"/>
+      <c r="I24" s="1" t="s">
+        <v>137</v>
+      </c>
       <c r="J24" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K24" s="1"/>
-      <c r="L24" s="1"/>
+      <c r="L24" s="1" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="D25" s="1">
-        <v>0.3</v>
+        <v>0.15</v>
       </c>
       <c r="E25" s="1">
         <v>0</v>
@@ -2158,25 +2197,29 @@
       <c r="F25" s="1"/>
       <c r="G25" s="1"/>
       <c r="H25" s="1"/>
-      <c r="I25" s="1"/>
+      <c r="I25" s="1" t="s">
+        <v>137</v>
+      </c>
       <c r="J25" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K25" s="1"/>
-      <c r="L25" s="1"/>
+      <c r="L25" s="1" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>133</v>
+        <v>124</v>
       </c>
       <c r="D26" s="1">
-        <v>0.15</v>
+        <v>70</v>
       </c>
       <c r="E26" s="1">
         <v>0</v>
@@ -2184,25 +2227,29 @@
       <c r="F26" s="1"/>
       <c r="G26" s="1"/>
       <c r="H26" s="1"/>
-      <c r="I26" s="1"/>
+      <c r="I26" s="1" t="s">
+        <v>137</v>
+      </c>
       <c r="J26" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K26" s="1"/>
-      <c r="L26" s="1"/>
+      <c r="L26" s="1" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="D27" s="1">
-        <v>70</v>
+        <v>0.4</v>
       </c>
       <c r="E27" s="1">
         <v>0</v>
@@ -2210,25 +2257,29 @@
       <c r="F27" s="1"/>
       <c r="G27" s="1"/>
       <c r="H27" s="1"/>
-      <c r="I27" s="1"/>
+      <c r="I27" s="1" t="s">
+        <v>137</v>
+      </c>
       <c r="J27" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K27" s="1"/>
-      <c r="L27" s="1"/>
+      <c r="L27" s="1" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="D28" s="1">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="E28" s="1">
         <v>0</v>
@@ -2236,25 +2287,29 @@
       <c r="F28" s="1"/>
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
-      <c r="I28" s="1"/>
+      <c r="I28" s="1" t="s">
+        <v>137</v>
+      </c>
       <c r="J28" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K28" s="1"/>
-      <c r="L28" s="1"/>
+      <c r="L28" s="1" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="D29" s="1">
-        <v>0.2</v>
+        <v>50</v>
       </c>
       <c r="E29" s="1">
         <v>0</v>
@@ -2262,25 +2317,29 @@
       <c r="F29" s="1"/>
       <c r="G29" s="1"/>
       <c r="H29" s="1"/>
-      <c r="I29" s="1"/>
+      <c r="I29" s="1" t="s">
+        <v>137</v>
+      </c>
       <c r="J29" s="1" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="K29" s="1"/>
-      <c r="L29" s="1"/>
+      <c r="L29" s="1" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="D30" s="1">
-        <v>50</v>
+        <v>1270</v>
       </c>
       <c r="E30" s="1">
         <v>0</v>
@@ -2288,49 +2347,59 @@
       <c r="F30" s="1"/>
       <c r="G30" s="1"/>
       <c r="H30" s="1"/>
-      <c r="I30" s="1"/>
+      <c r="I30" s="1" t="s">
+        <v>137</v>
+      </c>
       <c r="J30" s="1" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="K30" s="1"/>
-      <c r="L30" s="1"/>
+      <c r="L30" s="1" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>130</v>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="C31" s="1"/>
       <c r="D31" s="1">
-        <v>1270</v>
+        <v>6</v>
       </c>
       <c r="E31" s="1">
         <v>0</v>
       </c>
       <c r="F31" s="1"/>
       <c r="G31" s="1"/>
-      <c r="H31" s="1"/>
-      <c r="I31" s="1"/>
+      <c r="H31" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="I31" s="1" t="s">
+        <v>137</v>
+      </c>
       <c r="J31" s="1" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="K31" s="1"/>
-      <c r="L31" s="1"/>
+      <c r="L31" s="1" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C32" s="1"/>
+        <v>35</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>127</v>
+      </c>
       <c r="D32" s="1">
-        <v>6</v>
+        <v>1300</v>
       </c>
       <c r="E32" s="1">
         <v>0</v>
@@ -2338,51 +2407,62 @@
       <c r="F32" s="1"/>
       <c r="G32" s="1"/>
       <c r="H32" s="1"/>
-      <c r="I32" s="1"/>
+      <c r="I32" s="1" t="s">
+        <v>137</v>
+      </c>
       <c r="J32" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K32" s="1"/>
-      <c r="L32" s="1"/>
+      <c r="L32" s="1" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="D33" s="1">
-        <v>1300</v>
+        <f>1/(2.5*365)</f>
+        <v>1.095890410958904E-3</v>
       </c>
       <c r="E33" s="1">
         <v>0</v>
       </c>
       <c r="F33" s="1"/>
       <c r="G33" s="1"/>
-      <c r="H33" s="1"/>
-      <c r="I33" s="1"/>
+      <c r="H33" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="I33" s="1" t="s">
+        <v>137</v>
+      </c>
       <c r="J33" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="K33" s="1"/>
-      <c r="L33" s="1"/>
+      <c r="L33" s="1" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>37</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="D34" s="1">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="E34" s="1">
         <v>0</v>
@@ -2390,25 +2470,29 @@
       <c r="F34" s="1"/>
       <c r="G34" s="1"/>
       <c r="H34" s="1"/>
-      <c r="I34" s="1"/>
+      <c r="I34" s="1" t="s">
+        <v>137</v>
+      </c>
       <c r="J34" s="1" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="K34" s="1"/>
-      <c r="L34" s="1"/>
+      <c r="L34" s="1" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>38</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="D35" s="1">
-        <v>0.5</v>
+        <v>0.35</v>
       </c>
       <c r="E35" s="1">
         <v>0</v>
@@ -2416,25 +2500,29 @@
       <c r="F35" s="1"/>
       <c r="G35" s="1"/>
       <c r="H35" s="1"/>
-      <c r="I35" s="1"/>
+      <c r="I35" s="1" t="s">
+        <v>137</v>
+      </c>
       <c r="J35" s="1" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="K35" s="1"/>
-      <c r="L35" s="1"/>
+      <c r="L35" s="1" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>39</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="D36" s="1">
-        <v>0.35</v>
+        <v>128</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>40</v>
       </c>
       <c r="E36" s="1">
         <v>0</v>
@@ -2442,23 +2530,29 @@
       <c r="F36" s="1"/>
       <c r="G36" s="1"/>
       <c r="H36" s="1"/>
-      <c r="I36" s="1"/>
+      <c r="I36" s="1" t="s">
+        <v>137</v>
+      </c>
       <c r="J36" s="1" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="K36" s="1"/>
-      <c r="L36" s="1"/>
-    </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L36" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C37" s="1"/>
+        <v>35</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>125</v>
+      </c>
       <c r="D37" s="1">
-        <v>0</v>
+        <v>6.0100000000000001E-2</v>
       </c>
       <c r="E37" s="1">
         <v>0</v>
@@ -2466,25 +2560,29 @@
       <c r="F37" s="1"/>
       <c r="G37" s="1"/>
       <c r="H37" s="1"/>
-      <c r="I37" s="1"/>
+      <c r="I37" s="1" t="s">
+        <v>137</v>
+      </c>
       <c r="J37" s="1" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="K37" s="1"/>
-      <c r="L37" s="1"/>
-    </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L37" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>42</v>
+        <v>125</v>
+      </c>
+      <c r="D38" s="1">
+        <v>6.0100000000000001E-2</v>
       </c>
       <c r="E38" s="1">
         <v>0</v>
@@ -2492,451 +2590,463 @@
       <c r="F38" s="1"/>
       <c r="G38" s="1"/>
       <c r="H38" s="1"/>
-      <c r="I38" s="1"/>
+      <c r="I38" s="1" t="s">
+        <v>137</v>
+      </c>
       <c r="J38" s="1" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="K38" s="1"/>
-      <c r="L38" s="1"/>
-    </row>
-    <row r="39" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="L38" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B39" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B39" s="1" t="s">
-        <v>36</v>
-      </c>
       <c r="C39" s="1" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D39" s="1">
-        <v>6.0100000000000001E-2</v>
+        <v>12</v>
       </c>
       <c r="E39" s="1">
-        <v>0</v>
+        <v>2.4</v>
       </c>
       <c r="F39" s="1"/>
       <c r="G39" s="1"/>
-      <c r="H39" s="1"/>
+      <c r="H39" s="1" t="s">
+        <v>44</v>
+      </c>
       <c r="I39" s="1"/>
       <c r="J39" s="1" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="K39" s="1"/>
-      <c r="L39" s="1"/>
-    </row>
-    <row r="40" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="L39" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>44</v>
+        <v>12</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D40" s="1">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="E40" s="1">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F40" s="1"/>
       <c r="G40" s="1"/>
-      <c r="H40" s="1"/>
+      <c r="H40" s="1" t="s">
+        <v>44</v>
+      </c>
       <c r="I40" s="1"/>
       <c r="J40" s="1" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="K40" s="1"/>
-      <c r="L40" s="1"/>
-    </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L40" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="D41" s="1">
-        <v>12</v>
+        <v>0.2</v>
       </c>
       <c r="E41" s="1">
-        <v>2.4</v>
+        <v>0.04</v>
       </c>
       <c r="F41" s="1"/>
       <c r="G41" s="1"/>
       <c r="H41" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I41" s="1"/>
       <c r="J41" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K41" s="1"/>
       <c r="L41" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="D42" s="1">
-        <v>20</v>
+        <v>0.1</v>
       </c>
       <c r="E42" s="1">
-        <v>4</v>
+        <v>0.02</v>
       </c>
       <c r="F42" s="1"/>
       <c r="G42" s="1"/>
       <c r="H42" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I42" s="1"/>
       <c r="J42" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K42" s="1"/>
       <c r="L42" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="43" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>133</v>
+        <v>124</v>
       </c>
       <c r="D43" s="1">
-        <v>0.2</v>
+        <v>0.45</v>
       </c>
       <c r="E43" s="1">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
       <c r="F43" s="1"/>
       <c r="G43" s="1"/>
       <c r="H43" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="I43" s="1"/>
       <c r="J43" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K43" s="1"/>
       <c r="L43" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="44" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="D44" s="1">
-        <v>0.1</v>
+        <v>0.22</v>
       </c>
       <c r="E44" s="1">
-        <v>0.02</v>
+        <v>3.5000000000000003E-2</v>
       </c>
       <c r="F44" s="1"/>
       <c r="G44" s="1"/>
       <c r="H44" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="I44" s="1"/>
       <c r="J44" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K44" s="1"/>
       <c r="L44" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="D45" s="1">
-        <v>0.45</v>
+        <v>0.21</v>
       </c>
       <c r="E45" s="1">
-        <v>0.05</v>
+        <f>0.02</f>
+        <v>0.02</v>
       </c>
       <c r="F45" s="1"/>
       <c r="G45" s="1"/>
       <c r="H45" s="1" t="s">
-        <v>48</v>
+        <v>76</v>
       </c>
       <c r="I45" s="1"/>
       <c r="J45" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K45" s="1"/>
       <c r="L45" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="D46" s="1">
-        <v>0.22</v>
+        <v>212</v>
       </c>
       <c r="E46" s="1">
-        <v>3.5000000000000003E-2</v>
-      </c>
-      <c r="F46" s="1"/>
-      <c r="G46" s="1"/>
+        <v>157</v>
+      </c>
+      <c r="F46" s="1">
+        <v>77</v>
+      </c>
+      <c r="G46" s="1">
+        <v>290</v>
+      </c>
       <c r="H46" s="1" t="s">
-        <v>48</v>
+        <v>75</v>
       </c>
       <c r="I46" s="1"/>
       <c r="J46" s="1" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="K46" s="1"/>
       <c r="L46" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="D47" s="1">
-        <v>0.21</v>
+        <v>1428</v>
       </c>
       <c r="E47" s="1">
-        <f>0.02</f>
-        <v>0.02</v>
-      </c>
-      <c r="F47" s="1"/>
-      <c r="G47" s="1"/>
+        <v>114</v>
+      </c>
+      <c r="F47" s="1">
+        <v>1335</v>
+      </c>
+      <c r="G47" s="1">
+        <v>1481</v>
+      </c>
       <c r="H47" s="1" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="I47" s="1"/>
       <c r="J47" s="1" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="K47" s="1"/>
       <c r="L47" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C48" s="1" t="s">
-        <v>130</v>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="C48" s="1"/>
       <c r="D48" s="1">
-        <v>212</v>
+        <v>6</v>
       </c>
       <c r="E48" s="1">
-        <v>157</v>
-      </c>
-      <c r="F48" s="1">
-        <v>77</v>
-      </c>
-      <c r="G48" s="1">
-        <v>290</v>
-      </c>
-      <c r="H48" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="I48" s="1"/>
+        <v>0.06</v>
+      </c>
+      <c r="F48" s="1"/>
+      <c r="G48" s="1"/>
+      <c r="H48" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="I48" s="3"/>
       <c r="J48" s="1" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="K48" s="1"/>
       <c r="L48" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="D49" s="1">
-        <v>1428</v>
+        <v>880</v>
       </c>
       <c r="E49" s="1">
-        <v>114</v>
+        <v>70</v>
       </c>
       <c r="F49" s="1">
-        <v>1335</v>
+        <v>810</v>
       </c>
       <c r="G49" s="1">
-        <v>1481</v>
-      </c>
-      <c r="H49" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="I49" s="1"/>
+        <v>960</v>
+      </c>
+      <c r="H49" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="I49" s="3"/>
       <c r="J49" s="1" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="K49" s="1"/>
       <c r="L49" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C50" s="1"/>
+        <v>43</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>128</v>
+      </c>
       <c r="D50" s="1">
-        <v>6</v>
+        <v>5.7999999999999996E-3</v>
       </c>
       <c r="E50" s="1">
-        <v>0.06</v>
+        <v>3.3999999999999998E-3</v>
       </c>
       <c r="F50" s="1"/>
       <c r="G50" s="1"/>
-      <c r="H50" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="I50" s="3"/>
+      <c r="H50" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="I50" s="1"/>
       <c r="J50" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="K50" s="1"/>
       <c r="L50" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A51" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="D51" s="1">
+        <v>0.50930200000000003</v>
+      </c>
+      <c r="E51" s="1">
+        <v>2.9389999999999999E-2</v>
+      </c>
+      <c r="F51" s="1"/>
+      <c r="G51" s="1"/>
+      <c r="H51" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="I51" s="1"/>
+      <c r="J51" s="1" t="s">
         <v>71</v>
-      </c>
-    </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A51" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B51" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C51" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="D51" s="1">
-        <v>880</v>
-      </c>
-      <c r="E51" s="1">
-        <v>70</v>
-      </c>
-      <c r="F51" s="1">
-        <v>810</v>
-      </c>
-      <c r="G51" s="1">
-        <v>960</v>
-      </c>
-      <c r="H51" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="I51" s="3"/>
-      <c r="J51" s="1" t="s">
-        <v>73</v>
       </c>
       <c r="K51" s="1"/>
       <c r="L51" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="52" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="D52" s="1">
-        <v>5.7999999999999996E-3</v>
+        <v>0.35</v>
       </c>
       <c r="E52" s="1">
-        <v>3.3999999999999998E-3</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="F52" s="1"/>
       <c r="G52" s="1"/>
       <c r="H52" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="I52" s="1"/>
       <c r="J52" s="1" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="K52" s="1"/>
       <c r="L52" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="53" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="D53" s="1">
-        <v>0.50930200000000003</v>
+        <v>128</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>48</v>
       </c>
       <c r="E53" s="1">
-        <v>2.9389999999999999E-2</v>
+        <v>0</v>
       </c>
       <c r="F53" s="1"/>
       <c r="G53" s="1"/>
@@ -2945,206 +3055,210 @@
       </c>
       <c r="I53" s="1"/>
       <c r="J53" s="1" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="K53" s="1"/>
       <c r="L53" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="54" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="D54" s="1">
-        <v>0.35</v>
+        <v>6.0100000000000001E-2</v>
       </c>
       <c r="E54" s="1">
-        <v>7.0000000000000007E-2</v>
+        <v>1.2E-2</v>
       </c>
       <c r="F54" s="1"/>
       <c r="G54" s="1"/>
       <c r="H54" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I54" s="1"/>
       <c r="J54" s="1" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="K54" s="1"/>
       <c r="L54" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C55" s="1"/>
+        <v>43</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>125</v>
+      </c>
       <c r="D55" s="1">
-        <v>0</v>
+        <v>6.0100000000000001E-2</v>
       </c>
       <c r="E55" s="1">
-        <v>0</v>
+        <v>1.2E-2</v>
       </c>
       <c r="F55" s="1"/>
       <c r="G55" s="1"/>
-      <c r="H55" s="1"/>
-      <c r="I55" s="1"/>
+      <c r="H55" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="I55" s="1" t="s">
+        <v>110</v>
+      </c>
       <c r="J55" s="1" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="K55" s="1"/>
       <c r="L55" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="56" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="D56" s="2" t="s">
-        <v>50</v>
+        <v>123</v>
+      </c>
+      <c r="D56" s="1">
+        <v>12</v>
       </c>
       <c r="E56" s="1">
-        <v>0</v>
+        <v>2.4</v>
       </c>
       <c r="F56" s="1"/>
       <c r="G56" s="1"/>
       <c r="H56" s="1" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="I56" s="1"/>
       <c r="J56" s="1" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="K56" s="1"/>
       <c r="L56" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="57" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D57" s="1">
-        <v>6.0100000000000001E-2</v>
+        <v>20</v>
       </c>
       <c r="E57" s="1">
-        <v>1.2E-2</v>
+        <v>4</v>
       </c>
       <c r="F57" s="1"/>
       <c r="G57" s="1"/>
       <c r="H57" s="1" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="I57" s="1"/>
       <c r="J57" s="1" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="K57" s="1"/>
       <c r="L57" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="58" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
-        <v>44</v>
+        <v>13</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="C58" s="1" t="s">
         <v>129</v>
       </c>
       <c r="D58" s="1">
-        <v>6.0100000000000001E-2</v>
+        <v>0.2</v>
       </c>
       <c r="E58" s="1">
-        <v>1.2E-2</v>
+        <v>0.04</v>
       </c>
       <c r="F58" s="1"/>
       <c r="G58" s="1"/>
       <c r="H58" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="I58" s="1" t="s">
-        <v>114</v>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="I58" s="1"/>
       <c r="J58" s="1" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="K58" s="1"/>
       <c r="L58" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="D59" s="1">
-        <v>12</v>
+        <v>0.1</v>
       </c>
       <c r="E59" s="1">
-        <v>2.4</v>
+        <v>0.02</v>
       </c>
       <c r="F59" s="1"/>
       <c r="G59" s="1"/>
       <c r="H59" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I59" s="1"/>
       <c r="J59" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K59" s="1"/>
       <c r="L59" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="60" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="D60" s="1">
-        <v>20</v>
+        <v>0.45</v>
       </c>
       <c r="E60" s="1">
-        <v>4</v>
+        <v>0.05</v>
       </c>
       <c r="F60" s="1"/>
       <c r="G60" s="1"/>
@@ -3153,309 +3267,309 @@
       </c>
       <c r="I60" s="1"/>
       <c r="J60" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K60" s="1"/>
       <c r="L60" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="61" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="D61" s="1">
-        <v>0.2</v>
+        <v>0.22</v>
       </c>
       <c r="E61" s="1">
-        <v>0.04</v>
+        <v>3.5000000000000003E-2</v>
       </c>
       <c r="F61" s="1"/>
       <c r="G61" s="1"/>
       <c r="H61" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="I61" s="1"/>
       <c r="J61" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K61" s="1"/>
       <c r="L61" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="62" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="62" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="D62" s="1">
-        <v>0.1</v>
+        <v>0.21</v>
       </c>
       <c r="E62" s="1">
+        <f>0.02</f>
         <v>0.02</v>
       </c>
       <c r="F62" s="1"/>
       <c r="G62" s="1"/>
       <c r="H62" s="1" t="s">
-        <v>47</v>
+        <v>76</v>
       </c>
       <c r="I62" s="1"/>
       <c r="J62" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K62" s="1"/>
       <c r="L62" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="63" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="D63" s="1">
-        <v>0.45</v>
+        <v>212</v>
       </c>
       <c r="E63" s="1">
-        <v>0.05</v>
-      </c>
-      <c r="F63" s="1"/>
-      <c r="G63" s="1"/>
+        <v>157</v>
+      </c>
+      <c r="F63" s="1">
+        <v>77</v>
+      </c>
+      <c r="G63" s="1">
+        <v>290</v>
+      </c>
       <c r="H63" s="1" t="s">
-        <v>48</v>
+        <v>75</v>
       </c>
       <c r="I63" s="1"/>
       <c r="J63" s="1" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="K63" s="1"/>
       <c r="L63" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="D64" s="1">
-        <v>0.22</v>
+        <v>1428</v>
       </c>
       <c r="E64" s="1">
-        <v>3.5000000000000003E-2</v>
-      </c>
-      <c r="F64" s="1"/>
-      <c r="G64" s="1"/>
+        <v>114</v>
+      </c>
+      <c r="F64" s="1">
+        <v>1335</v>
+      </c>
+      <c r="G64" s="1">
+        <v>1481</v>
+      </c>
       <c r="H64" s="1" t="s">
-        <v>48</v>
+        <v>75</v>
       </c>
       <c r="I64" s="1"/>
       <c r="J64" s="1" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="K64" s="1"/>
       <c r="L64" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="65" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="C65" s="1" t="s">
-        <v>129</v>
-      </c>
+        <v>51</v>
+      </c>
+      <c r="C65" s="1"/>
       <c r="D65" s="1">
-        <v>0.21</v>
+        <v>6</v>
       </c>
       <c r="E65" s="1">
-        <f>0.02</f>
-        <v>0.02</v>
+        <v>0.06</v>
       </c>
       <c r="F65" s="1"/>
       <c r="G65" s="1"/>
-      <c r="H65" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="I65" s="1"/>
+      <c r="H65" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="I65" s="3"/>
       <c r="J65" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K65" s="1"/>
       <c r="L65" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="66" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="D66" s="1">
-        <v>212</v>
+        <v>880</v>
       </c>
       <c r="E66" s="1">
-        <v>157</v>
+        <v>70</v>
       </c>
       <c r="F66" s="1">
-        <v>77</v>
+        <v>810</v>
       </c>
       <c r="G66" s="1">
-        <v>290</v>
-      </c>
-      <c r="H66" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="I66" s="1"/>
+        <v>960</v>
+      </c>
+      <c r="H66" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="I66" s="3"/>
       <c r="J66" s="1" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="K66" s="1"/>
       <c r="L66" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="67" spans="1:12" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="67" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
-        <v>19</v>
+        <v>36</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D67" s="1">
-        <v>1428</v>
+        <v>5.7999999999999996E-3</v>
       </c>
       <c r="E67" s="1">
-        <v>114</v>
-      </c>
-      <c r="F67" s="1">
-        <v>1335</v>
-      </c>
-      <c r="G67" s="1">
-        <v>1481</v>
-      </c>
+        <v>3.3999999999999998E-3</v>
+      </c>
+      <c r="F67" s="1"/>
+      <c r="G67" s="1"/>
       <c r="H67" s="1" t="s">
-        <v>79</v>
+        <v>47</v>
       </c>
       <c r="I67" s="1"/>
       <c r="J67" s="1" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="K67" s="1"/>
       <c r="L67" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="68" spans="1:12" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="68" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="C68" s="1"/>
+        <v>51</v>
+      </c>
+      <c r="C68" s="1" t="s">
+        <v>125</v>
+      </c>
       <c r="D68" s="1">
-        <v>6</v>
+        <v>0.50930200000000003</v>
       </c>
       <c r="E68" s="1">
-        <v>0.06</v>
+        <v>2.9389999999999999E-2</v>
       </c>
       <c r="F68" s="1"/>
       <c r="G68" s="1"/>
-      <c r="H68" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="I68" s="3"/>
+      <c r="H68" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="I68" s="1"/>
       <c r="J68" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="K68" s="1"/>
       <c r="L68" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="69" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A69" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C69" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="D69" s="1">
+        <v>0.35</v>
+      </c>
+      <c r="E69" s="1">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="F69" s="1"/>
+      <c r="G69" s="1"/>
+      <c r="H69" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="I69" s="1"/>
+      <c r="J69" s="1" t="s">
         <v>71</v>
-      </c>
-    </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A69" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B69" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="C69" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="D69" s="1">
-        <v>880</v>
-      </c>
-      <c r="E69" s="1">
-        <v>70</v>
-      </c>
-      <c r="F69" s="1">
-        <v>810</v>
-      </c>
-      <c r="G69" s="1">
-        <v>960</v>
-      </c>
-      <c r="H69" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="I69" s="3"/>
-      <c r="J69" s="1" t="s">
-        <v>73</v>
       </c>
       <c r="K69" s="1"/>
       <c r="L69" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="70" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="D70" s="1">
-        <v>5.7999999999999996E-3</v>
+        <v>128</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>48</v>
       </c>
       <c r="E70" s="1">
-        <v>3.3999999999999998E-3</v>
+        <v>0</v>
       </c>
       <c r="F70" s="1"/>
       <c r="G70" s="1"/>
@@ -3464,925 +3578,756 @@
       </c>
       <c r="I70" s="1"/>
       <c r="J70" s="1" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="K70" s="1"/>
       <c r="L70" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="71" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="D71" s="1">
-        <v>0.50930200000000003</v>
+        <v>6.0100000000000001E-2</v>
       </c>
       <c r="E71" s="1">
-        <v>2.9389999999999999E-2</v>
+        <v>1.2E-2</v>
       </c>
       <c r="F71" s="1"/>
       <c r="G71" s="1"/>
-      <c r="H71" s="1" t="s">
-        <v>49</v>
-      </c>
+      <c r="H71" s="1"/>
       <c r="I71" s="1"/>
       <c r="J71" s="1" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="K71" s="1"/>
       <c r="L71" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="72" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="D72" s="1">
-        <v>0.35</v>
+        <v>6.0100000000000001E-2</v>
       </c>
       <c r="E72" s="1">
-        <v>7.0000000000000007E-2</v>
+        <v>1.2E-2</v>
       </c>
       <c r="F72" s="1"/>
       <c r="G72" s="1"/>
       <c r="H72" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="I72" s="1"/>
+        <v>109</v>
+      </c>
+      <c r="I72" s="1" t="s">
+        <v>110</v>
+      </c>
       <c r="J72" s="1" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="K72" s="1"/>
       <c r="L72" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="73" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="C73" s="1"/>
+        <v>51</v>
+      </c>
+      <c r="C73" s="1" t="s">
+        <v>128</v>
+      </c>
       <c r="D73" s="1">
-        <v>0</v>
+        <v>5.1000000000000004E-3</v>
       </c>
       <c r="E73" s="1">
-        <v>0</v>
+        <v>1E-3</v>
       </c>
       <c r="F73" s="1"/>
       <c r="G73" s="1"/>
-      <c r="H73" s="1"/>
+      <c r="H73" s="1" t="s">
+        <v>47</v>
+      </c>
       <c r="I73" s="1"/>
       <c r="J73" s="1" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="K73" s="1"/>
       <c r="L73" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="74" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="D74" s="2" t="s">
-        <v>50</v>
+        <v>125</v>
+      </c>
+      <c r="D74" s="1">
+        <v>0.6</v>
       </c>
       <c r="E74" s="1">
-        <v>0</v>
+        <v>0.12</v>
       </c>
       <c r="F74" s="1"/>
       <c r="G74" s="1"/>
       <c r="H74" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="I74" s="1"/>
       <c r="J74" s="1" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="K74" s="1"/>
       <c r="L74" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="75" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="D75" s="1">
-        <v>6.0100000000000001E-2</v>
+        <v>0.35</v>
       </c>
       <c r="E75" s="1">
-        <v>1.2E-2</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="F75" s="1"/>
       <c r="G75" s="1"/>
-      <c r="H75" s="1"/>
+      <c r="H75" s="1" t="s">
+        <v>47</v>
+      </c>
       <c r="I75" s="1"/>
       <c r="J75" s="1" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="K75" s="1"/>
       <c r="L75" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="76" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="76" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D76" s="1">
-        <v>6.0100000000000001E-2</v>
+        <v>1.6799999999999999E-2</v>
       </c>
       <c r="E76" s="1">
-        <v>1.2E-2</v>
+        <v>3.3999999999999998E-3</v>
       </c>
       <c r="F76" s="1"/>
       <c r="G76" s="1"/>
       <c r="H76" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="I76" s="1" t="s">
-        <v>114</v>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="I76" s="1"/>
       <c r="J76" s="1" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="K76" s="1"/>
       <c r="L76" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="77" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="77" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
-        <v>54</v>
+        <v>11</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="D77" s="1">
-        <v>5.1000000000000004E-3</v>
+        <v>10</v>
       </c>
       <c r="E77" s="1">
-        <v>1E-3</v>
+        <f>Table1[[#This Row],[Value]]*2</f>
+        <v>20</v>
       </c>
       <c r="F77" s="1"/>
       <c r="G77" s="1"/>
       <c r="H77" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="I77" s="1"/>
+        <v>83</v>
+      </c>
+      <c r="I77" s="1" t="s">
+        <v>84</v>
+      </c>
       <c r="J77" s="1" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="K77" s="1"/>
       <c r="L77" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="78" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="78" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
-        <v>55</v>
+        <v>12</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D78" s="1">
-        <v>0.6</v>
+        <v>26</v>
       </c>
       <c r="E78" s="1">
-        <v>0.12</v>
+        <f>Table1[[#This Row],[Value]]*2</f>
+        <v>52</v>
       </c>
       <c r="F78" s="1"/>
       <c r="G78" s="1"/>
       <c r="H78" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="I78" s="1"/>
+        <v>83</v>
+      </c>
+      <c r="I78" s="1" t="s">
+        <v>84</v>
+      </c>
       <c r="J78" s="1" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="K78" s="1"/>
       <c r="L78" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="79" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="79" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
-        <v>56</v>
+        <v>13</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="C79" s="1" t="s">
         <v>129</v>
       </c>
       <c r="D79" s="1">
-        <v>0.35</v>
+        <v>0.3</v>
       </c>
       <c r="E79" s="1">
-        <v>7.0000000000000007E-2</v>
+        <f>Table1[[#This Row],[Value]]*2</f>
+        <v>0.6</v>
       </c>
       <c r="F79" s="1"/>
       <c r="G79" s="1"/>
       <c r="H79" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="I79" s="1"/>
+        <v>83</v>
+      </c>
+      <c r="I79" s="1" t="s">
+        <v>84</v>
+      </c>
       <c r="J79" s="1" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="K79" s="1"/>
       <c r="L79" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="80" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B80" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B80" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="C80" s="1"/>
+      <c r="C80" s="1" t="s">
+        <v>129</v>
+      </c>
       <c r="D80" s="1">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="E80" s="1">
-        <v>0</v>
+        <f>Table1[[#This Row],[Value]]*2</f>
+        <v>0.3</v>
       </c>
       <c r="F80" s="1"/>
       <c r="G80" s="1"/>
-      <c r="H80" s="1"/>
-      <c r="I80" s="1"/>
+      <c r="H80" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="I80" s="1" t="s">
+        <v>84</v>
+      </c>
       <c r="J80" s="1" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="K80" s="1"/>
       <c r="L80" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="81" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="81" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
-        <v>58</v>
+        <v>15</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="D81" s="1">
-        <v>1.6799999999999999E-2</v>
+        <v>70</v>
       </c>
       <c r="E81" s="1">
-        <v>3.3999999999999998E-3</v>
+        <f>Table1[[#This Row],[Value]]*2</f>
+        <v>140</v>
       </c>
       <c r="F81" s="1"/>
       <c r="G81" s="1"/>
       <c r="H81" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="I81" s="1"/>
+        <v>83</v>
+      </c>
+      <c r="I81" s="1" t="s">
+        <v>84</v>
+      </c>
       <c r="J81" s="1" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="K81" s="1"/>
       <c r="L81" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="82" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="D82" s="1">
-        <v>10</v>
+        <v>0.4</v>
       </c>
       <c r="E82" s="1">
         <f>Table1[[#This Row],[Value]]*2</f>
-        <v>20</v>
+        <v>0.8</v>
       </c>
       <c r="F82" s="1"/>
       <c r="G82" s="1"/>
       <c r="H82" s="1" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="I82" s="1" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="J82" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K82" s="1"/>
       <c r="L82" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="83" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="D83" s="1">
-        <v>26</v>
+        <v>0.2</v>
       </c>
       <c r="E83" s="1">
         <f>Table1[[#This Row],[Value]]*2</f>
-        <v>52</v>
+        <v>0.4</v>
       </c>
       <c r="F83" s="1"/>
       <c r="G83" s="1"/>
       <c r="H83" s="1" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="I83" s="1" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="J83" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K83" s="1"/>
       <c r="L83" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="84" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="D84" s="1">
-        <v>0.3</v>
+        <v>433</v>
       </c>
       <c r="E84" s="1">
         <f>Table1[[#This Row],[Value]]*2</f>
-        <v>0.6</v>
+        <v>866</v>
       </c>
       <c r="F84" s="1"/>
       <c r="G84" s="1"/>
       <c r="H84" s="1" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="I84" s="1" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="J84" s="1" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="K84" s="1"/>
       <c r="L84" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="85" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="D85" s="1">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="E85" s="1">
         <f>Table1[[#This Row],[Value]]*2</f>
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="F85" s="1"/>
       <c r="G85" s="1"/>
       <c r="H85" s="1" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="I85" s="1" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="J85" s="1" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="K85" s="1"/>
       <c r="L85" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="86" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="C86" s="1" t="s">
-        <v>128</v>
-      </c>
+        <v>57</v>
+      </c>
+      <c r="C86" s="1"/>
       <c r="D86" s="1">
-        <v>70</v>
+        <v>6</v>
       </c>
       <c r="E86" s="1">
         <f>Table1[[#This Row],[Value]]*2</f>
-        <v>140</v>
+        <v>12</v>
       </c>
       <c r="F86" s="1"/>
       <c r="G86" s="1"/>
       <c r="H86" s="1" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="I86" s="1" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="J86" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K86" s="1"/>
       <c r="L86" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="87" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D87" s="1">
-        <v>0.4</v>
+        <v>1300</v>
       </c>
       <c r="E87" s="1">
         <f>Table1[[#This Row],[Value]]*2</f>
-        <v>0.8</v>
+        <v>2600</v>
       </c>
       <c r="F87" s="1"/>
       <c r="G87" s="1"/>
       <c r="H87" s="1" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="I87" s="1" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="J87" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K87" s="1"/>
       <c r="L87" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="88" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
-        <v>17</v>
+        <v>58</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D88" s="1">
-        <v>0.2</v>
+        <v>0.02</v>
       </c>
       <c r="E88" s="1">
         <f>Table1[[#This Row],[Value]]*2</f>
-        <v>0.4</v>
+        <v>0.04</v>
       </c>
       <c r="F88" s="1"/>
       <c r="G88" s="1"/>
       <c r="H88" s="1" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="I88" s="1" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="J88" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="K88" s="1"/>
       <c r="L88" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="89" spans="1:12" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="89" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
-        <v>18</v>
+        <v>59</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="D89" s="1">
-        <v>433</v>
+        <f>1/36</f>
+        <v>2.7777777777777776E-2</v>
       </c>
       <c r="E89" s="1">
         <f>Table1[[#This Row],[Value]]*2</f>
-        <v>866</v>
+        <v>5.5555555555555552E-2</v>
       </c>
       <c r="F89" s="1"/>
       <c r="G89" s="1"/>
-      <c r="H89" s="1" t="s">
-        <v>87</v>
+      <c r="H89" s="4" t="s">
+        <v>81</v>
       </c>
       <c r="I89" s="1" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="J89" s="1" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="K89" s="1"/>
       <c r="L89" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="90" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
-        <v>19</v>
+        <v>60</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="D90" s="1">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="E90" s="1">
         <f>Table1[[#This Row],[Value]]*2</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F90" s="1"/>
       <c r="G90" s="1"/>
       <c r="H90" s="1" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="I90" s="1" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="J90" s="1" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="K90" s="1"/>
       <c r="L90" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="91" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C91" s="1"/>
       <c r="D91" s="1">
-        <v>6</v>
+        <v>0.37</v>
       </c>
       <c r="E91" s="1">
         <f>Table1[[#This Row],[Value]]*2</f>
-        <v>12</v>
+        <v>0.74</v>
       </c>
       <c r="F91" s="1"/>
       <c r="G91" s="1"/>
       <c r="H91" s="1" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="I91" s="1" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="J91" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="K91" s="1"/>
       <c r="L91" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="92" spans="1:12" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="92" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
-        <v>21</v>
+        <v>62</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="D92" s="1">
-        <v>1300</v>
+        <v>130</v>
+      </c>
+      <c r="D92" s="5">
+        <v>2.7399999999999999E-5</v>
       </c>
       <c r="E92" s="1">
         <f>Table1[[#This Row],[Value]]*2</f>
-        <v>2600</v>
+        <v>5.4799999999999997E-5</v>
       </c>
       <c r="F92" s="1"/>
       <c r="G92" s="1"/>
       <c r="H92" s="1" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="I92" s="1" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="J92" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="K92" s="1"/>
       <c r="L92" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="93" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="D93" s="1">
-        <v>0.02</v>
+        <v>128</v>
+      </c>
+      <c r="D93" s="5">
+        <v>1.2999999999999999E-5</v>
       </c>
       <c r="E93" s="1">
         <f>Table1[[#This Row],[Value]]*2</f>
-        <v>0.04</v>
+        <v>2.5999999999999998E-5</v>
       </c>
       <c r="F93" s="1"/>
       <c r="G93" s="1"/>
       <c r="H93" s="1" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="I93" s="1" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="J93" s="1" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="K93" s="1"/>
       <c r="L93" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="94" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A94" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="B94" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="C94" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="D94" s="1">
-        <f>1/36</f>
-        <v>2.7777777777777776E-2</v>
-      </c>
-      <c r="E94" s="1">
-        <f>Table1[[#This Row],[Value]]*2</f>
-        <v>5.5555555555555552E-2</v>
-      </c>
-      <c r="F94" s="1"/>
-      <c r="G94" s="1"/>
-      <c r="H94" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="I94" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="J94" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="K94" s="1"/>
-      <c r="L94" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="95" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A95" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="B95" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="C95" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="D95" s="1">
-        <v>0.5</v>
-      </c>
-      <c r="E95" s="1">
-        <f>Table1[[#This Row],[Value]]*2</f>
-        <v>1</v>
-      </c>
-      <c r="F95" s="1"/>
-      <c r="G95" s="1"/>
-      <c r="H95" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="I95" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="J95" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="K95" s="1"/>
-      <c r="L95" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="96" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A96" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="B96" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="C96" s="1"/>
-      <c r="D96" s="1">
-        <v>0.37</v>
-      </c>
-      <c r="E96" s="1">
-        <f>Table1[[#This Row],[Value]]*2</f>
-        <v>0.74</v>
-      </c>
-      <c r="F96" s="1"/>
-      <c r="G96" s="1"/>
-      <c r="H96" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="I96" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="J96" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="K96" s="1"/>
-      <c r="L96" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="97" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A97" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="B97" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="C97" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="D97" s="1">
-        <v>0</v>
-      </c>
-      <c r="E97" s="1">
-        <v>0</v>
-      </c>
-      <c r="F97" s="1"/>
-      <c r="G97" s="1"/>
-      <c r="H97" s="1"/>
-      <c r="I97" s="1"/>
-      <c r="J97" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="K97" s="1"/>
-      <c r="L97" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="98" spans="1:12" ht="30" x14ac:dyDescent="0.25">
-      <c r="A98" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="B98" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="C98" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="D98" s="5">
-        <v>2.7399999999999999E-5</v>
-      </c>
-      <c r="E98" s="1">
-        <f>Table1[[#This Row],[Value]]*2</f>
-        <v>5.4799999999999997E-5</v>
-      </c>
-      <c r="F98" s="1"/>
-      <c r="G98" s="1"/>
-      <c r="H98" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="I98" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="J98" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="K98" s="1"/>
-      <c r="L98" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="99" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A99" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="B99" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="C99" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="D99" s="5">
-        <v>1.2999999999999999E-5</v>
-      </c>
-      <c r="E99" s="1">
-        <f>Table1[[#This Row],[Value]]*2</f>
-        <v>2.5999999999999998E-5</v>
-      </c>
-      <c r="F99" s="1"/>
-      <c r="G99" s="1"/>
-      <c r="H99" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="I99" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="J99" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="K99" s="1"/>
-      <c r="L99" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
@@ -4401,62 +4346,72 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="D1" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="E1" t="s">
         <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D2">
         <f xml:space="preserve"> 172*0.3*0.25*0.5</f>
         <v>6.45</v>
       </c>
       <c r="E2" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="F2" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C3" t="s">
         <v>9</v>
       </c>
+      <c r="D3">
+        <f xml:space="preserve"> 300*0.05*0.25*0.5</f>
+        <v>1.875</v>
+      </c>
+      <c r="E3" t="s">
+        <v>136</v>
+      </c>
+      <c r="F3" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C4" t="s">
         <v>9</v>
@@ -4465,18 +4420,18 @@
         <v>0.1</v>
       </c>
       <c r="E4" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="F4" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B5" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C5" t="s">
         <v>9</v>
@@ -4485,18 +4440,18 @@
         <v>0.1</v>
       </c>
       <c r="E5" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="F5" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B6" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C6" t="s">
         <v>10</v>
@@ -4505,18 +4460,18 @@
         <v>0.1</v>
       </c>
       <c r="E6" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="F6" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B7" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C7" t="s">
         <v>8</v>
@@ -4525,310 +4480,310 @@
         <v>0.1</v>
       </c>
       <c r="E7" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="F7" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B8" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C8" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="D8">
         <v>200</v>
       </c>
       <c r="E8" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="F8" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B9" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C9" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="D9">
         <v>200</v>
       </c>
       <c r="E9" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="F9" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B10" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C10" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="D10">
         <v>750</v>
       </c>
       <c r="E10" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="F10" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B11" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C11" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="D11">
         <v>6750</v>
       </c>
       <c r="E11" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="F11" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B12" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C12" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D12">
         <v>2500</v>
       </c>
       <c r="E12" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="F12" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B13" t="s">
+        <v>89</v>
+      </c>
+      <c r="C13" t="s">
         <v>93</v>
-      </c>
-      <c r="C13" t="s">
-        <v>97</v>
       </c>
       <c r="D13">
         <v>200</v>
       </c>
       <c r="E13" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="F13" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B14" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C14" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="D14">
         <v>1000</v>
       </c>
       <c r="E14" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="F14" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B15" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C15" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="D15">
         <v>2000</v>
       </c>
       <c r="E15" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="F15" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B16" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C16" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="D16">
         <v>10</v>
       </c>
       <c r="E16" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="F16" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B17" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C17" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="D17">
         <v>0.1</v>
       </c>
       <c r="E17" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="F17" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B18" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C18" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="D18">
         <v>400</v>
       </c>
       <c r="E18" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="F18" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B19" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C19" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="D19">
         <v>10</v>
       </c>
       <c r="E19" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="F19" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B20" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C20" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="D20">
         <v>1000</v>
       </c>
       <c r="E20" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="F20" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B21" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C21" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D21">
         <v>3000</v>
       </c>
       <c r="E21" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="F21" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B22" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C22" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="D22">
         <v>40</v>
       </c>
       <c r="E22" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="F22" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -4847,13 +4802,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -4861,7 +4816,7 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C2">
         <v>1</v>
@@ -4872,7 +4827,7 @@
         <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -4883,7 +4838,7 @@
         <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C4">
         <v>1</v>
@@ -4894,7 +4849,7 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -4905,7 +4860,7 @@
         <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -4916,7 +4871,7 @@
         <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -4927,7 +4882,7 @@
         <v>5</v>
       </c>
       <c r="B8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -4938,7 +4893,7 @@
         <v>6</v>
       </c>
       <c r="B9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C9">
         <v>1</v>
@@ -4949,7 +4904,7 @@
         <v>7</v>
       </c>
       <c r="B10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -4960,7 +4915,7 @@
         <v>8</v>
       </c>
       <c r="B11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -4971,7 +4926,7 @@
         <v>9</v>
       </c>
       <c r="B12" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C12">
         <v>1</v>
@@ -4982,7 +4937,7 @@
         <v>10</v>
       </c>
       <c r="B13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C13">
         <v>0</v>
@@ -4993,7 +4948,7 @@
         <v>5</v>
       </c>
       <c r="B14" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C14">
         <v>1</v>
@@ -5004,7 +4959,7 @@
         <v>6</v>
       </c>
       <c r="B15" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C15">
         <v>1</v>
@@ -5015,7 +4970,7 @@
         <v>7</v>
       </c>
       <c r="B16" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C16">
         <v>0</v>
@@ -5026,7 +4981,7 @@
         <v>8</v>
       </c>
       <c r="B17" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C17">
         <v>0</v>
@@ -5037,7 +4992,7 @@
         <v>9</v>
       </c>
       <c r="B18" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C18">
         <v>1</v>
@@ -5048,7 +5003,7 @@
         <v>10</v>
       </c>
       <c r="B19" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C19">
         <v>0</v>
@@ -5059,7 +5014,7 @@
         <v>5</v>
       </c>
       <c r="B20" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C20">
         <v>1</v>
@@ -5070,7 +5025,7 @@
         <v>6</v>
       </c>
       <c r="B21" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C21">
         <v>1</v>
@@ -5081,7 +5036,7 @@
         <v>7</v>
       </c>
       <c r="B22" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C22">
         <v>0</v>
@@ -5092,7 +5047,7 @@
         <v>8</v>
       </c>
       <c r="B23" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C23">
         <v>0</v>
@@ -5103,7 +5058,7 @@
         <v>9</v>
       </c>
       <c r="B24" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C24">
         <v>1</v>
@@ -5114,7 +5069,7 @@
         <v>10</v>
       </c>
       <c r="B25" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C25">
         <v>1</v>
@@ -5125,7 +5080,7 @@
         <v>5</v>
       </c>
       <c r="B26" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C26">
         <v>0</v>
@@ -5136,7 +5091,7 @@
         <v>6</v>
       </c>
       <c r="B27" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C27">
         <v>1</v>
@@ -5147,7 +5102,7 @@
         <v>7</v>
       </c>
       <c r="B28" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C28">
         <v>0</v>
@@ -5158,7 +5113,7 @@
         <v>8</v>
       </c>
       <c r="B29" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C29">
         <v>1</v>
@@ -5169,7 +5124,7 @@
         <v>9</v>
       </c>
       <c r="B30" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C30">
         <v>0</v>
@@ -5180,7 +5135,7 @@
         <v>10</v>
       </c>
       <c r="B31" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C31">
         <v>0</v>

</xml_diff>

<commit_message>
Added better effect size fitting and then proceeded to fit and spin-up.
</commit_message>
<xml_diff>
--- a/Data/scenarios.xlsx
+++ b/Data/scenarios.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rober\Documents\GitHub Repos\merging_SFW_decomposition_models\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A252B0D-9B1D-43E6-9CA2-1EA286133C0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8444547-9DD2-49C3-882C-4D20E7A024AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7C97690C-9E7B-4D0E-86C0-16835BCB4BB0}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{7C97690C-9E7B-4D0E-86C0-16835BCB4BB0}"/>
   </bookViews>
   <sheets>
     <sheet name="scenarios" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="753" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="756" uniqueCount="140">
   <si>
     <t>Parameter</t>
   </si>
@@ -187,9 +187,6 @@
     <t>Adapted from calculatation conduct on empirical data provided by Seastedt et al. 1983 and Seastedt 1984</t>
   </si>
   <si>
-    <t>Calculated based on emperical data provided by Seastedt et al. 1983</t>
-  </si>
-  <si>
     <t>MitePredator</t>
   </si>
   <si>
@@ -449,6 +446,15 @@
   </si>
   <si>
     <t>Need to refine</t>
+  </si>
+  <si>
+    <t>Fitted using the fitting function to achieve 56% increase in aggregate carbon indicated by Ross et al. 2024</t>
+  </si>
+  <si>
+    <t>Fitted to achieve a 33% reduction in litter carbon indicated by de Smelt et al., 2018</t>
+  </si>
+  <si>
+    <t>Calculated based on emperical data provided by Seastedt et al. 1983, but then changed from 0.0601 to 10.2047 to match the actual change in litter stock estimated from that paper.</t>
   </si>
 </sst>
 </file>
@@ -944,7 +950,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -958,6 +964,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1420,7 +1429,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>2</v>
@@ -1429,25 +1438,25 @@
         <v>3</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>64</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>65</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
@@ -1458,7 +1467,7 @@
         <v>34</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D2" s="1">
         <v>6</v>
@@ -1469,15 +1478,15 @@
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
       <c r="H2" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I2" s="1"/>
       <c r="J2" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K2" s="1"/>
       <c r="L2" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
@@ -1488,7 +1497,7 @@
         <v>34</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D3" s="1">
         <v>26</v>
@@ -1501,11 +1510,11 @@
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K3" s="1"/>
       <c r="L3" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
@@ -1516,7 +1525,7 @@
         <v>34</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D4" s="1">
         <v>0.3</v>
@@ -1529,11 +1538,11 @@
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K4" s="1"/>
       <c r="L4" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
@@ -1544,7 +1553,7 @@
         <v>34</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D5" s="1">
         <v>0.15</v>
@@ -1557,11 +1566,11 @@
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
       <c r="J5" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K5" s="1"/>
       <c r="L5" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
@@ -1572,7 +1581,7 @@
         <v>34</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D6" s="1">
         <v>73</v>
@@ -1587,15 +1596,15 @@
         <v>78</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="I6" s="1"/>
       <c r="J6" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K6" s="1"/>
       <c r="L6" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
@@ -1606,7 +1615,7 @@
         <v>34</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D7" s="1">
         <v>0.28000000000000003</v>
@@ -1621,15 +1630,15 @@
         <v>0.33</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="I7" s="1"/>
       <c r="J7" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K7" s="1"/>
       <c r="L7" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="30" x14ac:dyDescent="0.25">
@@ -1640,7 +1649,7 @@
         <v>34</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D8" s="1">
         <v>0.2</v>
@@ -1655,17 +1664,17 @@
         <v>0.3</v>
       </c>
       <c r="H8" t="s">
+        <v>117</v>
+      </c>
+      <c r="I8" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="I8" s="1" t="s">
-        <v>119</v>
-      </c>
       <c r="J8" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K8" s="1"/>
       <c r="L8" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
@@ -1676,7 +1685,7 @@
         <v>34</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D9" s="6">
         <f>D10*0.03</f>
@@ -1695,15 +1704,15 @@
         <v>17.920000000000002</v>
       </c>
       <c r="H9" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="I9" s="1"/>
       <c r="J9" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="K9" s="1"/>
       <c r="L9" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
@@ -1714,7 +1723,7 @@
         <v>34</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D10" s="1">
         <f>336/0.75</f>
@@ -1733,15 +1742,15 @@
         <v>448</v>
       </c>
       <c r="H10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="I10" s="1"/>
       <c r="J10" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="K10" s="1"/>
       <c r="L10" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
@@ -1765,15 +1774,15 @@
         <v>8</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="I11" s="1"/>
       <c r="J11" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K11" s="1"/>
       <c r="L11" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="30" x14ac:dyDescent="0.25">
@@ -1784,7 +1793,7 @@
         <v>34</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D12" s="1">
         <v>700</v>
@@ -1799,15 +1808,15 @@
         <v>1160</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I12" s="1"/>
       <c r="J12" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K12" s="1"/>
       <c r="L12" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="45" x14ac:dyDescent="0.25">
@@ -1818,7 +1827,7 @@
         <v>34</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D13" s="1">
         <f>0.217/365/6.45</f>
@@ -1834,15 +1843,15 @@
         <v>2.7906976744186045E-4</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="I13" s="1"/>
       <c r="J13" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K13" s="1"/>
       <c r="L13" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
@@ -1853,7 +1862,7 @@
         <v>34</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D14" s="1">
         <v>0.53</v>
@@ -1868,11 +1877,11 @@
       </c>
       <c r="I14" s="1"/>
       <c r="J14" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K14" s="1"/>
       <c r="L14" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
@@ -1883,7 +1892,7 @@
         <v>34</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D15" s="1">
         <v>0.09</v>
@@ -1898,11 +1907,11 @@
       </c>
       <c r="I15" s="1"/>
       <c r="J15" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K15" s="1"/>
       <c r="L15" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
@@ -1913,7 +1922,7 @@
         <v>34</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D16" s="1">
         <v>0.22</v>
@@ -1928,11 +1937,11 @@
       </c>
       <c r="I16" s="1"/>
       <c r="J16" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K16" s="1"/>
       <c r="L16" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="17" spans="1:12" ht="30" x14ac:dyDescent="0.25">
@@ -1943,7 +1952,7 @@
         <v>34</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D17" s="5">
         <f>0.00207/0.0375</f>
@@ -1955,15 +1964,15 @@
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
       <c r="H17" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="I17" s="1"/>
       <c r="J17" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K17" s="1"/>
       <c r="L17" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="18" spans="1:12" ht="30" x14ac:dyDescent="0.25">
@@ -1974,7 +1983,7 @@
         <v>34</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D18" s="5">
         <f>0.00207/0.0375</f>
@@ -1986,15 +1995,15 @@
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
       <c r="H18" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="I18" s="1"/>
       <c r="J18" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K18" s="1"/>
       <c r="L18" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="19" spans="1:12" ht="30" x14ac:dyDescent="0.25">
@@ -2005,7 +2014,7 @@
         <v>34</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D19" s="5">
         <f>0.00207/0.0375</f>
@@ -2017,15 +2026,15 @@
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
       <c r="H19" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="I19" s="1"/>
       <c r="J19" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K19" s="1"/>
       <c r="L19" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="30" x14ac:dyDescent="0.25">
@@ -2036,7 +2045,7 @@
         <v>34</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D20" s="1">
         <v>0</v>
@@ -2048,14 +2057,14 @@
       <c r="G20" s="1"/>
       <c r="H20" s="1"/>
       <c r="I20" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K20" s="1"/>
       <c r="L20" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="21" spans="1:12" ht="45" x14ac:dyDescent="0.25">
@@ -2066,26 +2075,28 @@
         <v>34</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D21" s="1">
-        <v>-0.02</v>
+        <v>-5.5040310000000002E-2</v>
       </c>
       <c r="E21" s="1">
         <v>0</v>
       </c>
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
-      <c r="H21" s="1"/>
+      <c r="H21" s="1" t="s">
+        <v>137</v>
+      </c>
       <c r="I21" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K21" s="1"/>
       <c r="L21" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
@@ -2096,7 +2107,7 @@
         <v>35</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D22" s="1">
         <v>6</v>
@@ -2108,14 +2119,14 @@
       <c r="G22" s="1"/>
       <c r="H22" s="1"/>
       <c r="I22" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K22" s="1"/>
       <c r="L22" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.25">
@@ -2126,7 +2137,7 @@
         <v>35</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D23" s="1">
         <v>26</v>
@@ -2138,14 +2149,14 @@
       <c r="G23" s="1"/>
       <c r="H23" s="1"/>
       <c r="I23" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K23" s="1"/>
       <c r="L23" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.25">
@@ -2156,7 +2167,7 @@
         <v>35</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D24" s="1">
         <v>0.3</v>
@@ -2168,14 +2179,14 @@
       <c r="G24" s="1"/>
       <c r="H24" s="1"/>
       <c r="I24" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K24" s="1"/>
       <c r="L24" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
@@ -2186,7 +2197,7 @@
         <v>35</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D25" s="1">
         <v>0.15</v>
@@ -2198,14 +2209,14 @@
       <c r="G25" s="1"/>
       <c r="H25" s="1"/>
       <c r="I25" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K25" s="1"/>
       <c r="L25" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.25">
@@ -2216,7 +2227,7 @@
         <v>35</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D26" s="1">
         <v>70</v>
@@ -2228,14 +2239,14 @@
       <c r="G26" s="1"/>
       <c r="H26" s="1"/>
       <c r="I26" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K26" s="1"/>
       <c r="L26" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.25">
@@ -2246,7 +2257,7 @@
         <v>35</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D27" s="1">
         <v>0.4</v>
@@ -2258,14 +2269,14 @@
       <c r="G27" s="1"/>
       <c r="H27" s="1"/>
       <c r="I27" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K27" s="1"/>
       <c r="L27" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
@@ -2276,7 +2287,7 @@
         <v>35</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D28" s="1">
         <v>0.2</v>
@@ -2288,14 +2299,14 @@
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
       <c r="I28" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K28" s="1"/>
       <c r="L28" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
@@ -2306,7 +2317,7 @@
         <v>35</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D29" s="1">
         <v>50</v>
@@ -2318,14 +2329,14 @@
       <c r="G29" s="1"/>
       <c r="H29" s="1"/>
       <c r="I29" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="J29" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="K29" s="1"/>
       <c r="L29" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.25">
@@ -2336,7 +2347,7 @@
         <v>35</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D30" s="1">
         <v>1270</v>
@@ -2348,14 +2359,14 @@
       <c r="G30" s="1"/>
       <c r="H30" s="1"/>
       <c r="I30" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="K30" s="1"/>
       <c r="L30" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.25">
@@ -2375,17 +2386,17 @@
       <c r="F31" s="1"/>
       <c r="G31" s="1"/>
       <c r="H31" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K31" s="1"/>
       <c r="L31" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.25">
@@ -2396,7 +2407,7 @@
         <v>35</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D32" s="1">
         <v>1300</v>
@@ -2408,14 +2419,14 @@
       <c r="G32" s="1"/>
       <c r="H32" s="1"/>
       <c r="I32" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K32" s="1"/>
       <c r="L32" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.25">
@@ -2426,7 +2437,7 @@
         <v>35</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D33" s="1">
         <f>1/(2.5*365)</f>
@@ -2438,17 +2449,17 @@
       <c r="F33" s="1"/>
       <c r="G33" s="1"/>
       <c r="H33" s="1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="I33" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="J33" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K33" s="1"/>
       <c r="L33" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.25">
@@ -2459,7 +2470,7 @@
         <v>35</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D34" s="1">
         <v>0.5</v>
@@ -2471,14 +2482,14 @@
       <c r="G34" s="1"/>
       <c r="H34" s="1"/>
       <c r="I34" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K34" s="1"/>
       <c r="L34" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.25">
@@ -2489,7 +2500,7 @@
         <v>35</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D35" s="1">
         <v>0.35</v>
@@ -2501,14 +2512,14 @@
       <c r="G35" s="1"/>
       <c r="H35" s="1"/>
       <c r="I35" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K35" s="1"/>
       <c r="L35" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.25">
@@ -2519,7 +2530,7 @@
         <v>35</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>40</v>
@@ -2531,14 +2542,14 @@
       <c r="G36" s="1"/>
       <c r="H36" s="1"/>
       <c r="I36" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="J36" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K36" s="1"/>
       <c r="L36" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="37" spans="1:12" ht="30" x14ac:dyDescent="0.25">
@@ -2549,26 +2560,28 @@
         <v>35</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="D37" s="1">
-        <v>6.0100000000000001E-2</v>
+        <v>124</v>
+      </c>
+      <c r="D37" s="7">
+        <v>0.4236007</v>
       </c>
       <c r="E37" s="1">
         <v>0</v>
       </c>
       <c r="F37" s="1"/>
       <c r="G37" s="1"/>
-      <c r="H37" s="1"/>
+      <c r="H37" s="1" t="s">
+        <v>138</v>
+      </c>
       <c r="I37" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="J37" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K37" s="1"/>
       <c r="L37" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="38" spans="1:12" ht="30" x14ac:dyDescent="0.25">
@@ -2579,26 +2592,28 @@
         <v>35</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="D38" s="1">
-        <v>6.0100000000000001E-2</v>
+        <v>124</v>
+      </c>
+      <c r="D38" s="7">
+        <v>0.4236007</v>
       </c>
       <c r="E38" s="1">
         <v>0</v>
       </c>
       <c r="F38" s="1"/>
       <c r="G38" s="1"/>
-      <c r="H38" s="1"/>
+      <c r="H38" s="1" t="s">
+        <v>138</v>
+      </c>
       <c r="I38" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="J38" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K38" s="1"/>
       <c r="L38" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.25">
@@ -2609,7 +2624,7 @@
         <v>43</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D39" s="1">
         <v>12</v>
@@ -2624,11 +2639,11 @@
       </c>
       <c r="I39" s="1"/>
       <c r="J39" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K39" s="1"/>
       <c r="L39" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.25">
@@ -2639,7 +2654,7 @@
         <v>43</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D40" s="1">
         <v>20</v>
@@ -2654,11 +2669,11 @@
       </c>
       <c r="I40" s="1"/>
       <c r="J40" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K40" s="1"/>
       <c r="L40" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="41" spans="1:12" ht="45" x14ac:dyDescent="0.25">
@@ -2669,7 +2684,7 @@
         <v>43</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D41" s="1">
         <v>0.2</v>
@@ -2684,11 +2699,11 @@
       </c>
       <c r="I41" s="1"/>
       <c r="J41" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K41" s="1"/>
       <c r="L41" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="42" spans="1:12" ht="45" x14ac:dyDescent="0.25">
@@ -2699,7 +2714,7 @@
         <v>43</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D42" s="1">
         <v>0.1</v>
@@ -2714,11 +2729,11 @@
       </c>
       <c r="I42" s="1"/>
       <c r="J42" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K42" s="1"/>
       <c r="L42" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.25">
@@ -2729,7 +2744,7 @@
         <v>43</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D43" s="1">
         <v>0.45</v>
@@ -2744,11 +2759,11 @@
       </c>
       <c r="I43" s="1"/>
       <c r="J43" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K43" s="1"/>
       <c r="L43" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.25">
@@ -2759,7 +2774,7 @@
         <v>43</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D44" s="1">
         <v>0.22</v>
@@ -2774,11 +2789,11 @@
       </c>
       <c r="I44" s="1"/>
       <c r="J44" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K44" s="1"/>
       <c r="L44" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.25">
@@ -2789,7 +2804,7 @@
         <v>43</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D45" s="1">
         <v>0.21</v>
@@ -2801,15 +2816,15 @@
       <c r="F45" s="1"/>
       <c r="G45" s="1"/>
       <c r="H45" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I45" s="1"/>
       <c r="J45" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K45" s="1"/>
       <c r="L45" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.25">
@@ -2820,7 +2835,7 @@
         <v>43</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D46" s="1">
         <v>212</v>
@@ -2835,15 +2850,15 @@
         <v>290</v>
       </c>
       <c r="H46" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I46" s="1"/>
       <c r="J46" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="K46" s="1"/>
       <c r="L46" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.25">
@@ -2854,7 +2869,7 @@
         <v>43</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D47" s="1">
         <v>1428</v>
@@ -2869,15 +2884,15 @@
         <v>1481</v>
       </c>
       <c r="H47" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I47" s="1"/>
       <c r="J47" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="K47" s="1"/>
       <c r="L47" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.25">
@@ -2897,15 +2912,15 @@
       <c r="F48" s="1"/>
       <c r="G48" s="1"/>
       <c r="H48" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I48" s="3"/>
       <c r="J48" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K48" s="1"/>
       <c r="L48" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.25">
@@ -2916,7 +2931,7 @@
         <v>43</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D49" s="1">
         <v>880</v>
@@ -2931,15 +2946,15 @@
         <v>960</v>
       </c>
       <c r="H49" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I49" s="3"/>
       <c r="J49" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K49" s="1"/>
       <c r="L49" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="50" spans="1:12" ht="30" x14ac:dyDescent="0.25">
@@ -2950,7 +2965,7 @@
         <v>43</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D50" s="1">
         <v>5.7999999999999996E-3</v>
@@ -2965,11 +2980,11 @@
       </c>
       <c r="I50" s="1"/>
       <c r="J50" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K50" s="1"/>
       <c r="L50" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="51" spans="1:12" ht="30" x14ac:dyDescent="0.25">
@@ -2980,7 +2995,7 @@
         <v>43</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D51" s="1">
         <v>0.50930200000000003</v>
@@ -2995,11 +3010,11 @@
       </c>
       <c r="I51" s="1"/>
       <c r="J51" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K51" s="1"/>
       <c r="L51" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="52" spans="1:12" ht="30" x14ac:dyDescent="0.25">
@@ -3010,7 +3025,7 @@
         <v>43</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D52" s="1">
         <v>0.35</v>
@@ -3025,11 +3040,11 @@
       </c>
       <c r="I52" s="1"/>
       <c r="J52" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K52" s="1"/>
       <c r="L52" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="53" spans="1:12" ht="30" x14ac:dyDescent="0.25">
@@ -3040,7 +3055,7 @@
         <v>43</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D53" s="2" t="s">
         <v>48</v>
@@ -3055,14 +3070,14 @@
       </c>
       <c r="I53" s="1"/>
       <c r="J53" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K53" s="1"/>
       <c r="L53" s="1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="54" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>41</v>
       </c>
@@ -3070,10 +3085,10 @@
         <v>43</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D54" s="1">
-        <v>6.0100000000000001E-2</v>
+        <v>10.204700000000001</v>
       </c>
       <c r="E54" s="1">
         <v>1.2E-2</v>
@@ -3081,15 +3096,15 @@
       <c r="F54" s="1"/>
       <c r="G54" s="1"/>
       <c r="H54" s="1" t="s">
-        <v>50</v>
+        <v>139</v>
       </c>
       <c r="I54" s="1"/>
       <c r="J54" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K54" s="1"/>
       <c r="L54" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="55" spans="1:12" ht="30" x14ac:dyDescent="0.25">
@@ -3100,10 +3115,10 @@
         <v>43</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D55" s="1">
-        <v>6.0100000000000001E-2</v>
+        <v>10.204700000000001</v>
       </c>
       <c r="E55" s="1">
         <v>1.2E-2</v>
@@ -3111,17 +3126,17 @@
       <c r="F55" s="1"/>
       <c r="G55" s="1"/>
       <c r="H55" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="I55" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="I55" s="1" t="s">
-        <v>110</v>
-      </c>
       <c r="J55" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K55" s="1"/>
       <c r="L55" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="56" spans="1:12" x14ac:dyDescent="0.25">
@@ -3129,10 +3144,10 @@
         <v>11</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D56" s="1">
         <v>12</v>
@@ -3147,11 +3162,11 @@
       </c>
       <c r="I56" s="1"/>
       <c r="J56" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K56" s="1"/>
       <c r="L56" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="57" spans="1:12" x14ac:dyDescent="0.25">
@@ -3159,10 +3174,10 @@
         <v>12</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D57" s="1">
         <v>20</v>
@@ -3177,11 +3192,11 @@
       </c>
       <c r="I57" s="1"/>
       <c r="J57" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K57" s="1"/>
       <c r="L57" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="58" spans="1:12" ht="45" x14ac:dyDescent="0.25">
@@ -3189,10 +3204,10 @@
         <v>13</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D58" s="1">
         <v>0.2</v>
@@ -3207,11 +3222,11 @@
       </c>
       <c r="I58" s="1"/>
       <c r="J58" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K58" s="1"/>
       <c r="L58" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="59" spans="1:12" ht="45" x14ac:dyDescent="0.25">
@@ -3219,10 +3234,10 @@
         <v>14</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D59" s="1">
         <v>0.1</v>
@@ -3237,11 +3252,11 @@
       </c>
       <c r="I59" s="1"/>
       <c r="J59" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K59" s="1"/>
       <c r="L59" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="60" spans="1:12" x14ac:dyDescent="0.25">
@@ -3249,10 +3264,10 @@
         <v>15</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D60" s="1">
         <v>0.45</v>
@@ -3267,11 +3282,11 @@
       </c>
       <c r="I60" s="1"/>
       <c r="J60" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K60" s="1"/>
       <c r="L60" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="61" spans="1:12" x14ac:dyDescent="0.25">
@@ -3279,10 +3294,10 @@
         <v>16</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D61" s="1">
         <v>0.22</v>
@@ -3297,11 +3312,11 @@
       </c>
       <c r="I61" s="1"/>
       <c r="J61" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K61" s="1"/>
       <c r="L61" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="62" spans="1:12" x14ac:dyDescent="0.25">
@@ -3309,10 +3324,10 @@
         <v>17</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D62" s="1">
         <v>0.21</v>
@@ -3324,15 +3339,15 @@
       <c r="F62" s="1"/>
       <c r="G62" s="1"/>
       <c r="H62" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I62" s="1"/>
       <c r="J62" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K62" s="1"/>
       <c r="L62" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="63" spans="1:12" x14ac:dyDescent="0.25">
@@ -3340,10 +3355,10 @@
         <v>18</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D63" s="1">
         <v>212</v>
@@ -3358,15 +3373,15 @@
         <v>290</v>
       </c>
       <c r="H63" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I63" s="1"/>
       <c r="J63" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="K63" s="1"/>
       <c r="L63" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.25">
@@ -3374,10 +3389,10 @@
         <v>19</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D64" s="1">
         <v>1428</v>
@@ -3392,15 +3407,15 @@
         <v>1481</v>
       </c>
       <c r="H64" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I64" s="1"/>
       <c r="J64" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="K64" s="1"/>
       <c r="L64" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="65" spans="1:12" x14ac:dyDescent="0.25">
@@ -3408,7 +3423,7 @@
         <v>20</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C65" s="1"/>
       <c r="D65" s="1">
@@ -3420,15 +3435,15 @@
       <c r="F65" s="1"/>
       <c r="G65" s="1"/>
       <c r="H65" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I65" s="3"/>
       <c r="J65" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K65" s="1"/>
       <c r="L65" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="66" spans="1:12" x14ac:dyDescent="0.25">
@@ -3436,10 +3451,10 @@
         <v>21</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D66" s="1">
         <v>880</v>
@@ -3454,15 +3469,15 @@
         <v>960</v>
       </c>
       <c r="H66" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I66" s="3"/>
       <c r="J66" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K66" s="1"/>
       <c r="L66" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="67" spans="1:12" ht="30" x14ac:dyDescent="0.25">
@@ -3470,10 +3485,10 @@
         <v>36</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D67" s="1">
         <v>5.7999999999999996E-3</v>
@@ -3488,11 +3503,11 @@
       </c>
       <c r="I67" s="1"/>
       <c r="J67" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K67" s="1"/>
       <c r="L67" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="68" spans="1:12" ht="30" x14ac:dyDescent="0.25">
@@ -3500,10 +3515,10 @@
         <v>37</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D68" s="1">
         <v>0.50930200000000003</v>
@@ -3518,11 +3533,11 @@
       </c>
       <c r="I68" s="1"/>
       <c r="J68" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K68" s="1"/>
       <c r="L68" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="69" spans="1:12" ht="30" x14ac:dyDescent="0.25">
@@ -3530,10 +3545,10 @@
         <v>38</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D69" s="1">
         <v>0.35</v>
@@ -3548,11 +3563,11 @@
       </c>
       <c r="I69" s="1"/>
       <c r="J69" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K69" s="1"/>
       <c r="L69" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="70" spans="1:12" ht="30" x14ac:dyDescent="0.25">
@@ -3560,10 +3575,10 @@
         <v>39</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D70" s="2" t="s">
         <v>48</v>
@@ -3578,11 +3593,11 @@
       </c>
       <c r="I70" s="1"/>
       <c r="J70" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K70" s="1"/>
       <c r="L70" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="71" spans="1:12" ht="30" x14ac:dyDescent="0.25">
@@ -3590,10 +3605,10 @@
         <v>41</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D71" s="1">
         <v>6.0100000000000001E-2</v>
@@ -3606,11 +3621,11 @@
       <c r="H71" s="1"/>
       <c r="I71" s="1"/>
       <c r="J71" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K71" s="1"/>
       <c r="L71" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="72" spans="1:12" ht="30" x14ac:dyDescent="0.25">
@@ -3618,10 +3633,10 @@
         <v>42</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D72" s="1">
         <v>6.0100000000000001E-2</v>
@@ -3632,28 +3647,28 @@
       <c r="F72" s="1"/>
       <c r="G72" s="1"/>
       <c r="H72" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="I72" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="I72" s="1" t="s">
-        <v>110</v>
-      </c>
       <c r="J72" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K72" s="1"/>
       <c r="L72" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="73" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D73" s="1">
         <v>5.1000000000000004E-3</v>
@@ -3668,22 +3683,22 @@
       </c>
       <c r="I73" s="1"/>
       <c r="J73" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K73" s="1"/>
       <c r="L73" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="74" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D74" s="1">
         <v>0.6</v>
@@ -3698,22 +3713,22 @@
       </c>
       <c r="I74" s="1"/>
       <c r="J74" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K74" s="1"/>
       <c r="L74" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="75" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D75" s="1">
         <v>0.35</v>
@@ -3728,22 +3743,22 @@
       </c>
       <c r="I75" s="1"/>
       <c r="J75" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K75" s="1"/>
       <c r="L75" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="76" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D76" s="1">
         <v>1.6799999999999999E-2</v>
@@ -3754,15 +3769,15 @@
       <c r="F76" s="1"/>
       <c r="G76" s="1"/>
       <c r="H76" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="I76" s="1"/>
       <c r="J76" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K76" s="1"/>
       <c r="L76" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="77" spans="1:12" x14ac:dyDescent="0.25">
@@ -3770,10 +3785,10 @@
         <v>11</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D77" s="1">
         <v>10</v>
@@ -3785,17 +3800,17 @@
       <c r="F77" s="1"/>
       <c r="G77" s="1"/>
       <c r="H77" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="I77" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="I77" s="1" t="s">
-        <v>84</v>
-      </c>
       <c r="J77" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K77" s="1"/>
       <c r="L77" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="78" spans="1:12" x14ac:dyDescent="0.25">
@@ -3803,10 +3818,10 @@
         <v>12</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D78" s="1">
         <v>26</v>
@@ -3818,17 +3833,17 @@
       <c r="F78" s="1"/>
       <c r="G78" s="1"/>
       <c r="H78" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="I78" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="I78" s="1" t="s">
-        <v>84</v>
-      </c>
       <c r="J78" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K78" s="1"/>
       <c r="L78" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="79" spans="1:12" x14ac:dyDescent="0.25">
@@ -3836,10 +3851,10 @@
         <v>13</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D79" s="1">
         <v>0.3</v>
@@ -3851,17 +3866,17 @@
       <c r="F79" s="1"/>
       <c r="G79" s="1"/>
       <c r="H79" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="I79" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="I79" s="1" t="s">
-        <v>84</v>
-      </c>
       <c r="J79" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K79" s="1"/>
       <c r="L79" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="80" spans="1:12" x14ac:dyDescent="0.25">
@@ -3869,10 +3884,10 @@
         <v>14</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D80" s="1">
         <v>0.15</v>
@@ -3884,17 +3899,17 @@
       <c r="F80" s="1"/>
       <c r="G80" s="1"/>
       <c r="H80" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="I80" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="I80" s="1" t="s">
-        <v>84</v>
-      </c>
       <c r="J80" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K80" s="1"/>
       <c r="L80" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="81" spans="1:12" x14ac:dyDescent="0.25">
@@ -3902,10 +3917,10 @@
         <v>15</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D81" s="1">
         <v>70</v>
@@ -3917,17 +3932,17 @@
       <c r="F81" s="1"/>
       <c r="G81" s="1"/>
       <c r="H81" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="I81" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="I81" s="1" t="s">
-        <v>84</v>
-      </c>
       <c r="J81" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K81" s="1"/>
       <c r="L81" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="82" spans="1:12" x14ac:dyDescent="0.25">
@@ -3935,10 +3950,10 @@
         <v>16</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D82" s="1">
         <v>0.4</v>
@@ -3950,17 +3965,17 @@
       <c r="F82" s="1"/>
       <c r="G82" s="1"/>
       <c r="H82" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="I82" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="I82" s="1" t="s">
-        <v>84</v>
-      </c>
       <c r="J82" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K82" s="1"/>
       <c r="L82" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="83" spans="1:12" x14ac:dyDescent="0.25">
@@ -3968,10 +3983,10 @@
         <v>17</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D83" s="1">
         <v>0.2</v>
@@ -3983,17 +3998,17 @@
       <c r="F83" s="1"/>
       <c r="G83" s="1"/>
       <c r="H83" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="I83" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="I83" s="1" t="s">
-        <v>84</v>
-      </c>
       <c r="J83" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K83" s="1"/>
       <c r="L83" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="84" spans="1:12" x14ac:dyDescent="0.25">
@@ -4001,10 +4016,10 @@
         <v>18</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D84" s="1">
         <v>433</v>
@@ -4016,17 +4031,17 @@
       <c r="F84" s="1"/>
       <c r="G84" s="1"/>
       <c r="H84" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="I84" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="I84" s="1" t="s">
-        <v>84</v>
-      </c>
       <c r="J84" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="K84" s="1"/>
       <c r="L84" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="85" spans="1:12" x14ac:dyDescent="0.25">
@@ -4034,10 +4049,10 @@
         <v>19</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D85" s="1">
         <v>0</v>
@@ -4049,17 +4064,17 @@
       <c r="F85" s="1"/>
       <c r="G85" s="1"/>
       <c r="H85" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="I85" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="I85" s="1" t="s">
-        <v>84</v>
-      </c>
       <c r="J85" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="K85" s="1"/>
       <c r="L85" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="86" spans="1:12" x14ac:dyDescent="0.25">
@@ -4067,7 +4082,7 @@
         <v>20</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C86" s="1"/>
       <c r="D86" s="1">
@@ -4080,17 +4095,17 @@
       <c r="F86" s="1"/>
       <c r="G86" s="1"/>
       <c r="H86" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="I86" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="I86" s="1" t="s">
-        <v>84</v>
-      </c>
       <c r="J86" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K86" s="1"/>
       <c r="L86" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="87" spans="1:12" x14ac:dyDescent="0.25">
@@ -4098,10 +4113,10 @@
         <v>21</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D87" s="1">
         <v>1300</v>
@@ -4113,28 +4128,28 @@
       <c r="F87" s="1"/>
       <c r="G87" s="1"/>
       <c r="H87" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="I87" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="I87" s="1" t="s">
-        <v>84</v>
-      </c>
       <c r="J87" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K87" s="1"/>
       <c r="L87" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="88" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D88" s="1">
         <v>0.02</v>
@@ -4146,28 +4161,28 @@
       <c r="F88" s="1"/>
       <c r="G88" s="1"/>
       <c r="H88" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="I88" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="I88" s="1" t="s">
-        <v>84</v>
-      </c>
       <c r="J88" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K88" s="1"/>
       <c r="L88" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="89" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D89" s="1">
         <f>1/36</f>
@@ -4180,28 +4195,28 @@
       <c r="F89" s="1"/>
       <c r="G89" s="1"/>
       <c r="H89" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I89" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="I89" s="1" t="s">
-        <v>82</v>
-      </c>
       <c r="J89" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K89" s="1"/>
       <c r="L89" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="90" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D90" s="1">
         <v>0.5</v>
@@ -4213,25 +4228,25 @@
       <c r="F90" s="1"/>
       <c r="G90" s="1"/>
       <c r="H90" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="I90" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J90" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K90" s="1"/>
       <c r="L90" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="91" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C91" s="1"/>
       <c r="D91" s="1">
@@ -4244,28 +4259,28 @@
       <c r="F91" s="1"/>
       <c r="G91" s="1"/>
       <c r="H91" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="I91" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J91" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K91" s="1"/>
       <c r="L91" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="92" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D92" s="5">
         <v>2.7399999999999999E-5</v>
@@ -4277,28 +4292,28 @@
       <c r="F92" s="1"/>
       <c r="G92" s="1"/>
       <c r="H92" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I92" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J92" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K92" s="1"/>
       <c r="L92" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="93" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D93" s="5">
         <v>1.2999999999999999E-5</v>
@@ -4310,17 +4325,17 @@
       <c r="F93" s="1"/>
       <c r="G93" s="1"/>
       <c r="H93" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I93" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J93" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K93" s="1"/>
       <c r="L93" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -4346,27 +4361,27 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>86</v>
+      </c>
+      <c r="D1" t="s">
         <v>87</v>
-      </c>
-      <c r="D1" t="s">
-        <v>88</v>
       </c>
       <c r="E1" t="s">
         <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B2" t="s">
         <v>34</v>
@@ -4379,15 +4394,15 @@
         <v>6.45</v>
       </c>
       <c r="E2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B3" t="s">
         <v>35</v>
@@ -4400,15 +4415,15 @@
         <v>1.875</v>
       </c>
       <c r="E3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B4" t="s">
         <v>43</v>
@@ -4420,18 +4435,18 @@
         <v>0.1</v>
       </c>
       <c r="E4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C5" t="s">
         <v>9</v>
@@ -4440,18 +4455,18 @@
         <v>0.1</v>
       </c>
       <c r="E5" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C6" t="s">
         <v>10</v>
@@ -4460,18 +4475,18 @@
         <v>0.1</v>
       </c>
       <c r="E6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C7" t="s">
         <v>8</v>
@@ -4480,310 +4495,310 @@
         <v>0.1</v>
       </c>
       <c r="E7" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D8">
         <v>200</v>
       </c>
       <c r="E8" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D9">
         <v>200</v>
       </c>
       <c r="E9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>88</v>
+      </c>
+      <c r="B10" t="s">
+        <v>88</v>
+      </c>
+      <c r="C10" t="s">
         <v>89</v>
-      </c>
-      <c r="B10" t="s">
-        <v>89</v>
-      </c>
-      <c r="C10" t="s">
-        <v>90</v>
       </c>
       <c r="D10">
         <v>750</v>
       </c>
       <c r="E10" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F10" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B11" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C11" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D11">
         <v>6750</v>
       </c>
       <c r="E11" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F11" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B12" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C12" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D12">
         <v>2500</v>
       </c>
       <c r="E12" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F12" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B13" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C13" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D13">
         <v>200</v>
       </c>
       <c r="E13" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F13" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B14" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C14" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D14">
         <v>1000</v>
       </c>
       <c r="E14" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F14" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B15" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C15" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D15">
         <v>2000</v>
       </c>
       <c r="E15" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B16" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C16" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D16">
         <v>10</v>
       </c>
       <c r="E16" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B17" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C17" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D17">
         <v>0.1</v>
       </c>
       <c r="E17" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F17" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B18" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C18" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D18">
         <v>400</v>
       </c>
       <c r="E18" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F18" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B19" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C19" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D19">
         <v>10</v>
       </c>
       <c r="E19" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F19" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B20" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C20" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D20">
         <v>1000</v>
       </c>
       <c r="E20" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F20" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B21" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C21" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D21">
         <v>3000</v>
       </c>
       <c r="E21" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F21" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B22" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C22" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D22">
         <v>40</v>
       </c>
       <c r="E22" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F22" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -4802,13 +4817,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -5014,7 +5029,7 @@
         <v>5</v>
       </c>
       <c r="B20" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C20">
         <v>1</v>
@@ -5025,7 +5040,7 @@
         <v>6</v>
       </c>
       <c r="B21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C21">
         <v>1</v>
@@ -5036,7 +5051,7 @@
         <v>7</v>
       </c>
       <c r="B22" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C22">
         <v>0</v>
@@ -5047,7 +5062,7 @@
         <v>8</v>
       </c>
       <c r="B23" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C23">
         <v>0</v>
@@ -5058,7 +5073,7 @@
         <v>9</v>
       </c>
       <c r="B24" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C24">
         <v>1</v>
@@ -5069,7 +5084,7 @@
         <v>10</v>
       </c>
       <c r="B25" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C25">
         <v>1</v>
@@ -5080,7 +5095,7 @@
         <v>5</v>
       </c>
       <c r="B26" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C26">
         <v>0</v>
@@ -5091,7 +5106,7 @@
         <v>6</v>
       </c>
       <c r="B27" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C27">
         <v>1</v>
@@ -5102,7 +5117,7 @@
         <v>7</v>
       </c>
       <c r="B28" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C28">
         <v>0</v>
@@ -5113,7 +5128,7 @@
         <v>8</v>
       </c>
       <c r="B29" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C29">
         <v>1</v>
@@ -5124,7 +5139,7 @@
         <v>9</v>
       </c>
       <c r="B30" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C30">
         <v>0</v>
@@ -5135,7 +5150,7 @@
         <v>10</v>
       </c>
       <c r="B31" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C31">
         <v>0</v>

</xml_diff>

<commit_message>
Updated scenario inputs with IU group edits.
</commit_message>
<xml_diff>
--- a/Data/scenarios.xlsx
+++ b/Data/scenarios.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rober\Documents\GitHub Repos\merging_SFW_decomposition_models\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66AC3B62-5DF2-4B0F-B986-A0633F966EF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58121FC9-7A10-4CEF-9D21-C059D2F07BA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{7C97690C-9E7B-4D0E-86C0-16835BCB4BB0}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{7C97690C-9E7B-4D0E-86C0-16835BCB4BB0}"/>
   </bookViews>
   <sheets>
     <sheet name="scenarios" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="756" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="613" uniqueCount="146">
   <si>
     <t>Parameter</t>
   </si>
@@ -190,21 +190,6 @@
     <t>MitePredator</t>
   </si>
   <si>
-    <t>d_detpredator</t>
-  </si>
-  <si>
-    <t>a_detpredator</t>
-  </si>
-  <si>
-    <t>p_detpredator</t>
-  </si>
-  <si>
-    <t>c_detpredator</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Calculated based on the data presented by Barros et al. 2025 and Castilho et al. 2009 on the predation rates of soil Mesostigmata feeding on Astigmata in laboratory conditions </t>
-  </si>
-  <si>
     <t>RootHerbivore</t>
   </si>
   <si>
@@ -265,9 +250,6 @@
     <t>Wieder et al. 2015; SD is a placeholder</t>
   </si>
   <si>
-    <t>Barreto et al. 2024</t>
-  </si>
-  <si>
     <t>Yoo et al. in prep</t>
   </si>
   <si>
@@ -277,15 +259,9 @@
     <t>Provide SD or min-max</t>
   </si>
   <si>
-    <t>Bongers and Bongers, 1998; van den Hoogen et al. 2019</t>
-  </si>
-  <si>
     <t>SD or min/max</t>
   </si>
   <si>
-    <t>????</t>
-  </si>
-  <si>
     <t>Reference and SD</t>
   </si>
   <si>
@@ -455,13 +431,55 @@
   </si>
   <si>
     <t>Buchkowski et al. 2024; Buchkowski and Schmitz 2022 for average weight from WE plots; 25% dry weight, 50% carbon</t>
+  </si>
+  <si>
+    <t>Konza Prarie LTER: https://kpbs.konza.k-state.edu provides range</t>
+  </si>
+  <si>
+    <t>unchanged from defaults- but can calculate from temp min/max (full temp range is 29.3C; tamp =14.65)</t>
+  </si>
+  <si>
+    <t>unchanged from defaults; suggested min and max are from nelson et al 2004 (https://doi.org/10.1023/B:PLSO.0000020957.83641.62)</t>
+  </si>
+  <si>
+    <t>unchanged from defaults; suggested min and max are from morgan et al, 2016 (https://doi.org/10.1016/j.rama.2016.05.002)</t>
+  </si>
+  <si>
+    <t>Konza Prarie LTER: https://kpbs.konza.k-state.edu states silty clay loam; min max based on USDA soil texture (https://soilseries.sc.egov.usda.gov/OSD_Docs/K/KONZA.html)</t>
+  </si>
+  <si>
+    <t>Based on USDA soil texture for silty clay loam</t>
+  </si>
+  <si>
+    <t>unchanged from defaults; brandt et al  2010 have range of 6.61% (se: 0.55) - 8.10% (0.37) percent lignin (https://doi.org/10.1007/s10021-010-9353-2)</t>
+  </si>
+  <si>
+    <t>Franco et al., 2020</t>
+  </si>
+  <si>
+    <t>None - trees are excluded completely from this model</t>
+  </si>
+  <si>
+    <t>described as moderately alkanine to moderately acidic - https://soilseries.sc.egov.usda.gov/OSD_Docs/K/KONZA.html</t>
+  </si>
+  <si>
+    <t>Haveren et al, 1983; https://doi.org/10.2307/3898346</t>
+  </si>
+  <si>
+    <t>Calculated using the carbon biomass of nematodes (avg. 1.82*10-6 gC/m2) and root carbon (avg. 95.28 gC/m2) from Franco 2020 and the parameters below; calculated F then c</t>
+  </si>
+  <si>
+    <t>Chitambar et al. 2018</t>
+  </si>
+  <si>
+    <t>Barreto et al. 2024; these are percentages reported in suppl.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -608,8 +626,16 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="33">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -789,6 +815,18 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="10">
     <border>
@@ -906,7 +944,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="42">
+  <cellStyleXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
@@ -949,8 +987,9 @@
     <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -959,7 +998,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -969,8 +1007,19 @@
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" xfId="42" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="42">
+  <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
     <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
     <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
@@ -1004,6 +1053,7 @@
     <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
     <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
     <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Hyperlink" xfId="42" builtinId="8"/>
     <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
     <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
     <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
@@ -1071,8 +1121,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1759F6D4-436C-4273-8592-6F473E4E1FC6}" name="Table1" displayName="Table1" ref="A1:L93" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
-  <autoFilter ref="A1:L93" xr:uid="{1759F6D4-436C-4273-8592-6F473E4E1FC6}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1759F6D4-436C-4273-8592-6F473E4E1FC6}" name="Table1" displayName="Table1" ref="A1:L72" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+  <autoFilter ref="A1:L72" xr:uid="{1759F6D4-436C-4273-8592-6F473E4E1FC6}"/>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{9C63AD24-02BE-4FC6-8589-25FEAC9E29E1}" name="Parameter" dataDxfId="11"/>
     <tableColumn id="2" xr3:uid="{6FFFFAD3-CDDD-4A47-9019-7C5E6785F73D}" name="Scenario" dataDxfId="10"/>
@@ -1408,14 +1458,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD4418A0-EB93-4361-AE80-4D25DF544368}">
-  <dimension ref="A1:L93"/>
+  <dimension ref="A1:L72"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.26953125" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="22.7265625" customWidth="1"/>
-    <col min="4" max="4" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.90625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.36328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.6328125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="52.26953125" bestFit="1" customWidth="1"/>
     <col min="9" max="10" width="23" customWidth="1"/>
     <col min="11" max="11" width="13.26953125" customWidth="1"/>
@@ -1429,7 +1480,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>2</v>
@@ -1438,25 +1489,25 @@
         <v>3</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.35">
@@ -1467,7 +1518,7 @@
         <v>34</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="D2" s="1">
         <v>6</v>
@@ -1478,15 +1529,15 @@
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
       <c r="H2" s="1" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="I2" s="1"/>
       <c r="J2" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="K2" s="1"/>
       <c r="L2" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
@@ -1497,7 +1548,7 @@
         <v>34</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="D3" s="1">
         <v>26</v>
@@ -1510,11 +1561,11 @@
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="K3" s="1"/>
       <c r="L3" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.35">
@@ -1525,7 +1576,7 @@
         <v>34</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="D4" s="1">
         <v>0.3</v>
@@ -1538,11 +1589,11 @@
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="K4" s="1"/>
       <c r="L4" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
@@ -1553,7 +1604,7 @@
         <v>34</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="D5" s="1">
         <v>0.15</v>
@@ -1566,11 +1617,11 @@
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
       <c r="J5" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="K5" s="1"/>
       <c r="L5" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.35">
@@ -1581,7 +1632,7 @@
         <v>34</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="D6" s="1">
         <v>73</v>
@@ -1596,15 +1647,15 @@
         <v>78</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="I6" s="1"/>
       <c r="J6" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="K6" s="1"/>
       <c r="L6" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.35">
@@ -1615,7 +1666,7 @@
         <v>34</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="D7" s="1">
         <v>0.28000000000000003</v>
@@ -1630,15 +1681,15 @@
         <v>0.33</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="I7" s="1"/>
       <c r="J7" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="K7" s="1"/>
       <c r="L7" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="29" x14ac:dyDescent="0.35">
@@ -1649,7 +1700,7 @@
         <v>34</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="D8" s="1">
         <v>0.2</v>
@@ -1664,17 +1715,17 @@
         <v>0.3</v>
       </c>
       <c r="H8" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="K8" s="1"/>
       <c r="L8" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.35">
@@ -1685,34 +1736,34 @@
         <v>34</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="D9" s="6">
+        <v>116</v>
+      </c>
+      <c r="D9" s="5">
         <f>D10*0.03</f>
         <v>13.44</v>
       </c>
-      <c r="E9" s="6">
+      <c r="E9" s="5">
         <f>STDEV(Table1[[#This Row],[Min]:[Max]])</f>
         <v>9.9843477503540505</v>
       </c>
-      <c r="F9" s="6">
+      <c r="F9" s="5">
         <f>F10*0.01</f>
         <v>3.8000000000000003</v>
       </c>
-      <c r="G9" s="6">
+      <c r="G9" s="5">
         <f>G10*0.04</f>
         <v>17.920000000000002</v>
       </c>
       <c r="H9" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="I9" s="1"/>
       <c r="J9" s="1" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="K9" s="1"/>
       <c r="L9" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.35">
@@ -1723,13 +1774,13 @@
         <v>34</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="D10" s="1">
         <f>336/0.75</f>
         <v>448</v>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="5">
         <f>STDEV(Table1[[#This Row],[Min]:[Max]])</f>
         <v>48.083261120685229</v>
       </c>
@@ -1742,15 +1793,15 @@
         <v>448</v>
       </c>
       <c r="H10" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="I10" s="1"/>
       <c r="J10" s="1" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="K10" s="1"/>
       <c r="L10" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.35">
@@ -1774,15 +1825,15 @@
         <v>8</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="I11" s="1"/>
       <c r="J11" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="K11" s="1"/>
       <c r="L11" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="29" x14ac:dyDescent="0.35">
@@ -1793,7 +1844,7 @@
         <v>34</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="D12" s="1">
         <v>700</v>
@@ -1808,15 +1859,15 @@
         <v>1160</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="I12" s="1"/>
       <c r="J12" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="K12" s="1"/>
       <c r="L12" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="29" x14ac:dyDescent="0.35">
@@ -1827,7 +1878,7 @@
         <v>34</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="D13" s="1">
         <f>0.217/365/6.45</f>
@@ -1843,15 +1894,15 @@
         <v>2.7906976744186045E-4</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="I13" s="1"/>
       <c r="J13" s="1" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="K13" s="1"/>
       <c r="L13" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.35">
@@ -1862,7 +1913,7 @@
         <v>34</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="D14" s="1">
         <v>0.53</v>
@@ -1877,11 +1928,11 @@
       </c>
       <c r="I14" s="1"/>
       <c r="J14" s="1" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="K14" s="1"/>
       <c r="L14" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.35">
@@ -1892,7 +1943,7 @@
         <v>34</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="D15" s="1">
         <v>0.09</v>
@@ -1907,11 +1958,11 @@
       </c>
       <c r="I15" s="1"/>
       <c r="J15" s="1" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="K15" s="1"/>
       <c r="L15" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.35">
@@ -1922,7 +1973,7 @@
         <v>34</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="D16" s="1">
         <v>0.22</v>
@@ -1937,11 +1988,11 @@
       </c>
       <c r="I16" s="1"/>
       <c r="J16" s="1" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="K16" s="1"/>
       <c r="L16" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="17" spans="1:12" ht="29" x14ac:dyDescent="0.35">
@@ -1952,9 +2003,9 @@
         <v>34</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="D17" s="5">
+        <v>118</v>
+      </c>
+      <c r="D17" s="4">
         <f>0.00207/0.0375</f>
         <v>5.5199999999999999E-2</v>
       </c>
@@ -1964,15 +2015,15 @@
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
       <c r="H17" s="1" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="I17" s="1"/>
       <c r="J17" s="1" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="K17" s="1"/>
       <c r="L17" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="18" spans="1:12" ht="29" x14ac:dyDescent="0.35">
@@ -1983,9 +2034,9 @@
         <v>34</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="D18" s="5">
+        <v>118</v>
+      </c>
+      <c r="D18" s="4">
         <f>0.00207/0.0375</f>
         <v>5.5199999999999999E-2</v>
       </c>
@@ -1995,15 +2046,15 @@
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
       <c r="H18" s="1" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="I18" s="1"/>
       <c r="J18" s="1" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="K18" s="1"/>
       <c r="L18" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="19" spans="1:12" ht="29" x14ac:dyDescent="0.35">
@@ -2014,9 +2065,9 @@
         <v>34</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="D19" s="5">
+        <v>118</v>
+      </c>
+      <c r="D19" s="4">
         <f>0.00207/0.0375</f>
         <v>5.5199999999999999E-2</v>
       </c>
@@ -2026,15 +2077,15 @@
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
       <c r="H19" s="1" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="I19" s="1"/>
       <c r="J19" s="1" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="K19" s="1"/>
       <c r="L19" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="29" x14ac:dyDescent="0.35">
@@ -2045,7 +2096,7 @@
         <v>34</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="D20" s="1">
         <v>0</v>
@@ -2057,14 +2108,14 @@
       <c r="G20" s="1"/>
       <c r="H20" s="1"/>
       <c r="I20" s="1" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="K20" s="1"/>
       <c r="L20" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="21" spans="1:12" ht="29" x14ac:dyDescent="0.35">
@@ -2075,7 +2126,7 @@
         <v>34</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="D21" s="1">
         <v>-5.5040310000000002E-2</v>
@@ -2086,17 +2137,17 @@
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
       <c r="H21" s="1" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="K21" s="1"/>
       <c r="L21" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.35">
@@ -2107,7 +2158,7 @@
         <v>35</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="D22" s="1">
         <v>6</v>
@@ -2119,14 +2170,14 @@
       <c r="G22" s="1"/>
       <c r="H22" s="1"/>
       <c r="I22" s="1" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="K22" s="1"/>
       <c r="L22" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.35">
@@ -2137,7 +2188,7 @@
         <v>35</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="D23" s="1">
         <v>26</v>
@@ -2149,14 +2200,14 @@
       <c r="G23" s="1"/>
       <c r="H23" s="1"/>
       <c r="I23" s="1" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="K23" s="1"/>
       <c r="L23" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.35">
@@ -2167,7 +2218,7 @@
         <v>35</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="D24" s="1">
         <v>0.3</v>
@@ -2179,14 +2230,14 @@
       <c r="G24" s="1"/>
       <c r="H24" s="1"/>
       <c r="I24" s="1" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="K24" s="1"/>
       <c r="L24" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.35">
@@ -2197,7 +2248,7 @@
         <v>35</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="D25" s="1">
         <v>0.15</v>
@@ -2209,14 +2260,14 @@
       <c r="G25" s="1"/>
       <c r="H25" s="1"/>
       <c r="I25" s="1" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="K25" s="1"/>
       <c r="L25" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.35">
@@ -2227,7 +2278,7 @@
         <v>35</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="D26" s="1">
         <v>70</v>
@@ -2239,14 +2290,14 @@
       <c r="G26" s="1"/>
       <c r="H26" s="1"/>
       <c r="I26" s="1" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="K26" s="1"/>
       <c r="L26" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.35">
@@ -2257,7 +2308,7 @@
         <v>35</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="D27" s="1">
         <v>0.4</v>
@@ -2269,14 +2320,14 @@
       <c r="G27" s="1"/>
       <c r="H27" s="1"/>
       <c r="I27" s="1" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="K27" s="1"/>
       <c r="L27" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.35">
@@ -2287,7 +2338,7 @@
         <v>35</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="D28" s="1">
         <v>0.2</v>
@@ -2299,14 +2350,14 @@
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
       <c r="I28" s="1" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="K28" s="1"/>
       <c r="L28" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.35">
@@ -2317,7 +2368,7 @@
         <v>35</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="D29" s="1">
         <v>50</v>
@@ -2329,14 +2380,14 @@
       <c r="G29" s="1"/>
       <c r="H29" s="1"/>
       <c r="I29" s="1" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="J29" s="1" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="K29" s="1"/>
       <c r="L29" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.35">
@@ -2347,7 +2398,7 @@
         <v>35</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="D30" s="1">
         <v>1270</v>
@@ -2359,14 +2410,14 @@
       <c r="G30" s="1"/>
       <c r="H30" s="1"/>
       <c r="I30" s="1" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="K30" s="1"/>
       <c r="L30" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.35">
@@ -2386,17 +2437,17 @@
       <c r="F31" s="1"/>
       <c r="G31" s="1"/>
       <c r="H31" s="1" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="K31" s="1"/>
       <c r="L31" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.35">
@@ -2407,7 +2458,7 @@
         <v>35</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="D32" s="1">
         <v>1300</v>
@@ -2419,14 +2470,14 @@
       <c r="G32" s="1"/>
       <c r="H32" s="1"/>
       <c r="I32" s="1" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="K32" s="1"/>
       <c r="L32" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.35">
@@ -2437,7 +2488,7 @@
         <v>35</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="D33" s="1">
         <f>1/(2.5*365)</f>
@@ -2449,17 +2500,17 @@
       <c r="F33" s="1"/>
       <c r="G33" s="1"/>
       <c r="H33" s="1" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="I33" s="1" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="J33" s="1" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="K33" s="1"/>
       <c r="L33" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.35">
@@ -2470,7 +2521,7 @@
         <v>35</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="D34" s="1">
         <v>0.5</v>
@@ -2482,14 +2533,14 @@
       <c r="G34" s="1"/>
       <c r="H34" s="1"/>
       <c r="I34" s="1" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="K34" s="1"/>
       <c r="L34" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.35">
@@ -2500,7 +2551,7 @@
         <v>35</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="D35" s="1">
         <v>0.35</v>
@@ -2512,14 +2563,14 @@
       <c r="G35" s="1"/>
       <c r="H35" s="1"/>
       <c r="I35" s="1" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="K35" s="1"/>
       <c r="L35" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.35">
@@ -2530,7 +2581,7 @@
         <v>35</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>40</v>
@@ -2542,14 +2593,14 @@
       <c r="G36" s="1"/>
       <c r="H36" s="1"/>
       <c r="I36" s="1" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="J36" s="1" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="K36" s="1"/>
       <c r="L36" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="37" spans="1:12" ht="29" x14ac:dyDescent="0.35">
@@ -2560,9 +2611,9 @@
         <v>35</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D37" s="7">
+        <v>115</v>
+      </c>
+      <c r="D37" s="6">
         <v>0.4236007</v>
       </c>
       <c r="E37" s="1">
@@ -2571,17 +2622,17 @@
       <c r="F37" s="1"/>
       <c r="G37" s="1"/>
       <c r="H37" s="1" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="J37" s="1" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="K37" s="1"/>
       <c r="L37" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="38" spans="1:12" ht="29" x14ac:dyDescent="0.35">
@@ -2592,9 +2643,9 @@
         <v>35</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D38" s="7">
+        <v>115</v>
+      </c>
+      <c r="D38" s="6">
         <v>0.4236007</v>
       </c>
       <c r="E38" s="1">
@@ -2603,17 +2654,17 @@
       <c r="F38" s="1"/>
       <c r="G38" s="1"/>
       <c r="H38" s="1" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="I38" s="1" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="J38" s="1" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="K38" s="1"/>
       <c r="L38" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.35">
@@ -2624,7 +2675,7 @@
         <v>43</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="D39" s="1">
         <v>12</v>
@@ -2639,11 +2690,11 @@
       </c>
       <c r="I39" s="1"/>
       <c r="J39" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="K39" s="1"/>
       <c r="L39" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.35">
@@ -2654,7 +2705,7 @@
         <v>43</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="D40" s="1">
         <v>20</v>
@@ -2669,11 +2720,11 @@
       </c>
       <c r="I40" s="1"/>
       <c r="J40" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="K40" s="1"/>
       <c r="L40" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="41" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
@@ -2684,7 +2735,7 @@
         <v>43</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="D41" s="1">
         <v>0.2</v>
@@ -2699,11 +2750,11 @@
       </c>
       <c r="I41" s="1"/>
       <c r="J41" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="K41" s="1"/>
       <c r="L41" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="42" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
@@ -2714,7 +2765,7 @@
         <v>43</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="D42" s="1">
         <v>0.1</v>
@@ -2729,11 +2780,11 @@
       </c>
       <c r="I42" s="1"/>
       <c r="J42" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="K42" s="1"/>
       <c r="L42" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.35">
@@ -2744,7 +2795,7 @@
         <v>43</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="D43" s="1">
         <v>0.45</v>
@@ -2759,11 +2810,11 @@
       </c>
       <c r="I43" s="1"/>
       <c r="J43" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="K43" s="1"/>
       <c r="L43" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.35">
@@ -2774,7 +2825,7 @@
         <v>43</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="D44" s="1">
         <v>0.22</v>
@@ -2789,11 +2840,11 @@
       </c>
       <c r="I44" s="1"/>
       <c r="J44" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="K44" s="1"/>
       <c r="L44" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.35">
@@ -2804,7 +2855,7 @@
         <v>43</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="D45" s="1">
         <v>0.21</v>
@@ -2816,15 +2867,15 @@
       <c r="F45" s="1"/>
       <c r="G45" s="1"/>
       <c r="H45" s="1" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="I45" s="1"/>
       <c r="J45" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="K45" s="1"/>
       <c r="L45" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.35">
@@ -2835,7 +2886,7 @@
         <v>43</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="D46" s="1">
         <v>212</v>
@@ -2850,15 +2901,15 @@
         <v>290</v>
       </c>
       <c r="H46" s="1" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="I46" s="1"/>
       <c r="J46" s="1" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="K46" s="1"/>
       <c r="L46" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.35">
@@ -2869,7 +2920,7 @@
         <v>43</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="D47" s="1">
         <v>1428</v>
@@ -2884,15 +2935,15 @@
         <v>1481</v>
       </c>
       <c r="H47" s="1" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="I47" s="1"/>
       <c r="J47" s="1" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="K47" s="1"/>
       <c r="L47" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.35">
@@ -2912,15 +2963,15 @@
       <c r="F48" s="1"/>
       <c r="G48" s="1"/>
       <c r="H48" s="3" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="I48" s="3"/>
       <c r="J48" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="K48" s="1"/>
       <c r="L48" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.35">
@@ -2931,7 +2982,7 @@
         <v>43</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="D49" s="1">
         <v>880</v>
@@ -2946,15 +2997,15 @@
         <v>960</v>
       </c>
       <c r="H49" s="3" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="I49" s="3"/>
       <c r="J49" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="K49" s="1"/>
       <c r="L49" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="50" spans="1:12" ht="29" x14ac:dyDescent="0.35">
@@ -2965,7 +3016,7 @@
         <v>43</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="D50" s="1">
         <v>5.7999999999999996E-3</v>
@@ -2980,11 +3031,11 @@
       </c>
       <c r="I50" s="1"/>
       <c r="J50" s="1" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="K50" s="1"/>
       <c r="L50" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="51" spans="1:12" ht="29" x14ac:dyDescent="0.35">
@@ -2995,7 +3046,7 @@
         <v>43</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="D51" s="1">
         <v>0.50930200000000003</v>
@@ -3010,11 +3061,11 @@
       </c>
       <c r="I51" s="1"/>
       <c r="J51" s="1" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="K51" s="1"/>
       <c r="L51" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="52" spans="1:12" ht="29" x14ac:dyDescent="0.35">
@@ -3025,7 +3076,7 @@
         <v>43</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="D52" s="1">
         <v>0.35</v>
@@ -3040,11 +3091,11 @@
       </c>
       <c r="I52" s="1"/>
       <c r="J52" s="1" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="K52" s="1"/>
       <c r="L52" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="53" spans="1:12" ht="29" x14ac:dyDescent="0.35">
@@ -3055,7 +3106,7 @@
         <v>43</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="D53" s="2" t="s">
         <v>48</v>
@@ -3070,11 +3121,11 @@
       </c>
       <c r="I53" s="1"/>
       <c r="J53" s="1" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="K53" s="1"/>
       <c r="L53" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="54" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
@@ -3085,7 +3136,7 @@
         <v>43</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="D54" s="1">
         <v>10.204700000000001</v>
@@ -3096,15 +3147,15 @@
       <c r="F54" s="1"/>
       <c r="G54" s="1"/>
       <c r="H54" s="1" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
       <c r="I54" s="1"/>
       <c r="J54" s="1" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="K54" s="1"/>
       <c r="L54" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="55" spans="1:12" ht="29" x14ac:dyDescent="0.35">
@@ -3115,7 +3166,7 @@
         <v>43</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="D55" s="1">
         <v>10.204700000000001</v>
@@ -3126,77 +3177,85 @@
       <c r="F55" s="1"/>
       <c r="G55" s="1"/>
       <c r="H55" s="1" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="I55" s="1" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="J55" s="1" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="K55" s="1"/>
       <c r="L55" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.35">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="D56" s="1">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E56" s="1">
-        <v>2.4</v>
-      </c>
-      <c r="F56" s="1"/>
-      <c r="G56" s="1"/>
-      <c r="H56" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="I56" s="1"/>
+        <v>20</v>
+      </c>
+      <c r="F56" s="7">
+        <v>-2.7</v>
+      </c>
+      <c r="G56" s="7">
+        <v>26.6</v>
+      </c>
+      <c r="H56" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="I56" s="1" t="s">
+        <v>75</v>
+      </c>
       <c r="J56" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="K56" s="1"/>
       <c r="L56" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.35">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="D57" s="1">
-        <v>20</v>
-      </c>
-      <c r="E57" s="1">
-        <v>4</v>
-      </c>
-      <c r="F57" s="1"/>
-      <c r="G57" s="1"/>
-      <c r="H57" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="I57" s="1"/>
+        <v>113</v>
+      </c>
+      <c r="D57" s="9">
+        <v>26</v>
+      </c>
+      <c r="E57" s="9">
+        <v>52</v>
+      </c>
+      <c r="F57" s="7"/>
+      <c r="G57" s="7"/>
+      <c r="H57" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="I57" s="1" t="s">
+        <v>75</v>
+      </c>
       <c r="J57" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="K57" s="1"/>
       <c r="L57" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="58" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
@@ -3204,29 +3263,35 @@
         <v>13</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="D58" s="1">
+        <v>0.3</v>
+      </c>
+      <c r="E58" s="1">
+        <v>0.6</v>
+      </c>
+      <c r="F58" s="7">
+        <v>0.15</v>
+      </c>
+      <c r="G58" s="7">
         <v>0.2</v>
       </c>
-      <c r="E58" s="1">
-        <v>0.04</v>
-      </c>
-      <c r="F58" s="1"/>
-      <c r="G58" s="1"/>
-      <c r="H58" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="I58" s="1"/>
+      <c r="H58" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="I58" s="1" t="s">
+        <v>75</v>
+      </c>
       <c r="J58" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="K58" s="1"/>
       <c r="L58" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="59" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
@@ -3234,59 +3299,71 @@
         <v>14</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="D59" s="1">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="E59" s="1">
-        <v>0.02</v>
-      </c>
-      <c r="F59" s="1"/>
-      <c r="G59" s="1"/>
-      <c r="H59" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="I59" s="1"/>
+        <v>0.3</v>
+      </c>
+      <c r="F59" s="7">
+        <v>0.05</v>
+      </c>
+      <c r="G59" s="7">
+        <v>0.2</v>
+      </c>
+      <c r="H59" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="I59" s="1" t="s">
+        <v>75</v>
+      </c>
       <c r="J59" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="K59" s="1"/>
       <c r="L59" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.35">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12" ht="58" x14ac:dyDescent="0.35">
       <c r="A60" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="D60" s="1">
-        <v>0.45</v>
+        <v>70</v>
       </c>
       <c r="E60" s="1">
-        <v>0.05</v>
-      </c>
-      <c r="F60" s="1"/>
-      <c r="G60" s="1"/>
-      <c r="H60" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="I60" s="1"/>
+        <v>140</v>
+      </c>
+      <c r="F60" s="7">
+        <v>80</v>
+      </c>
+      <c r="G60" s="7">
+        <v>100</v>
+      </c>
+      <c r="H60" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="I60" s="1" t="s">
+        <v>75</v>
+      </c>
       <c r="J60" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="K60" s="1"/>
       <c r="L60" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="61" spans="1:12" x14ac:dyDescent="0.35">
@@ -3294,60 +3371,67 @@
         <v>16</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="D61" s="1">
-        <v>0.22</v>
+        <v>0.4</v>
       </c>
       <c r="E61" s="1">
-        <v>3.5000000000000003E-2</v>
-      </c>
-      <c r="F61" s="1"/>
-      <c r="G61" s="1"/>
-      <c r="H61" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="I61" s="1"/>
+        <v>0.8</v>
+      </c>
+      <c r="F61" s="7">
+        <v>0.25</v>
+      </c>
+      <c r="G61" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="H61" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="I61" s="1" t="s">
+        <v>75</v>
+      </c>
       <c r="J61" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="K61" s="1"/>
       <c r="L61" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.35">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="62" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A62" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="D62" s="1">
-        <v>0.21</v>
+        <v>0.2</v>
       </c>
       <c r="E62" s="1">
-        <f>0.02</f>
-        <v>0.02</v>
-      </c>
-      <c r="F62" s="1"/>
-      <c r="G62" s="1"/>
-      <c r="H62" s="1" t="s">
+        <v>0.4</v>
+      </c>
+      <c r="F62" s="7"/>
+      <c r="G62" s="7"/>
+      <c r="H62" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="I62" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="I62" s="1"/>
       <c r="J62" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="K62" s="1"/>
       <c r="L62" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="63" spans="1:12" x14ac:dyDescent="0.35">
@@ -3355,33 +3439,35 @@
         <v>18</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="D63" s="1">
-        <v>212</v>
-      </c>
-      <c r="E63" s="1">
-        <v>157</v>
-      </c>
-      <c r="F63" s="1">
-        <v>77</v>
-      </c>
-      <c r="G63" s="1">
-        <v>290</v>
-      </c>
-      <c r="H63" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="I63" s="1"/>
+        <v>116</v>
+      </c>
+      <c r="D63" s="7">
+        <v>433.83</v>
+      </c>
+      <c r="E63" s="7">
+        <v>210.79</v>
+      </c>
+      <c r="F63" s="7">
+        <v>124.2</v>
+      </c>
+      <c r="G63" s="7">
+        <v>905.48</v>
+      </c>
+      <c r="H63" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="I63" s="1" t="s">
+        <v>75</v>
+      </c>
       <c r="J63" s="1" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="K63" s="1"/>
       <c r="L63" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.35">
@@ -3389,61 +3475,65 @@
         <v>19</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="D64" s="1">
-        <v>1428</v>
+        <v>0</v>
       </c>
       <c r="E64" s="1">
-        <v>114</v>
-      </c>
-      <c r="F64" s="1">
-        <v>1335</v>
-      </c>
-      <c r="G64" s="1">
-        <v>1481</v>
-      </c>
-      <c r="H64" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="I64" s="1"/>
+        <v>0</v>
+      </c>
+      <c r="F64" s="7"/>
+      <c r="G64" s="7"/>
+      <c r="H64" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="I64" s="1" t="s">
+        <v>75</v>
+      </c>
       <c r="J64" s="1" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="K64" s="1"/>
       <c r="L64" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.35">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="65" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A65" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C65" s="1"/>
-      <c r="D65" s="1">
-        <v>6</v>
-      </c>
-      <c r="E65" s="1">
-        <v>0.06</v>
-      </c>
-      <c r="F65" s="1"/>
-      <c r="G65" s="1"/>
-      <c r="H65" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="I65" s="3"/>
+      <c r="D65" s="7">
+        <v>7</v>
+      </c>
+      <c r="E65" s="7">
+        <v>14</v>
+      </c>
+      <c r="F65" s="7">
+        <v>5</v>
+      </c>
+      <c r="G65" s="7">
+        <v>9</v>
+      </c>
+      <c r="H65" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="I65" s="1" t="s">
+        <v>75</v>
+      </c>
       <c r="J65" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="K65" s="1"/>
       <c r="L65" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="66" spans="1:12" x14ac:dyDescent="0.35">
@@ -3451,905 +3541,254 @@
         <v>21</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="D66" s="1">
-        <v>880</v>
-      </c>
-      <c r="E66" s="1">
-        <v>70</v>
-      </c>
-      <c r="F66" s="1">
-        <v>810</v>
-      </c>
-      <c r="G66" s="1">
-        <v>960</v>
-      </c>
-      <c r="H66" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="I66" s="3"/>
+        <v>117</v>
+      </c>
+      <c r="D66" s="7">
+        <v>1410</v>
+      </c>
+      <c r="E66" s="7">
+        <v>2820</v>
+      </c>
+      <c r="F66" s="7">
+        <v>1370</v>
+      </c>
+      <c r="G66" s="7">
+        <v>1450</v>
+      </c>
+      <c r="H66" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="I66" s="1" t="s">
+        <v>75</v>
+      </c>
       <c r="J66" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="K66" s="1"/>
       <c r="L66" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="67" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="67" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A67" s="1" t="s">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="D67" s="1">
-        <v>5.7999999999999996E-3</v>
-      </c>
-      <c r="E67" s="1">
-        <v>3.3999999999999998E-3</v>
-      </c>
-      <c r="F67" s="1"/>
-      <c r="G67" s="1"/>
-      <c r="H67" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="I67" s="1"/>
+        <v>118</v>
+      </c>
+      <c r="D67" s="10">
+        <v>1.384623481E-3</v>
+      </c>
+      <c r="E67" s="10">
+        <v>5.4402432010000005E-4</v>
+      </c>
+      <c r="F67" s="10">
+        <v>7.1040402530000003E-4</v>
+      </c>
+      <c r="G67" s="10">
+        <v>1.936006955E-3</v>
+      </c>
+      <c r="H67" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="I67" s="1" t="s">
+        <v>75</v>
+      </c>
       <c r="J67" s="1" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="K67" s="1"/>
       <c r="L67" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="68" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="68" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A68" s="1" t="s">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D68" s="1">
-        <v>0.50930200000000003</v>
-      </c>
-      <c r="E68" s="1">
-        <v>2.9389999999999999E-2</v>
-      </c>
-      <c r="F68" s="1"/>
-      <c r="G68" s="1"/>
-      <c r="H68" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="I68" s="1"/>
+        <v>115</v>
+      </c>
+      <c r="D68" s="7">
+        <v>1.8181818181818181E-2</v>
+      </c>
+      <c r="E68" s="7">
+        <v>3.6363636363636362E-2</v>
+      </c>
+      <c r="F68" s="7"/>
+      <c r="G68" s="7"/>
+      <c r="H68" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="I68" s="1" t="s">
+        <v>74</v>
+      </c>
       <c r="J68" s="1" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="K68" s="1"/>
       <c r="L68" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="69" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="69" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A69" s="1" t="s">
-        <v>38</v>
+        <v>54</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="D69" s="1">
-        <v>0.35</v>
-      </c>
-      <c r="E69" s="1">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="F69" s="1"/>
-      <c r="G69" s="1"/>
+        <v>0.5</v>
+      </c>
+      <c r="E69" s="7">
+        <v>0</v>
+      </c>
+      <c r="F69" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="G69" s="7">
+        <v>0.5</v>
+      </c>
       <c r="H69" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="I69" s="1"/>
+        <v>145</v>
+      </c>
+      <c r="I69" s="1" t="s">
+        <v>73</v>
+      </c>
       <c r="J69" s="1" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="K69" s="1"/>
       <c r="L69" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="70" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="70" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A70" s="1" t="s">
-        <v>39</v>
+        <v>55</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C70" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="D70" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E70" s="1">
-        <v>0</v>
-      </c>
-      <c r="F70" s="1"/>
-      <c r="G70" s="1"/>
+        <v>51</v>
+      </c>
+      <c r="C70" s="1"/>
+      <c r="D70" s="1">
+        <v>0.37</v>
+      </c>
+      <c r="E70" s="7">
+        <v>0</v>
+      </c>
+      <c r="F70" s="7">
+        <v>0.37</v>
+      </c>
+      <c r="G70" s="7">
+        <v>0.37</v>
+      </c>
       <c r="H70" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="I70" s="1"/>
+        <v>145</v>
+      </c>
+      <c r="I70" s="1" t="s">
+        <v>73</v>
+      </c>
       <c r="J70" s="1" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="K70" s="1"/>
       <c r="L70" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="71" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A71" s="1" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D71" s="1">
-        <v>6.0100000000000001E-2</v>
+        <v>120</v>
+      </c>
+      <c r="D71" s="4">
+        <v>2.7399999999999999E-5</v>
       </c>
       <c r="E71" s="1">
-        <v>1.2E-2</v>
-      </c>
-      <c r="F71" s="1"/>
-      <c r="G71" s="1"/>
-      <c r="H71" s="1"/>
-      <c r="I71" s="1"/>
+        <v>5.4799999999999997E-5</v>
+      </c>
+      <c r="F71" s="7"/>
+      <c r="G71" s="7"/>
+      <c r="H71" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="I71" s="1" t="s">
+        <v>73</v>
+      </c>
       <c r="J71" s="1" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="K71" s="1"/>
       <c r="L71" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="72" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A72" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C72" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="D72" s="4">
+        <v>1.2999999999999999E-5</v>
+      </c>
+      <c r="E72" s="1">
+        <v>2.5999999999999998E-5</v>
+      </c>
+      <c r="F72" s="7"/>
+      <c r="G72" s="7"/>
+      <c r="H72" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="I72" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="J72" s="1" t="s">
         <v>66</v>
-      </c>
-    </row>
-    <row r="72" spans="1:12" ht="29" x14ac:dyDescent="0.35">
-      <c r="A72" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="B72" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C72" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D72" s="1">
-        <v>6.0100000000000001E-2</v>
-      </c>
-      <c r="E72" s="1">
-        <v>1.2E-2</v>
-      </c>
-      <c r="F72" s="1"/>
-      <c r="G72" s="1"/>
-      <c r="H72" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="I72" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="J72" s="1" t="s">
-        <v>71</v>
       </c>
       <c r="K72" s="1"/>
       <c r="L72" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="73" spans="1:12" ht="29" x14ac:dyDescent="0.35">
-      <c r="A73" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="B73" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C73" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="D73" s="1">
-        <v>5.1000000000000004E-3</v>
-      </c>
-      <c r="E73" s="1">
-        <v>1E-3</v>
-      </c>
-      <c r="F73" s="1"/>
-      <c r="G73" s="1"/>
-      <c r="H73" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="I73" s="1"/>
-      <c r="J73" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="K73" s="1"/>
-      <c r="L73" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="74" spans="1:12" ht="29" x14ac:dyDescent="0.35">
-      <c r="A74" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B74" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C74" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D74" s="1">
-        <v>0.6</v>
-      </c>
-      <c r="E74" s="1">
-        <v>0.12</v>
-      </c>
-      <c r="F74" s="1"/>
-      <c r="G74" s="1"/>
-      <c r="H74" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="I74" s="1"/>
-      <c r="J74" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="K74" s="1"/>
-      <c r="L74" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="75" spans="1:12" ht="29" x14ac:dyDescent="0.35">
-      <c r="A75" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="B75" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C75" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D75" s="1">
-        <v>0.35</v>
-      </c>
-      <c r="E75" s="1">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="F75" s="1"/>
-      <c r="G75" s="1"/>
-      <c r="H75" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="I75" s="1"/>
-      <c r="J75" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="K75" s="1"/>
-      <c r="L75" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="76" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A76" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="B76" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C76" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="D76" s="1">
-        <v>1.6799999999999999E-2</v>
-      </c>
-      <c r="E76" s="1">
-        <v>3.3999999999999998E-3</v>
-      </c>
-      <c r="F76" s="1"/>
-      <c r="G76" s="1"/>
-      <c r="H76" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="I76" s="1"/>
-      <c r="J76" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="K76" s="1"/>
-      <c r="L76" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="77" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A77" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B77" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C77" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="D77" s="1">
-        <v>10</v>
-      </c>
-      <c r="E77" s="1">
-        <f>Table1[[#This Row],[Value]]*2</f>
-        <v>20</v>
-      </c>
-      <c r="F77" s="1"/>
-      <c r="G77" s="1"/>
-      <c r="H77" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="I77" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="J77" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="K77" s="1"/>
-      <c r="L77" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="78" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A78" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B78" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C78" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="D78" s="1">
-        <v>26</v>
-      </c>
-      <c r="E78" s="1">
-        <f>Table1[[#This Row],[Value]]*2</f>
-        <v>52</v>
-      </c>
-      <c r="F78" s="1"/>
-      <c r="G78" s="1"/>
-      <c r="H78" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="I78" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="J78" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="K78" s="1"/>
-      <c r="L78" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="79" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A79" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B79" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C79" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="D79" s="1">
-        <v>0.3</v>
-      </c>
-      <c r="E79" s="1">
-        <f>Table1[[#This Row],[Value]]*2</f>
-        <v>0.6</v>
-      </c>
-      <c r="F79" s="1"/>
-      <c r="G79" s="1"/>
-      <c r="H79" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="I79" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="J79" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="K79" s="1"/>
-      <c r="L79" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="80" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A80" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B80" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C80" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="D80" s="1">
-        <v>0.15</v>
-      </c>
-      <c r="E80" s="1">
-        <f>Table1[[#This Row],[Value]]*2</f>
-        <v>0.3</v>
-      </c>
-      <c r="F80" s="1"/>
-      <c r="G80" s="1"/>
-      <c r="H80" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="I80" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="J80" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="K80" s="1"/>
-      <c r="L80" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="81" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A81" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B81" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C81" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="D81" s="1">
-        <v>70</v>
-      </c>
-      <c r="E81" s="1">
-        <f>Table1[[#This Row],[Value]]*2</f>
-        <v>140</v>
-      </c>
-      <c r="F81" s="1"/>
-      <c r="G81" s="1"/>
-      <c r="H81" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="I81" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="J81" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="K81" s="1"/>
-      <c r="L81" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="82" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A82" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B82" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C82" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D82" s="1">
-        <v>0.4</v>
-      </c>
-      <c r="E82" s="1">
-        <f>Table1[[#This Row],[Value]]*2</f>
-        <v>0.8</v>
-      </c>
-      <c r="F82" s="1"/>
-      <c r="G82" s="1"/>
-      <c r="H82" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="I82" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="J82" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="K82" s="1"/>
-      <c r="L82" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="83" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A83" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B83" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C83" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D83" s="1">
-        <v>0.2</v>
-      </c>
-      <c r="E83" s="1">
-        <f>Table1[[#This Row],[Value]]*2</f>
-        <v>0.4</v>
-      </c>
-      <c r="F83" s="1"/>
-      <c r="G83" s="1"/>
-      <c r="H83" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="I83" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="J83" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="K83" s="1"/>
-      <c r="L83" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="84" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A84" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B84" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C84" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="D84" s="1">
-        <v>433</v>
-      </c>
-      <c r="E84" s="1">
-        <f>Table1[[#This Row],[Value]]*2</f>
-        <v>866</v>
-      </c>
-      <c r="F84" s="1"/>
-      <c r="G84" s="1"/>
-      <c r="H84" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="I84" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="J84" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="K84" s="1"/>
-      <c r="L84" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="85" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A85" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="B85" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C85" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="D85" s="1">
-        <v>0</v>
-      </c>
-      <c r="E85" s="1">
-        <f>Table1[[#This Row],[Value]]*2</f>
-        <v>0</v>
-      </c>
-      <c r="F85" s="1"/>
-      <c r="G85" s="1"/>
-      <c r="H85" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="I85" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="J85" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="K85" s="1"/>
-      <c r="L85" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="86" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A86" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B86" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C86" s="1"/>
-      <c r="D86" s="1">
-        <v>6</v>
-      </c>
-      <c r="E86" s="1">
-        <f>Table1[[#This Row],[Value]]*2</f>
-        <v>12</v>
-      </c>
-      <c r="F86" s="1"/>
-      <c r="G86" s="1"/>
-      <c r="H86" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="I86" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="J86" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="K86" s="1"/>
-      <c r="L86" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="87" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A87" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B87" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C87" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="D87" s="1">
-        <v>1300</v>
-      </c>
-      <c r="E87" s="1">
-        <f>Table1[[#This Row],[Value]]*2</f>
-        <v>2600</v>
-      </c>
-      <c r="F87" s="1"/>
-      <c r="G87" s="1"/>
-      <c r="H87" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="I87" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="J87" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="K87" s="1"/>
-      <c r="L87" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="88" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A88" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="B88" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C88" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="D88" s="1">
-        <v>0.02</v>
-      </c>
-      <c r="E88" s="1">
-        <f>Table1[[#This Row],[Value]]*2</f>
-        <v>0.04</v>
-      </c>
-      <c r="F88" s="1"/>
-      <c r="G88" s="1"/>
-      <c r="H88" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="I88" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="J88" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="K88" s="1"/>
-      <c r="L88" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="89" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A89" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="B89" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C89" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D89" s="1">
-        <f>1/36</f>
-        <v>2.7777777777777776E-2</v>
-      </c>
-      <c r="E89" s="1">
-        <f>Table1[[#This Row],[Value]]*2</f>
-        <v>5.5555555555555552E-2</v>
-      </c>
-      <c r="F89" s="1"/>
-      <c r="G89" s="1"/>
-      <c r="H89" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="I89" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="J89" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="K89" s="1"/>
-      <c r="L89" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="90" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A90" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="B90" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C90" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D90" s="1">
-        <v>0.5</v>
-      </c>
-      <c r="E90" s="1">
-        <f>Table1[[#This Row],[Value]]*2</f>
-        <v>1</v>
-      </c>
-      <c r="F90" s="1"/>
-      <c r="G90" s="1"/>
-      <c r="H90" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="I90" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="J90" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="K90" s="1"/>
-      <c r="L90" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="91" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A91" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="B91" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C91" s="1"/>
-      <c r="D91" s="1">
-        <v>0.37</v>
-      </c>
-      <c r="E91" s="1">
-        <f>Table1[[#This Row],[Value]]*2</f>
-        <v>0.74</v>
-      </c>
-      <c r="F91" s="1"/>
-      <c r="G91" s="1"/>
-      <c r="H91" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="I91" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="J91" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="K91" s="1"/>
-      <c r="L91" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="92" spans="1:12" ht="29" x14ac:dyDescent="0.35">
-      <c r="A92" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="B92" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C92" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="D92" s="5">
-        <v>2.7399999999999999E-5</v>
-      </c>
-      <c r="E92" s="1">
-        <f>Table1[[#This Row],[Value]]*2</f>
-        <v>5.4799999999999997E-5</v>
-      </c>
-      <c r="F92" s="1"/>
-      <c r="G92" s="1"/>
-      <c r="H92" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="I92" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="J92" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="K92" s="1"/>
-      <c r="L92" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="93" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A93" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="B93" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C93" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="D93" s="5">
-        <v>1.2999999999999999E-5</v>
-      </c>
-      <c r="E93" s="1">
-        <f>Table1[[#This Row],[Value]]*2</f>
-        <v>2.5999999999999998E-5</v>
-      </c>
-      <c r="F93" s="1"/>
-      <c r="G93" s="1"/>
-      <c r="H93" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="I93" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="J93" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="K93" s="1"/>
-      <c r="L93" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="H56" r:id="rId1" display="https://kpbs.konza.k-state.edu/location/" xr:uid="{98608C20-26EF-4289-9EC6-968CD5323926}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA0710C0-AB94-4FBF-AB29-E5085BC4F559}">
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.7265625" customWidth="1"/>
@@ -4361,27 +3800,27 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="D1" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="E1" t="s">
         <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="B2" t="s">
         <v>34</v>
@@ -4394,15 +3833,15 @@
         <v>6.45</v>
       </c>
       <c r="E2" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="F2" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="B3" t="s">
         <v>35</v>
@@ -4415,15 +3854,15 @@
         <v>1.875</v>
       </c>
       <c r="E3" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="F3" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="B4" t="s">
         <v>43</v>
@@ -4435,370 +3874,350 @@
         <v>0.1</v>
       </c>
       <c r="E4" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="F4" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="B5" t="s">
         <v>50</v>
       </c>
       <c r="C5" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D5">
         <v>0.1</v>
       </c>
       <c r="E5" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="F5" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="B6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C6" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D6">
         <v>0.1</v>
       </c>
       <c r="E6" t="s">
-        <v>107</v>
+        <v>98</v>
       </c>
       <c r="F6" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="B7" t="s">
-        <v>56</v>
+        <v>80</v>
       </c>
       <c r="C7" t="s">
-        <v>8</v>
+        <v>94</v>
       </c>
       <c r="D7">
-        <v>0.1</v>
+        <v>200</v>
       </c>
       <c r="E7" t="s">
-        <v>106</v>
+        <v>97</v>
       </c>
       <c r="F7" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="B8" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="C8" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="D8">
         <v>200</v>
       </c>
       <c r="E8" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="F8" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="B9" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="C9" t="s">
-        <v>103</v>
+        <v>81</v>
       </c>
       <c r="D9">
-        <v>200</v>
+        <v>750</v>
       </c>
       <c r="E9" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="F9" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="B10" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="C10" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="D10">
-        <v>750</v>
+        <v>6750</v>
       </c>
       <c r="E10" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="F10" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="B11" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="C11" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="D11">
-        <v>6750</v>
+        <v>2500</v>
       </c>
       <c r="E11" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="F11" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="B12" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="C12" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="D12">
-        <v>2500</v>
+        <v>200</v>
       </c>
       <c r="E12" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="F12" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="B13" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="C13" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="D13">
-        <v>200</v>
+        <v>1000</v>
       </c>
       <c r="E13" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="F13" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="B14" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="C14" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="D14">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="E14" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="F14" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="B15" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="C15" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="D15">
-        <v>2000</v>
+        <v>10</v>
       </c>
       <c r="E15" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="F15" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="B16" t="s">
+        <v>80</v>
+      </c>
+      <c r="C16" t="s">
         <v>88</v>
       </c>
-      <c r="C16" t="s">
-        <v>95</v>
-      </c>
       <c r="D16">
-        <v>10</v>
+        <v>0.1</v>
       </c>
       <c r="E16" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="F16" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="B17" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="C17" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="D17">
-        <v>0.1</v>
+        <v>400</v>
       </c>
       <c r="E17" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="F17" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="B18" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="C18" t="s">
+        <v>90</v>
+      </c>
+      <c r="D18">
+        <v>10</v>
+      </c>
+      <c r="E18" t="s">
         <v>97</v>
       </c>
-      <c r="D18">
-        <v>400</v>
-      </c>
-      <c r="E18" t="s">
-        <v>105</v>
-      </c>
       <c r="F18" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="B19" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="C19" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="D19">
-        <v>10</v>
+        <v>1000</v>
       </c>
       <c r="E19" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="F19" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="B20" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="C20" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="D20">
-        <v>1000</v>
+        <v>3000</v>
       </c>
       <c r="E20" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="F20" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="B21" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="C21" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="D21">
-        <v>3000</v>
+        <v>40</v>
       </c>
       <c r="E21" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="F21" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
-        <v>104</v>
-      </c>
-      <c r="B22" t="s">
-        <v>88</v>
-      </c>
-      <c r="C22" t="s">
-        <v>101</v>
-      </c>
-      <c r="D22">
-        <v>40</v>
-      </c>
-      <c r="E22" t="s">
-        <v>105</v>
-      </c>
-      <c r="F22" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -4808,7 +4227,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC182590-26D0-4168-8E7C-B448CD67FE47}">
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.7265625" bestFit="1" customWidth="1"/>
@@ -4817,13 +4236,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
@@ -5029,10 +4448,10 @@
         <v>5</v>
       </c>
       <c r="B20" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C20">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.35">
@@ -5040,7 +4459,7 @@
         <v>6</v>
       </c>
       <c r="B21" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C21">
         <v>1</v>
@@ -5051,7 +4470,7 @@
         <v>7</v>
       </c>
       <c r="B22" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C22">
         <v>0</v>
@@ -5062,10 +4481,10 @@
         <v>8</v>
       </c>
       <c r="B23" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C23">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.35">
@@ -5073,10 +4492,10 @@
         <v>9</v>
       </c>
       <c r="B24" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C24">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.35">
@@ -5084,75 +4503,9 @@
         <v>10</v>
       </c>
       <c r="B25" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C25">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
-        <v>5</v>
-      </c>
-      <c r="B26" t="s">
-        <v>56</v>
-      </c>
-      <c r="C26">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
-        <v>6</v>
-      </c>
-      <c r="B27" t="s">
-        <v>56</v>
-      </c>
-      <c r="C27">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
-        <v>7</v>
-      </c>
-      <c r="B28" t="s">
-        <v>56</v>
-      </c>
-      <c r="C28">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
-        <v>8</v>
-      </c>
-      <c r="B29" t="s">
-        <v>56</v>
-      </c>
-      <c r="C29">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
-        <v>9</v>
-      </c>
-      <c r="B30" t="s">
-        <v>56</v>
-      </c>
-      <c r="C30">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A31" t="s">
-        <v>10</v>
-      </c>
-      <c r="B31" t="s">
-        <v>56</v>
-      </c>
-      <c r="C31">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Reran the model with the latest parameter values from the updates that the team provided.
</commit_message>
<xml_diff>
--- a/Data/scenarios.xlsx
+++ b/Data/scenarios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rober\Documents\GitHub Repos\merging_SFW_decomposition_models\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58121FC9-7A10-4CEF-9D21-C059D2F07BA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B86018D-D56A-4987-822D-92A3E7138A29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{7C97690C-9E7B-4D0E-86C0-16835BCB4BB0}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="613" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="608" uniqueCount="145">
   <si>
     <t>Parameter</t>
   </si>
@@ -166,9 +166,6 @@
     <t>slope_pint_det_k_frag_organic</t>
   </si>
   <si>
-    <t>Mite</t>
-  </si>
-  <si>
     <t>climate-data.org (Murphy, NC)</t>
   </si>
   <si>
@@ -187,9 +184,6 @@
     <t>Adapted from calculatation conduct on empirical data provided by Seastedt et al. 1983 and Seastedt 1984</t>
   </si>
   <si>
-    <t>MitePredator</t>
-  </si>
-  <si>
     <t>RootHerbivore</t>
   </si>
   <si>
@@ -473,6 +467,9 @@
   </si>
   <si>
     <t>Barreto et al. 2024; these are percentages reported in suppl.</t>
+  </si>
+  <si>
+    <t>Microarthropod</t>
   </si>
 </sst>
 </file>
@@ -828,7 +825,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -943,6 +940,17 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -989,7 +997,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1018,6 +1026,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="19" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1480,7 +1491,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>2</v>
@@ -1489,25 +1500,25 @@
         <v>3</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.35">
@@ -1518,7 +1529,7 @@
         <v>34</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D2" s="1">
         <v>6</v>
@@ -1529,15 +1540,15 @@
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
       <c r="H2" s="1" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="I2" s="1"/>
       <c r="J2" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="K2" s="1"/>
       <c r="L2" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
@@ -1548,7 +1559,7 @@
         <v>34</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D3" s="1">
         <v>26</v>
@@ -1561,11 +1572,11 @@
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="K3" s="1"/>
       <c r="L3" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.35">
@@ -1576,7 +1587,7 @@
         <v>34</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D4" s="1">
         <v>0.3</v>
@@ -1589,11 +1600,11 @@
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="K4" s="1"/>
       <c r="L4" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
@@ -1604,7 +1615,7 @@
         <v>34</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D5" s="1">
         <v>0.15</v>
@@ -1617,11 +1628,11 @@
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
       <c r="J5" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="K5" s="1"/>
       <c r="L5" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.35">
@@ -1632,7 +1643,7 @@
         <v>34</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D6" s="1">
         <v>73</v>
@@ -1647,15 +1658,15 @@
         <v>78</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I6" s="1"/>
       <c r="J6" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="K6" s="1"/>
       <c r="L6" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.35">
@@ -1666,7 +1677,7 @@
         <v>34</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D7" s="1">
         <v>0.28000000000000003</v>
@@ -1681,15 +1692,15 @@
         <v>0.33</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I7" s="1"/>
       <c r="J7" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="K7" s="1"/>
       <c r="L7" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="29" x14ac:dyDescent="0.35">
@@ -1700,7 +1711,7 @@
         <v>34</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D8" s="1">
         <v>0.2</v>
@@ -1715,17 +1726,17 @@
         <v>0.3</v>
       </c>
       <c r="H8" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="K8" s="1"/>
       <c r="L8" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.35">
@@ -1736,7 +1747,7 @@
         <v>34</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D9" s="5">
         <f>D10*0.03</f>
@@ -1755,15 +1766,15 @@
         <v>17.920000000000002</v>
       </c>
       <c r="H9" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="I9" s="1"/>
       <c r="J9" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="K9" s="1"/>
       <c r="L9" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.35">
@@ -1774,7 +1785,7 @@
         <v>34</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D10" s="1">
         <f>336/0.75</f>
@@ -1793,15 +1804,15 @@
         <v>448</v>
       </c>
       <c r="H10" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="I10" s="1"/>
       <c r="J10" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="K10" s="1"/>
       <c r="L10" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.35">
@@ -1825,15 +1836,15 @@
         <v>8</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I11" s="1"/>
       <c r="J11" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="K11" s="1"/>
       <c r="L11" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="29" x14ac:dyDescent="0.35">
@@ -1844,7 +1855,7 @@
         <v>34</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D12" s="1">
         <v>700</v>
@@ -1859,15 +1870,15 @@
         <v>1160</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="I12" s="1"/>
       <c r="J12" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="K12" s="1"/>
       <c r="L12" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="29" x14ac:dyDescent="0.35">
@@ -1878,31 +1889,31 @@
         <v>34</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D13" s="1">
-        <f>0.217/365/6.45</f>
+        <f>0.217/365/state_variables_value!D2</f>
         <v>9.2173728363597747E-5</v>
       </c>
       <c r="E13" s="1"/>
       <c r="F13" s="1">
-        <f>0.217/365/6.45</f>
-        <v>9.2173728363597747E-5</v>
+        <f>0.217/365</f>
+        <v>5.9452054794520545E-4</v>
       </c>
       <c r="G13" s="1">
-        <f>0.0018/6.45</f>
-        <v>2.7906976744186045E-4</v>
+        <f>0.0018</f>
+        <v>1.8E-3</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="I13" s="1"/>
       <c r="J13" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="K13" s="1"/>
       <c r="L13" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.35">
@@ -1913,7 +1924,7 @@
         <v>34</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D14" s="1">
         <v>0.53</v>
@@ -1928,11 +1939,11 @@
       </c>
       <c r="I14" s="1"/>
       <c r="J14" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="K14" s="1"/>
       <c r="L14" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.35">
@@ -1943,7 +1954,7 @@
         <v>34</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D15" s="1">
         <v>0.09</v>
@@ -1958,11 +1969,11 @@
       </c>
       <c r="I15" s="1"/>
       <c r="J15" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="K15" s="1"/>
       <c r="L15" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.35">
@@ -1973,7 +1984,7 @@
         <v>34</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D16" s="1">
         <v>0.22</v>
@@ -1988,11 +1999,11 @@
       </c>
       <c r="I16" s="1"/>
       <c r="J16" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="K16" s="1"/>
       <c r="L16" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="17" spans="1:12" ht="29" x14ac:dyDescent="0.35">
@@ -2003,7 +2014,7 @@
         <v>34</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D17" s="4">
         <f>0.00207/0.0375</f>
@@ -2015,15 +2026,15 @@
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
       <c r="H17" s="1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="I17" s="1"/>
       <c r="J17" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="K17" s="1"/>
       <c r="L17" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="18" spans="1:12" ht="29" x14ac:dyDescent="0.35">
@@ -2034,7 +2045,7 @@
         <v>34</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D18" s="4">
         <f>0.00207/0.0375</f>
@@ -2046,15 +2057,15 @@
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
       <c r="H18" s="1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="I18" s="1"/>
       <c r="J18" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="K18" s="1"/>
       <c r="L18" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="19" spans="1:12" ht="29" x14ac:dyDescent="0.35">
@@ -2065,7 +2076,7 @@
         <v>34</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D19" s="4">
         <f>0.00207/0.0375</f>
@@ -2077,15 +2088,15 @@
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
       <c r="H19" s="1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="I19" s="1"/>
       <c r="J19" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="K19" s="1"/>
       <c r="L19" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="29" x14ac:dyDescent="0.35">
@@ -2096,7 +2107,7 @@
         <v>34</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D20" s="1">
         <v>0</v>
@@ -2108,14 +2119,14 @@
       <c r="G20" s="1"/>
       <c r="H20" s="1"/>
       <c r="I20" s="1" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="K20" s="1"/>
       <c r="L20" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="21" spans="1:12" ht="29" x14ac:dyDescent="0.35">
@@ -2126,7 +2137,7 @@
         <v>34</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D21" s="1">
         <v>-5.5040310000000002E-2</v>
@@ -2137,17 +2148,17 @@
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
       <c r="H21" s="1" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="K21" s="1"/>
       <c r="L21" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.35">
@@ -2158,7 +2169,7 @@
         <v>35</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D22" s="1">
         <v>6</v>
@@ -2170,14 +2181,14 @@
       <c r="G22" s="1"/>
       <c r="H22" s="1"/>
       <c r="I22" s="1" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="K22" s="1"/>
       <c r="L22" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.35">
@@ -2188,7 +2199,7 @@
         <v>35</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D23" s="1">
         <v>26</v>
@@ -2200,14 +2211,14 @@
       <c r="G23" s="1"/>
       <c r="H23" s="1"/>
       <c r="I23" s="1" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="K23" s="1"/>
       <c r="L23" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.35">
@@ -2218,7 +2229,7 @@
         <v>35</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D24" s="1">
         <v>0.3</v>
@@ -2230,14 +2241,14 @@
       <c r="G24" s="1"/>
       <c r="H24" s="1"/>
       <c r="I24" s="1" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="K24" s="1"/>
       <c r="L24" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.35">
@@ -2248,7 +2259,7 @@
         <v>35</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D25" s="1">
         <v>0.15</v>
@@ -2260,14 +2271,14 @@
       <c r="G25" s="1"/>
       <c r="H25" s="1"/>
       <c r="I25" s="1" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="K25" s="1"/>
       <c r="L25" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.35">
@@ -2278,7 +2289,7 @@
         <v>35</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D26" s="1">
         <v>70</v>
@@ -2290,14 +2301,14 @@
       <c r="G26" s="1"/>
       <c r="H26" s="1"/>
       <c r="I26" s="1" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="K26" s="1"/>
       <c r="L26" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.35">
@@ -2308,7 +2319,7 @@
         <v>35</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D27" s="1">
         <v>0.4</v>
@@ -2320,14 +2331,14 @@
       <c r="G27" s="1"/>
       <c r="H27" s="1"/>
       <c r="I27" s="1" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="K27" s="1"/>
       <c r="L27" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.35">
@@ -2338,7 +2349,7 @@
         <v>35</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D28" s="1">
         <v>0.2</v>
@@ -2350,14 +2361,14 @@
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
       <c r="I28" s="1" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="K28" s="1"/>
       <c r="L28" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.35">
@@ -2368,7 +2379,7 @@
         <v>35</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D29" s="1">
         <v>50</v>
@@ -2380,14 +2391,14 @@
       <c r="G29" s="1"/>
       <c r="H29" s="1"/>
       <c r="I29" s="1" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J29" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="K29" s="1"/>
       <c r="L29" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.35">
@@ -2398,7 +2409,7 @@
         <v>35</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D30" s="1">
         <v>1270</v>
@@ -2410,14 +2421,14 @@
       <c r="G30" s="1"/>
       <c r="H30" s="1"/>
       <c r="I30" s="1" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="K30" s="1"/>
       <c r="L30" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.35">
@@ -2437,17 +2448,17 @@
       <c r="F31" s="1"/>
       <c r="G31" s="1"/>
       <c r="H31" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="I31" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="I31" s="1" t="s">
-        <v>127</v>
-      </c>
       <c r="J31" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="K31" s="1"/>
       <c r="L31" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.35">
@@ -2458,7 +2469,7 @@
         <v>35</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D32" s="1">
         <v>1300</v>
@@ -2470,14 +2481,14 @@
       <c r="G32" s="1"/>
       <c r="H32" s="1"/>
       <c r="I32" s="1" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="K32" s="1"/>
       <c r="L32" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.35">
@@ -2488,11 +2499,11 @@
         <v>35</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D33" s="1">
-        <f>1/(2.5*365)</f>
-        <v>1.095890410958904E-3</v>
+        <f>1/(2.5*365*state_variables_value!D3)</f>
+        <v>5.8447488584474887E-4</v>
       </c>
       <c r="E33" s="1">
         <v>0</v>
@@ -2500,17 +2511,17 @@
       <c r="F33" s="1"/>
       <c r="G33" s="1"/>
       <c r="H33" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I33" s="1" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J33" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="K33" s="1"/>
       <c r="L33" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.35">
@@ -2521,7 +2532,7 @@
         <v>35</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D34" s="1">
         <v>0.5</v>
@@ -2533,14 +2544,14 @@
       <c r="G34" s="1"/>
       <c r="H34" s="1"/>
       <c r="I34" s="1" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="K34" s="1"/>
       <c r="L34" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.35">
@@ -2551,7 +2562,7 @@
         <v>35</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D35" s="1">
         <v>0.35</v>
@@ -2563,14 +2574,14 @@
       <c r="G35" s="1"/>
       <c r="H35" s="1"/>
       <c r="I35" s="1" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="K35" s="1"/>
       <c r="L35" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.35">
@@ -2581,7 +2592,7 @@
         <v>35</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>40</v>
@@ -2593,14 +2604,14 @@
       <c r="G36" s="1"/>
       <c r="H36" s="1"/>
       <c r="I36" s="1" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J36" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="K36" s="1"/>
       <c r="L36" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="37" spans="1:12" ht="29" x14ac:dyDescent="0.35">
@@ -2611,7 +2622,7 @@
         <v>35</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D37" s="6">
         <v>0.4236007</v>
@@ -2622,17 +2633,17 @@
       <c r="F37" s="1"/>
       <c r="G37" s="1"/>
       <c r="H37" s="1" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J37" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="K37" s="1"/>
       <c r="L37" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="38" spans="1:12" ht="29" x14ac:dyDescent="0.35">
@@ -2643,7 +2654,7 @@
         <v>35</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D38" s="6">
         <v>0.4236007</v>
@@ -2654,17 +2665,17 @@
       <c r="F38" s="1"/>
       <c r="G38" s="1"/>
       <c r="H38" s="1" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="I38" s="1" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J38" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="K38" s="1"/>
       <c r="L38" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.35">
@@ -2672,10 +2683,10 @@
         <v>11</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>43</v>
+        <v>144</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D39" s="1">
         <v>12</v>
@@ -2686,15 +2697,15 @@
       <c r="F39" s="1"/>
       <c r="G39" s="1"/>
       <c r="H39" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="I39" s="1"/>
       <c r="J39" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="K39" s="1"/>
       <c r="L39" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.35">
@@ -2702,10 +2713,10 @@
         <v>12</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>43</v>
+        <v>144</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D40" s="1">
         <v>20</v>
@@ -2716,15 +2727,15 @@
       <c r="F40" s="1"/>
       <c r="G40" s="1"/>
       <c r="H40" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="I40" s="1"/>
       <c r="J40" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="K40" s="1"/>
       <c r="L40" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="41" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
@@ -2732,10 +2743,10 @@
         <v>13</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>43</v>
+        <v>144</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D41" s="1">
         <v>0.2</v>
@@ -2746,15 +2757,15 @@
       <c r="F41" s="1"/>
       <c r="G41" s="1"/>
       <c r="H41" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="I41" s="1"/>
       <c r="J41" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="K41" s="1"/>
       <c r="L41" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="42" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
@@ -2762,10 +2773,10 @@
         <v>14</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>43</v>
+        <v>144</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D42" s="1">
         <v>0.1</v>
@@ -2776,15 +2787,15 @@
       <c r="F42" s="1"/>
       <c r="G42" s="1"/>
       <c r="H42" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="I42" s="1"/>
       <c r="J42" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="K42" s="1"/>
       <c r="L42" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.35">
@@ -2792,10 +2803,10 @@
         <v>15</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>43</v>
+        <v>144</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D43" s="1">
         <v>0.45</v>
@@ -2806,15 +2817,15 @@
       <c r="F43" s="1"/>
       <c r="G43" s="1"/>
       <c r="H43" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I43" s="1"/>
       <c r="J43" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="K43" s="1"/>
       <c r="L43" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.35">
@@ -2822,10 +2833,10 @@
         <v>16</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>43</v>
+        <v>144</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D44" s="1">
         <v>0.22</v>
@@ -2836,15 +2847,15 @@
       <c r="F44" s="1"/>
       <c r="G44" s="1"/>
       <c r="H44" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I44" s="1"/>
       <c r="J44" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="K44" s="1"/>
       <c r="L44" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.35">
@@ -2852,10 +2863,10 @@
         <v>17</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>43</v>
+        <v>144</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D45" s="1">
         <v>0.21</v>
@@ -2867,15 +2878,15 @@
       <c r="F45" s="1"/>
       <c r="G45" s="1"/>
       <c r="H45" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="I45" s="1"/>
       <c r="J45" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="K45" s="1"/>
       <c r="L45" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.35">
@@ -2883,10 +2894,10 @@
         <v>18</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>43</v>
+        <v>144</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D46" s="1">
         <v>212</v>
@@ -2901,15 +2912,15 @@
         <v>290</v>
       </c>
       <c r="H46" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I46" s="1"/>
       <c r="J46" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="K46" s="1"/>
       <c r="L46" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.35">
@@ -2917,10 +2928,10 @@
         <v>19</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>43</v>
+        <v>144</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D47" s="1">
         <v>1428</v>
@@ -2935,15 +2946,15 @@
         <v>1481</v>
       </c>
       <c r="H47" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I47" s="1"/>
       <c r="J47" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="K47" s="1"/>
       <c r="L47" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.35">
@@ -2951,7 +2962,7 @@
         <v>20</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>43</v>
+        <v>144</v>
       </c>
       <c r="C48" s="1"/>
       <c r="D48" s="1">
@@ -2963,15 +2974,15 @@
       <c r="F48" s="1"/>
       <c r="G48" s="1"/>
       <c r="H48" s="3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="I48" s="3"/>
       <c r="J48" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="K48" s="1"/>
       <c r="L48" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.35">
@@ -2979,10 +2990,10 @@
         <v>21</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>43</v>
+        <v>144</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D49" s="1">
         <v>880</v>
@@ -2997,15 +3008,15 @@
         <v>960</v>
       </c>
       <c r="H49" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="I49" s="3"/>
       <c r="J49" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="K49" s="1"/>
       <c r="L49" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="50" spans="1:12" ht="29" x14ac:dyDescent="0.35">
@@ -3013,13 +3024,14 @@
         <v>36</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>43</v>
+        <v>144</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D50" s="1">
-        <v>5.7999999999999996E-3</v>
+        <f>0.0058/state_variables_value!D4</f>
+        <v>5.7999999999999996E-2</v>
       </c>
       <c r="E50" s="1">
         <v>3.3999999999999998E-3</v>
@@ -3027,15 +3039,15 @@
       <c r="F50" s="1"/>
       <c r="G50" s="1"/>
       <c r="H50" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="I50" s="1"/>
       <c r="J50" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="K50" s="1"/>
       <c r="L50" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="51" spans="1:12" ht="29" x14ac:dyDescent="0.35">
@@ -3043,10 +3055,10 @@
         <v>37</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>43</v>
+        <v>144</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D51" s="1">
         <v>0.50930200000000003</v>
@@ -3057,15 +3069,15 @@
       <c r="F51" s="1"/>
       <c r="G51" s="1"/>
       <c r="H51" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="I51" s="1"/>
       <c r="J51" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="K51" s="1"/>
       <c r="L51" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="52" spans="1:12" ht="29" x14ac:dyDescent="0.35">
@@ -3073,10 +3085,10 @@
         <v>38</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>43</v>
+        <v>144</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D52" s="1">
         <v>0.35</v>
@@ -3087,15 +3099,15 @@
       <c r="F52" s="1"/>
       <c r="G52" s="1"/>
       <c r="H52" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="I52" s="1"/>
       <c r="J52" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="K52" s="1"/>
       <c r="L52" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="53" spans="1:12" ht="29" x14ac:dyDescent="0.35">
@@ -3103,13 +3115,13 @@
         <v>39</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>43</v>
+        <v>144</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E53" s="1">
         <v>0</v>
@@ -3117,15 +3129,15 @@
       <c r="F53" s="1"/>
       <c r="G53" s="1"/>
       <c r="H53" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I53" s="1"/>
       <c r="J53" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="K53" s="1"/>
       <c r="L53" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="54" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
@@ -3133,10 +3145,10 @@
         <v>41</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>43</v>
+        <v>144</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D54" s="1">
         <v>10.204700000000001</v>
@@ -3147,15 +3159,15 @@
       <c r="F54" s="1"/>
       <c r="G54" s="1"/>
       <c r="H54" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="I54" s="1"/>
       <c r="J54" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="K54" s="1"/>
       <c r="L54" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="55" spans="1:12" ht="29" x14ac:dyDescent="0.35">
@@ -3163,10 +3175,10 @@
         <v>42</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>43</v>
+        <v>144</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D55" s="1">
         <v>10.204700000000001</v>
@@ -3177,17 +3189,17 @@
       <c r="F55" s="1"/>
       <c r="G55" s="1"/>
       <c r="H55" s="1" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I55" s="1" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="J55" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="K55" s="1"/>
       <c r="L55" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="56" spans="1:12" ht="29" x14ac:dyDescent="0.35">
@@ -3195,10 +3207,10 @@
         <v>11</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D56" s="1">
         <v>10</v>
@@ -3213,17 +3225,17 @@
         <v>26.6</v>
       </c>
       <c r="H56" s="8" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="I56" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J56" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="K56" s="1"/>
       <c r="L56" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="57" spans="1:12" ht="29" x14ac:dyDescent="0.35">
@@ -3231,10 +3243,10 @@
         <v>12</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D57" s="9">
         <v>26</v>
@@ -3245,17 +3257,17 @@
       <c r="F57" s="7"/>
       <c r="G57" s="7"/>
       <c r="H57" s="7" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="I57" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J57" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="K57" s="1"/>
       <c r="L57" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="58" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
@@ -3263,10 +3275,10 @@
         <v>13</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D58" s="1">
         <v>0.3</v>
@@ -3281,17 +3293,17 @@
         <v>0.2</v>
       </c>
       <c r="H58" s="7" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="I58" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J58" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="K58" s="1"/>
       <c r="L58" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="59" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
@@ -3299,10 +3311,10 @@
         <v>14</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D59" s="1">
         <v>0.15</v>
@@ -3317,17 +3329,17 @@
         <v>0.2</v>
       </c>
       <c r="H59" s="7" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I59" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J59" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="K59" s="1"/>
       <c r="L59" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="60" spans="1:12" ht="58" x14ac:dyDescent="0.35">
@@ -3335,10 +3347,10 @@
         <v>15</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D60" s="1">
         <v>70</v>
@@ -3353,17 +3365,17 @@
         <v>100</v>
       </c>
       <c r="H60" s="7" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I60" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J60" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="K60" s="1"/>
       <c r="L60" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="61" spans="1:12" x14ac:dyDescent="0.35">
@@ -3371,10 +3383,10 @@
         <v>16</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D61" s="1">
         <v>0.4</v>
@@ -3389,17 +3401,17 @@
         <v>0.4</v>
       </c>
       <c r="H61" s="7" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="I61" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J61" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="K61" s="1"/>
       <c r="L61" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="62" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
@@ -3407,10 +3419,10 @@
         <v>17</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D62" s="1">
         <v>0.2</v>
@@ -3421,17 +3433,17 @@
       <c r="F62" s="7"/>
       <c r="G62" s="7"/>
       <c r="H62" s="7" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="I62" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J62" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="K62" s="1"/>
       <c r="L62" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="63" spans="1:12" x14ac:dyDescent="0.35">
@@ -3439,10 +3451,10 @@
         <v>18</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D63" s="7">
         <v>433.83</v>
@@ -3457,17 +3469,17 @@
         <v>905.48</v>
       </c>
       <c r="H63" s="7" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="I63" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J63" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="K63" s="1"/>
       <c r="L63" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.35">
@@ -3475,10 +3487,10 @@
         <v>19</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D64" s="1">
         <v>0</v>
@@ -3489,17 +3501,17 @@
       <c r="F64" s="7"/>
       <c r="G64" s="7"/>
       <c r="H64" s="7" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="I64" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J64" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="K64" s="1"/>
       <c r="L64" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="65" spans="1:12" ht="29" x14ac:dyDescent="0.35">
@@ -3507,7 +3519,7 @@
         <v>20</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C65" s="1"/>
       <c r="D65" s="7">
@@ -3523,17 +3535,17 @@
         <v>9</v>
       </c>
       <c r="H65" s="7" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="I65" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J65" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="K65" s="1"/>
       <c r="L65" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="66" spans="1:12" x14ac:dyDescent="0.35">
@@ -3541,10 +3553,10 @@
         <v>21</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D66" s="7">
         <v>1410</v>
@@ -3559,28 +3571,28 @@
         <v>1450</v>
       </c>
       <c r="H66" s="7" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="I66" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J66" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="K66" s="1"/>
       <c r="L66" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="67" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A67" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D67" s="10">
         <v>1.384623481E-3</v>
@@ -3595,31 +3607,32 @@
         <v>1.936006955E-3</v>
       </c>
       <c r="H67" s="7" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="I67" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J67" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="K67" s="1"/>
       <c r="L67" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="68" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A68" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D68" s="7">
-        <v>1.8181818181818181E-2</v>
+        <f>0.0181818181818182/state_variables_value!D5</f>
+        <v>0.18181818181818196</v>
       </c>
       <c r="E68" s="7">
         <v>3.6363636363636362E-2</v>
@@ -3627,28 +3640,28 @@
       <c r="F68" s="7"/>
       <c r="G68" s="7"/>
       <c r="H68" s="11" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="I68" s="1" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="J68" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="K68" s="1"/>
       <c r="L68" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="69" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A69" s="1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D69" s="1">
         <v>0.5</v>
@@ -3663,25 +3676,25 @@
         <v>0.5</v>
       </c>
       <c r="H69" s="1" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="I69" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="J69" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="K69" s="1"/>
       <c r="L69" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="70" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A70" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C70" s="1"/>
       <c r="D70" s="1">
@@ -3697,28 +3710,28 @@
         <v>0.37</v>
       </c>
       <c r="H70" s="1" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="I70" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="J70" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="K70" s="1"/>
       <c r="L70" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="71" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A71" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="D71" s="4">
         <v>2.7399999999999999E-5</v>
@@ -3729,28 +3742,28 @@
       <c r="F71" s="7"/>
       <c r="G71" s="7"/>
       <c r="H71" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="I71" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="I71" s="1" t="s">
-        <v>73</v>
-      </c>
       <c r="J71" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="K71" s="1"/>
       <c r="L71" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="72" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A72" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D72" s="4">
         <v>1.2999999999999999E-5</v>
@@ -3761,17 +3774,17 @@
       <c r="F72" s="7"/>
       <c r="G72" s="7"/>
       <c r="H72" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="I72" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="I72" s="1" t="s">
-        <v>73</v>
-      </c>
       <c r="J72" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="K72" s="1"/>
       <c r="L72" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -3788,7 +3801,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA0710C0-AB94-4FBF-AB29-E5085BC4F559}">
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.7265625" customWidth="1"/>
@@ -3800,27 +3813,27 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D1" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E1" t="s">
         <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B2" t="s">
         <v>34</v>
@@ -3833,15 +3846,15 @@
         <v>6.45</v>
       </c>
       <c r="E2" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="F2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B3" t="s">
         <v>35</v>
@@ -3854,18 +3867,18 @@
         <v>1.875</v>
       </c>
       <c r="E3" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="F3" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>80</v>
-      </c>
-      <c r="B4" t="s">
-        <v>43</v>
+        <v>78</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>144</v>
       </c>
       <c r="C4" t="s">
         <v>9</v>
@@ -3874,350 +3887,330 @@
         <v>0.1</v>
       </c>
       <c r="E4" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="F4" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C5" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D5">
         <v>0.1</v>
       </c>
       <c r="E5" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="F5" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B6" t="s">
-        <v>51</v>
+        <v>78</v>
       </c>
       <c r="C6" t="s">
-        <v>8</v>
+        <v>92</v>
       </c>
       <c r="D6">
-        <v>0.1</v>
+        <v>200</v>
       </c>
       <c r="E6" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="F6" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B7" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D7">
         <v>200</v>
       </c>
       <c r="E7" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F7" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B8" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C8" t="s">
+        <v>79</v>
+      </c>
+      <c r="D8">
+        <v>750</v>
+      </c>
+      <c r="E8" t="s">
         <v>95</v>
       </c>
-      <c r="D8">
-        <v>200</v>
-      </c>
-      <c r="E8" t="s">
-        <v>97</v>
-      </c>
       <c r="F8" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
+        <v>78</v>
+      </c>
+      <c r="B9" t="s">
+        <v>78</v>
+      </c>
+      <c r="C9" t="s">
         <v>80</v>
       </c>
-      <c r="B9" t="s">
-        <v>80</v>
-      </c>
-      <c r="C9" t="s">
-        <v>81</v>
-      </c>
       <c r="D9">
-        <v>750</v>
+        <v>6750</v>
       </c>
       <c r="E9" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F9" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B10" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D10">
-        <v>6750</v>
+        <v>2500</v>
       </c>
       <c r="E10" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F10" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="B11" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C11" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D11">
-        <v>2500</v>
+        <v>200</v>
       </c>
       <c r="E11" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F11" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B12" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C12" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D12">
-        <v>200</v>
+        <v>1000</v>
       </c>
       <c r="E12" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F12" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B13" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C13" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D13">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="E13" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F13" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B14" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C14" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D14">
-        <v>2000</v>
+        <v>10</v>
       </c>
       <c r="E14" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F14" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B15" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C15" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D15">
-        <v>10</v>
+        <v>0.1</v>
       </c>
       <c r="E15" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F15" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B16" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C16" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D16">
-        <v>0.1</v>
+        <v>400</v>
       </c>
       <c r="E16" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F16" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B17" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C17" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D17">
-        <v>400</v>
+        <v>10</v>
       </c>
       <c r="E17" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F17" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B18" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C18" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D18">
-        <v>10</v>
+        <v>1000</v>
       </c>
       <c r="E18" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F18" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C19" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D19">
-        <v>1000</v>
+        <v>3000</v>
       </c>
       <c r="E19" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F19" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B20" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C20" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D20">
-        <v>3000</v>
+        <v>40</v>
       </c>
       <c r="E20" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F20" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
-        <v>96</v>
-      </c>
-      <c r="B21" t="s">
-        <v>80</v>
-      </c>
-      <c r="C21" t="s">
-        <v>93</v>
-      </c>
-      <c r="D21">
-        <v>40</v>
-      </c>
-      <c r="E21" t="s">
-        <v>97</v>
-      </c>
-      <c r="F21" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -4236,13 +4229,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
@@ -4382,7 +4375,7 @@
         <v>5</v>
       </c>
       <c r="B14" t="s">
-        <v>43</v>
+        <v>144</v>
       </c>
       <c r="C14">
         <v>1</v>
@@ -4393,7 +4386,7 @@
         <v>6</v>
       </c>
       <c r="B15" t="s">
-        <v>43</v>
+        <v>144</v>
       </c>
       <c r="C15">
         <v>1</v>
@@ -4404,7 +4397,7 @@
         <v>7</v>
       </c>
       <c r="B16" t="s">
-        <v>43</v>
+        <v>144</v>
       </c>
       <c r="C16">
         <v>0</v>
@@ -4415,7 +4408,7 @@
         <v>8</v>
       </c>
       <c r="B17" t="s">
-        <v>43</v>
+        <v>144</v>
       </c>
       <c r="C17">
         <v>0</v>
@@ -4426,7 +4419,7 @@
         <v>9</v>
       </c>
       <c r="B18" t="s">
-        <v>43</v>
+        <v>144</v>
       </c>
       <c r="C18">
         <v>1</v>
@@ -4437,7 +4430,7 @@
         <v>10</v>
       </c>
       <c r="B19" t="s">
-        <v>43</v>
+        <v>144</v>
       </c>
       <c r="C19">
         <v>0</v>
@@ -4448,7 +4441,7 @@
         <v>5</v>
       </c>
       <c r="B20" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C20">
         <v>0</v>
@@ -4459,7 +4452,7 @@
         <v>6</v>
       </c>
       <c r="B21" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C21">
         <v>1</v>
@@ -4470,7 +4463,7 @@
         <v>7</v>
       </c>
       <c r="B22" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C22">
         <v>0</v>
@@ -4481,7 +4474,7 @@
         <v>8</v>
       </c>
       <c r="B23" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C23">
         <v>1</v>
@@ -4492,7 +4485,7 @@
         <v>9</v>
       </c>
       <c r="B24" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C24">
         <v>0</v>
@@ -4503,7 +4496,7 @@
         <v>10</v>
       </c>
       <c r="B25" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C25">
         <v>0</v>

</xml_diff>

<commit_message>
fixed one error in scenarios file.
</commit_message>
<xml_diff>
--- a/Data/scenarios.xlsx
+++ b/Data/scenarios.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rober\Documents\GitHub Repos\merging_SFW_decomposition_models\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B86018D-D56A-4987-822D-92A3E7138A29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF9891EA-450D-4493-A9E2-8E6DB8C1DE21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{7C97690C-9E7B-4D0E-86C0-16835BCB4BB0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7C97690C-9E7B-4D0E-86C0-16835BCB4BB0}"/>
   </bookViews>
   <sheets>
     <sheet name="scenarios" sheetId="1" r:id="rId1"/>
@@ -1470,20 +1470,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD4418A0-EB93-4361-AE80-4D25DF544368}">
   <dimension ref="A1:L72"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.26953125" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="22.7265625" customWidth="1"/>
-    <col min="4" max="4" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.90625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.36328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.6328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="52.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="22.7109375" customWidth="1"/>
+    <col min="4" max="4" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="52.28515625" bestFit="1" customWidth="1"/>
     <col min="9" max="10" width="23" customWidth="1"/>
-    <col min="11" max="11" width="13.26953125" customWidth="1"/>
+    <col min="11" max="11" width="13.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1521,7 +1521,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
@@ -1551,7 +1551,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
@@ -1579,7 +1579,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>13</v>
       </c>
@@ -1607,7 +1607,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>14</v>
       </c>
@@ -1635,7 +1635,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
@@ -1669,7 +1669,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>16</v>
       </c>
@@ -1703,7 +1703,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>17</v>
       </c>
@@ -1739,7 +1739,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>18</v>
       </c>
@@ -1777,7 +1777,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>19</v>
       </c>
@@ -1815,7 +1815,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
@@ -1847,7 +1847,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>21</v>
       </c>
@@ -1881,7 +1881,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>22</v>
       </c>
@@ -1916,7 +1916,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>23</v>
       </c>
@@ -1946,7 +1946,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>25</v>
       </c>
@@ -1976,7 +1976,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>27</v>
       </c>
@@ -2006,7 +2006,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="17" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>29</v>
       </c>
@@ -2037,7 +2037,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="18" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>30</v>
       </c>
@@ -2068,7 +2068,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="19" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>31</v>
       </c>
@@ -2099,7 +2099,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="20" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>32</v>
       </c>
@@ -2129,7 +2129,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="21" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>33</v>
       </c>
@@ -2161,7 +2161,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>11</v>
       </c>
@@ -2191,7 +2191,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>12</v>
       </c>
@@ -2221,7 +2221,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>13</v>
       </c>
@@ -2251,7 +2251,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>14</v>
       </c>
@@ -2281,7 +2281,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>15</v>
       </c>
@@ -2311,7 +2311,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>16</v>
       </c>
@@ -2341,7 +2341,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>17</v>
       </c>
@@ -2371,7 +2371,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>18</v>
       </c>
@@ -2401,7 +2401,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>19</v>
       </c>
@@ -2431,7 +2431,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>20</v>
       </c>
@@ -2461,7 +2461,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>21</v>
       </c>
@@ -2491,7 +2491,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>36</v>
       </c>
@@ -2524,7 +2524,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>37</v>
       </c>
@@ -2554,7 +2554,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>38</v>
       </c>
@@ -2584,7 +2584,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>39</v>
       </c>
@@ -2614,7 +2614,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="37" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>41</v>
       </c>
@@ -2646,7 +2646,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="38" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>42</v>
       </c>
@@ -2678,7 +2678,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>11</v>
       </c>
@@ -2708,7 +2708,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>12</v>
       </c>
@@ -2738,7 +2738,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="41" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>13</v>
       </c>
@@ -2768,7 +2768,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="42" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>14</v>
       </c>
@@ -2798,7 +2798,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>15</v>
       </c>
@@ -2828,7 +2828,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>16</v>
       </c>
@@ -2858,7 +2858,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>17</v>
       </c>
@@ -2889,7 +2889,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>18</v>
       </c>
@@ -2923,7 +2923,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>19</v>
       </c>
@@ -2957,7 +2957,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>20</v>
       </c>
@@ -2985,7 +2985,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>21</v>
       </c>
@@ -3019,7 +3019,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="50" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>36</v>
       </c>
@@ -3050,7 +3050,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="51" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>37</v>
       </c>
@@ -3080,7 +3080,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="52" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>38</v>
       </c>
@@ -3110,7 +3110,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="53" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>39</v>
       </c>
@@ -3140,7 +3140,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="54" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>41</v>
       </c>
@@ -3170,7 +3170,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="55" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>42</v>
       </c>
@@ -3202,7 +3202,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="56" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>11</v>
       </c>
@@ -3238,7 +3238,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="57" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>12</v>
       </c>
@@ -3249,10 +3249,10 @@
         <v>111</v>
       </c>
       <c r="D57" s="9">
-        <v>26</v>
+        <v>14.65</v>
       </c>
       <c r="E57" s="9">
-        <v>52</v>
+        <v>2</v>
       </c>
       <c r="F57" s="7"/>
       <c r="G57" s="7"/>
@@ -3270,7 +3270,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="58" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>13</v>
       </c>
@@ -3306,7 +3306,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="59" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>14</v>
       </c>
@@ -3342,7 +3342,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="60" spans="1:12" ht="58" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>15</v>
       </c>
@@ -3378,7 +3378,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>16</v>
       </c>
@@ -3414,7 +3414,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="62" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>17</v>
       </c>
@@ -3446,7 +3446,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>18</v>
       </c>
@@ -3482,7 +3482,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>19</v>
       </c>
@@ -3514,7 +3514,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="65" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>20</v>
       </c>
@@ -3548,7 +3548,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>21</v>
       </c>
@@ -3584,7 +3584,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="67" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>50</v>
       </c>
@@ -3620,7 +3620,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="68" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>51</v>
       </c>
@@ -3653,7 +3653,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>52</v>
       </c>
@@ -3689,7 +3689,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>53</v>
       </c>
@@ -3723,7 +3723,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="71" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>54</v>
       </c>
@@ -3755,7 +3755,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>55</v>
       </c>
@@ -3802,16 +3802,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA0710C0-AB94-4FBF-AB29-E5085BC4F559}">
   <dimension ref="A1:F20"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.7265625" customWidth="1"/>
+    <col min="1" max="1" width="11.7109375" customWidth="1"/>
     <col min="2" max="2" width="20" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.81640625" customWidth="1"/>
+    <col min="3" max="3" width="13.85546875" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="35.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="35.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>75</v>
       </c>
@@ -3831,7 +3831,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>78</v>
       </c>
@@ -3852,7 +3852,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>78</v>
       </c>
@@ -3873,7 +3873,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>78</v>
       </c>
@@ -3893,7 +3893,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>78</v>
       </c>
@@ -3913,7 +3913,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>78</v>
       </c>
@@ -3933,7 +3933,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>78</v>
       </c>
@@ -3953,7 +3953,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>78</v>
       </c>
@@ -3973,7 +3973,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>78</v>
       </c>
@@ -3993,7 +3993,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>78</v>
       </c>
@@ -4013,7 +4013,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>94</v>
       </c>
@@ -4033,7 +4033,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>94</v>
       </c>
@@ -4053,7 +4053,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>94</v>
       </c>
@@ -4073,7 +4073,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>94</v>
       </c>
@@ -4093,7 +4093,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>94</v>
       </c>
@@ -4113,7 +4113,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>94</v>
       </c>
@@ -4133,7 +4133,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>94</v>
       </c>
@@ -4153,7 +4153,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>94</v>
       </c>
@@ -4173,7 +4173,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>94</v>
       </c>
@@ -4193,7 +4193,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>94</v>
       </c>
@@ -4221,13 +4221,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC182590-26D0-4168-8E7C-B448CD67FE47}">
   <dimension ref="A1:C25"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>76</v>
       </c>
@@ -4238,7 +4238,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -4249,7 +4249,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -4260,7 +4260,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -4271,7 +4271,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -4282,7 +4282,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -4293,7 +4293,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -4304,7 +4304,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -4315,7 +4315,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>6</v>
       </c>
@@ -4326,7 +4326,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>7</v>
       </c>
@@ -4337,7 +4337,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -4348,7 +4348,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -4359,7 +4359,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>10</v>
       </c>
@@ -4370,7 +4370,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>5</v>
       </c>
@@ -4381,7 +4381,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>6</v>
       </c>
@@ -4392,7 +4392,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>7</v>
       </c>
@@ -4403,7 +4403,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>8</v>
       </c>
@@ -4414,7 +4414,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>9</v>
       </c>
@@ -4425,7 +4425,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>10</v>
       </c>
@@ -4436,7 +4436,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>5</v>
       </c>
@@ -4447,7 +4447,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>6</v>
       </c>
@@ -4458,7 +4458,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>7</v>
       </c>
@@ -4469,7 +4469,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>8</v>
       </c>
@@ -4480,7 +4480,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>9</v>
       </c>
@@ -4491,7 +4491,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Cleaned up the sensitivity analysis to remove the distinction between animal and ecosystem parameters. Now show the results together on one figure.
</commit_message>
<xml_diff>
--- a/Data/scenarios.xlsx
+++ b/Data/scenarios.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rober\Documents\GitHub Repos\merging_SFW_decomposition_models\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF9891EA-450D-4493-A9E2-8E6DB8C1DE21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95C1FBC3-3FEF-4DD6-85E1-6A13A4F3FCAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7C97690C-9E7B-4D0E-86C0-16835BCB4BB0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" xr2:uid="{7C97690C-9E7B-4D0E-86C0-16835BCB4BB0}"/>
   </bookViews>
   <sheets>
     <sheet name="scenarios" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="608" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="608" uniqueCount="146">
   <si>
     <t>Parameter</t>
   </si>
@@ -470,6 +470,9 @@
   </si>
   <si>
     <t>Microarthropod</t>
+  </si>
+  <si>
+    <t>Need the SD of mean annual temperature, not temperature over the year.</t>
   </si>
 </sst>
 </file>
@@ -1897,12 +1900,12 @@
       </c>
       <c r="E13" s="1"/>
       <c r="F13" s="1">
-        <f>0.217/365</f>
-        <v>5.9452054794520545E-4</v>
+        <f>0.217/365/state_variables_value!D2</f>
+        <v>9.2173728363597747E-5</v>
       </c>
       <c r="G13" s="1">
-        <f>0.0018</f>
-        <v>1.8E-3</v>
+        <f>0.0018/state_variables_value!D2</f>
+        <v>2.7906976744186045E-4</v>
       </c>
       <c r="H13" s="1" t="s">
         <v>120</v>
@@ -3202,7 +3205,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="56" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>11</v>
       </c>
@@ -3215,20 +3218,14 @@
       <c r="D56" s="1">
         <v>10</v>
       </c>
-      <c r="E56" s="1">
-        <v>20</v>
-      </c>
-      <c r="F56" s="7">
-        <v>-2.7</v>
-      </c>
-      <c r="G56" s="7">
-        <v>26.6</v>
-      </c>
+      <c r="E56" s="1"/>
+      <c r="F56" s="7"/>
+      <c r="G56" s="7"/>
       <c r="H56" s="8" t="s">
         <v>130</v>
       </c>
       <c r="I56" s="1" t="s">
-        <v>73</v>
+        <v>145</v>
       </c>
       <c r="J56" s="1" t="s">
         <v>61</v>

</xml_diff>

<commit_message>
Went back to the split model to highlight parameter differences based on how they were defined. Need to finalize #5.
</commit_message>
<xml_diff>
--- a/Data/scenarios.xlsx
+++ b/Data/scenarios.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rober\Documents\GitHub Repos\merging_SFW_decomposition_models\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95C1FBC3-3FEF-4DD6-85E1-6A13A4F3FCAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D625E2A7-BDE2-4E7B-B2AD-91C71BD8B5DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" xr2:uid="{7C97690C-9E7B-4D0E-86C0-16835BCB4BB0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7C97690C-9E7B-4D0E-86C0-16835BCB4BB0}"/>
   </bookViews>
   <sheets>
     <sheet name="scenarios" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="608" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="609" uniqueCount="146">
   <si>
     <t>Parameter</t>
   </si>
@@ -406,9 +406,6 @@
     <t>Warburg et al. 1984 2.5 year lifespan</t>
   </si>
   <si>
-    <t>Topp et al. 2006 SBB</t>
-  </si>
-  <si>
     <t>Topp et al. 2006 for density, NM&amp;M lab for weight</t>
   </si>
   <si>
@@ -473,6 +470,9 @@
   </si>
   <si>
     <t>Need the SD of mean annual temperature, not temperature over the year.</t>
+  </si>
+  <si>
+    <t>Topp et al. 2006 SBB; min/max made up</t>
   </si>
 </sst>
 </file>
@@ -1537,15 +1537,19 @@
       <c r="D2" s="1">
         <v>6</v>
       </c>
-      <c r="E2" s="1">
-        <v>0</v>
-      </c>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1">
+        <v>3</v>
+      </c>
+      <c r="G2" s="1">
+        <v>9</v>
+      </c>
       <c r="H2" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="I2" s="1"/>
+      <c r="I2" s="1" t="s">
+        <v>124</v>
+      </c>
       <c r="J2" s="1" t="s">
         <v>61</v>
       </c>
@@ -1567,9 +1571,7 @@
       <c r="D3" s="1">
         <v>26</v>
       </c>
-      <c r="E3" s="1">
-        <v>0</v>
-      </c>
+      <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
@@ -1595,11 +1597,13 @@
       <c r="D4" s="1">
         <v>0.3</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="1"/>
+      <c r="F4" s="1">
         <v>0</v>
       </c>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
+      <c r="G4" s="1">
+        <v>1</v>
+      </c>
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1" t="s">
@@ -1623,9 +1627,7 @@
       <c r="D5" s="1">
         <v>0.15</v>
       </c>
-      <c r="E5" s="1">
-        <v>0</v>
-      </c>
+      <c r="E5" s="1"/>
       <c r="F5" s="1"/>
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
@@ -1651,9 +1653,7 @@
       <c r="D6" s="1">
         <v>73</v>
       </c>
-      <c r="E6" s="1">
-        <v>0</v>
-      </c>
+      <c r="E6" s="1"/>
       <c r="F6" s="1">
         <v>71</v>
       </c>
@@ -1685,9 +1685,7 @@
       <c r="D7" s="1">
         <v>0.28000000000000003</v>
       </c>
-      <c r="E7" s="1">
-        <v>0</v>
-      </c>
+      <c r="E7" s="1"/>
       <c r="F7" s="1">
         <v>0.26</v>
       </c>
@@ -1719,9 +1717,7 @@
       <c r="D8" s="1">
         <v>0.2</v>
       </c>
-      <c r="E8" s="1">
-        <v>0</v>
-      </c>
+      <c r="E8" s="1"/>
       <c r="F8" s="1">
         <v>0.12</v>
       </c>
@@ -1829,9 +1825,7 @@
       <c r="D11" s="1">
         <v>7.7</v>
       </c>
-      <c r="E11" s="1">
-        <v>0</v>
-      </c>
+      <c r="E11" s="1"/>
       <c r="F11" s="1">
         <v>7.5</v>
       </c>
@@ -1935,8 +1929,12 @@
       <c r="E14" s="1">
         <v>0.06</v>
       </c>
-      <c r="F14" s="1"/>
-      <c r="G14" s="1"/>
+      <c r="F14" s="1">
+        <v>0</v>
+      </c>
+      <c r="G14" s="1">
+        <v>1</v>
+      </c>
       <c r="H14" s="1" t="s">
         <v>24</v>
       </c>
@@ -1965,8 +1963,12 @@
       <c r="E15" s="1">
         <v>0.06</v>
       </c>
-      <c r="F15" s="1"/>
-      <c r="G15" s="1"/>
+      <c r="F15" s="1">
+        <v>0</v>
+      </c>
+      <c r="G15" s="1">
+        <v>1</v>
+      </c>
       <c r="H15" s="1" t="s">
         <v>26</v>
       </c>
@@ -1995,8 +1997,12 @@
       <c r="E16" s="1">
         <v>7.0300000000000001E-2</v>
       </c>
-      <c r="F16" s="1"/>
-      <c r="G16" s="1"/>
+      <c r="F16" s="1">
+        <v>0</v>
+      </c>
+      <c r="G16" s="1">
+        <v>1</v>
+      </c>
       <c r="H16" s="1" t="s">
         <v>28</v>
       </c>
@@ -2023,9 +2029,7 @@
         <f>0.00207/0.0375</f>
         <v>5.5199999999999999E-2</v>
       </c>
-      <c r="E17" s="1">
-        <v>0</v>
-      </c>
+      <c r="E17" s="1"/>
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
       <c r="H17" s="1" t="s">
@@ -2054,9 +2058,7 @@
         <f>0.00207/0.0375</f>
         <v>5.5199999999999999E-2</v>
       </c>
-      <c r="E18" s="1">
-        <v>0</v>
-      </c>
+      <c r="E18" s="1"/>
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
       <c r="H18" s="1" t="s">
@@ -2085,9 +2087,7 @@
         <f>0.00207/0.0375</f>
         <v>5.5199999999999999E-2</v>
       </c>
-      <c r="E19" s="1">
-        <v>0</v>
-      </c>
+      <c r="E19" s="1"/>
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
       <c r="H19" s="1" t="s">
@@ -2115,11 +2115,13 @@
       <c r="D20" s="1">
         <v>0</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20" s="1"/>
+      <c r="F20" s="1">
         <v>0</v>
       </c>
-      <c r="F20" s="1"/>
-      <c r="G20" s="1"/>
+      <c r="G20" s="1">
+        <v>1</v>
+      </c>
       <c r="H20" s="1"/>
       <c r="I20" s="1" t="s">
         <v>109</v>
@@ -2145,13 +2147,11 @@
       <c r="D21" s="1">
         <v>-5.5040310000000002E-2</v>
       </c>
-      <c r="E21" s="1">
-        <v>0</v>
-      </c>
+      <c r="E21" s="1"/>
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
       <c r="H21" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I21" s="1" t="s">
         <v>121</v>
@@ -2177,14 +2177,16 @@
       <c r="D22" s="1">
         <v>6</v>
       </c>
-      <c r="E22" s="1">
-        <v>0</v>
-      </c>
-      <c r="F22" s="1"/>
-      <c r="G22" s="1"/>
+      <c r="E22" s="1"/>
+      <c r="F22" s="1">
+        <v>3</v>
+      </c>
+      <c r="G22" s="1">
+        <v>9</v>
+      </c>
       <c r="H22" s="1"/>
       <c r="I22" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="J22" s="1" t="s">
         <v>61</v>
@@ -2207,14 +2209,12 @@
       <c r="D23" s="1">
         <v>26</v>
       </c>
-      <c r="E23" s="1">
-        <v>0</v>
-      </c>
+      <c r="E23" s="1"/>
       <c r="F23" s="1"/>
       <c r="G23" s="1"/>
       <c r="H23" s="1"/>
       <c r="I23" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="J23" s="1" t="s">
         <v>61</v>
@@ -2237,14 +2237,16 @@
       <c r="D24" s="1">
         <v>0.3</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E24" s="1"/>
+      <c r="F24" s="1">
         <v>0</v>
       </c>
-      <c r="F24" s="1"/>
-      <c r="G24" s="1"/>
+      <c r="G24" s="1">
+        <v>0.5</v>
+      </c>
       <c r="H24" s="1"/>
       <c r="I24" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="J24" s="1" t="s">
         <v>61</v>
@@ -2267,14 +2269,12 @@
       <c r="D25" s="1">
         <v>0.15</v>
       </c>
-      <c r="E25" s="1">
-        <v>0</v>
-      </c>
+      <c r="E25" s="1"/>
       <c r="F25" s="1"/>
       <c r="G25" s="1"/>
       <c r="H25" s="1"/>
       <c r="I25" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="J25" s="1" t="s">
         <v>61</v>
@@ -2297,14 +2297,16 @@
       <c r="D26" s="1">
         <v>70</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26" s="1"/>
+      <c r="F26" s="1">
         <v>0</v>
       </c>
-      <c r="F26" s="1"/>
-      <c r="G26" s="1"/>
+      <c r="G26" s="1">
+        <v>100</v>
+      </c>
       <c r="H26" s="1"/>
       <c r="I26" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="J26" s="1" t="s">
         <v>61</v>
@@ -2327,14 +2329,16 @@
       <c r="D27" s="1">
         <v>0.4</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27" s="1"/>
+      <c r="F27" s="1">
         <v>0</v>
       </c>
-      <c r="F27" s="1"/>
-      <c r="G27" s="1"/>
+      <c r="G27" s="1">
+        <v>1</v>
+      </c>
       <c r="H27" s="1"/>
       <c r="I27" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="J27" s="1" t="s">
         <v>61</v>
@@ -2357,14 +2361,16 @@
       <c r="D28" s="1">
         <v>0.2</v>
       </c>
-      <c r="E28" s="1">
+      <c r="E28" s="1"/>
+      <c r="F28" s="1">
         <v>0</v>
       </c>
-      <c r="F28" s="1"/>
-      <c r="G28" s="1"/>
+      <c r="G28" s="1">
+        <v>1</v>
+      </c>
       <c r="H28" s="1"/>
       <c r="I28" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="J28" s="1" t="s">
         <v>61</v>
@@ -2387,14 +2393,12 @@
       <c r="D29" s="1">
         <v>50</v>
       </c>
-      <c r="E29" s="1">
-        <v>0</v>
-      </c>
+      <c r="E29" s="1"/>
       <c r="F29" s="1"/>
       <c r="G29" s="1"/>
       <c r="H29" s="1"/>
       <c r="I29" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="J29" s="1" t="s">
         <v>62</v>
@@ -2417,14 +2421,12 @@
       <c r="D30" s="1">
         <v>1270</v>
       </c>
-      <c r="E30" s="1">
-        <v>0</v>
-      </c>
+      <c r="E30" s="1"/>
       <c r="F30" s="1"/>
       <c r="G30" s="1"/>
       <c r="H30" s="1"/>
       <c r="I30" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="J30" s="1" t="s">
         <v>62</v>
@@ -2445,16 +2447,18 @@
       <c r="D31" s="1">
         <v>6</v>
       </c>
-      <c r="E31" s="1">
-        <v>0</v>
-      </c>
-      <c r="F31" s="1"/>
-      <c r="G31" s="1"/>
+      <c r="E31" s="1"/>
+      <c r="F31" s="1">
+        <v>2</v>
+      </c>
+      <c r="G31" s="1">
+        <v>10</v>
+      </c>
       <c r="H31" s="1" t="s">
-        <v>123</v>
+        <v>145</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="J31" s="1" t="s">
         <v>61</v>
@@ -2477,14 +2481,12 @@
       <c r="D32" s="1">
         <v>1300</v>
       </c>
-      <c r="E32" s="1">
-        <v>0</v>
-      </c>
+      <c r="E32" s="1"/>
       <c r="F32" s="1"/>
       <c r="G32" s="1"/>
       <c r="H32" s="1"/>
       <c r="I32" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="J32" s="1" t="s">
         <v>61</v>
@@ -2508,16 +2510,14 @@
         <f>1/(2.5*365*state_variables_value!D3)</f>
         <v>5.8447488584474887E-4</v>
       </c>
-      <c r="E33" s="1">
-        <v>0</v>
-      </c>
+      <c r="E33" s="1"/>
       <c r="F33" s="1"/>
       <c r="G33" s="1"/>
       <c r="H33" s="1" t="s">
         <v>122</v>
       </c>
       <c r="I33" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="J33" s="1" t="s">
         <v>63</v>
@@ -2540,14 +2540,12 @@
       <c r="D34" s="1">
         <v>0.5</v>
       </c>
-      <c r="E34" s="1">
-        <v>0</v>
-      </c>
+      <c r="E34" s="1"/>
       <c r="F34" s="1"/>
       <c r="G34" s="1"/>
       <c r="H34" s="1"/>
       <c r="I34" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="J34" s="1" t="s">
         <v>63</v>
@@ -2570,14 +2568,12 @@
       <c r="D35" s="1">
         <v>0.35</v>
       </c>
-      <c r="E35" s="1">
-        <v>0</v>
-      </c>
+      <c r="E35" s="1"/>
       <c r="F35" s="1"/>
       <c r="G35" s="1"/>
       <c r="H35" s="1"/>
       <c r="I35" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="J35" s="1" t="s">
         <v>63</v>
@@ -2600,14 +2596,12 @@
       <c r="D36" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="E36" s="1">
-        <v>0</v>
-      </c>
+      <c r="E36" s="1"/>
       <c r="F36" s="1"/>
       <c r="G36" s="1"/>
       <c r="H36" s="1"/>
       <c r="I36" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="J36" s="1" t="s">
         <v>63</v>
@@ -2630,16 +2624,14 @@
       <c r="D37" s="6">
         <v>0.4236007</v>
       </c>
-      <c r="E37" s="1">
-        <v>0</v>
-      </c>
+      <c r="E37" s="1"/>
       <c r="F37" s="1"/>
       <c r="G37" s="1"/>
       <c r="H37" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="J37" s="1" t="s">
         <v>64</v>
@@ -2662,16 +2654,14 @@
       <c r="D38" s="6">
         <v>0.4236007</v>
       </c>
-      <c r="E38" s="1">
-        <v>0</v>
-      </c>
+      <c r="E38" s="1"/>
       <c r="F38" s="1"/>
       <c r="G38" s="1"/>
       <c r="H38" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="I38" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="J38" s="1" t="s">
         <v>64</v>
@@ -2686,7 +2676,7 @@
         <v>11</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>111</v>
@@ -2716,7 +2706,7 @@
         <v>12</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>111</v>
@@ -2746,7 +2736,7 @@
         <v>13</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>117</v>
@@ -2776,7 +2766,7 @@
         <v>14</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>117</v>
@@ -2806,16 +2796,16 @@
         <v>15</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C43" s="1" t="s">
         <v>112</v>
       </c>
       <c r="D43" s="1">
-        <v>0.45</v>
+        <v>45</v>
       </c>
       <c r="E43" s="1">
-        <v>0.05</v>
+        <v>5</v>
       </c>
       <c r="F43" s="1"/>
       <c r="G43" s="1"/>
@@ -2836,7 +2826,7 @@
         <v>16</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C44" s="1" t="s">
         <v>113</v>
@@ -2866,7 +2856,7 @@
         <v>17</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C45" s="1" t="s">
         <v>113</v>
@@ -2897,7 +2887,7 @@
         <v>18</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C46" s="1" t="s">
         <v>114</v>
@@ -2931,7 +2921,7 @@
         <v>19</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C47" s="1" t="s">
         <v>114</v>
@@ -2965,7 +2955,7 @@
         <v>20</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C48" s="1"/>
       <c r="D48" s="1">
@@ -2993,7 +2983,7 @@
         <v>21</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C49" s="1" t="s">
         <v>115</v>
@@ -3027,7 +3017,7 @@
         <v>36</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C50" s="1" t="s">
         <v>116</v>
@@ -3058,7 +3048,7 @@
         <v>37</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>113</v>
@@ -3088,7 +3078,7 @@
         <v>38</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C52" s="1" t="s">
         <v>113</v>
@@ -3118,7 +3108,7 @@
         <v>39</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C53" s="1" t="s">
         <v>116</v>
@@ -3126,9 +3116,7 @@
       <c r="D53" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="E53" s="1">
-        <v>0</v>
-      </c>
+      <c r="E53" s="1"/>
       <c r="F53" s="1"/>
       <c r="G53" s="1"/>
       <c r="H53" s="1" t="s">
@@ -3148,7 +3136,7 @@
         <v>41</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C54" s="1" t="s">
         <v>113</v>
@@ -3162,7 +3150,7 @@
       <c r="F54" s="1"/>
       <c r="G54" s="1"/>
       <c r="H54" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="I54" s="1"/>
       <c r="J54" s="1" t="s">
@@ -3178,7 +3166,7 @@
         <v>42</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C55" s="1" t="s">
         <v>113</v>
@@ -3219,13 +3207,17 @@
         <v>10</v>
       </c>
       <c r="E56" s="1"/>
-      <c r="F56" s="7"/>
-      <c r="G56" s="7"/>
+      <c r="F56" s="7">
+        <v>5</v>
+      </c>
+      <c r="G56" s="7">
+        <v>15</v>
+      </c>
       <c r="H56" s="8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I56" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="J56" s="1" t="s">
         <v>61</v>
@@ -3254,7 +3246,7 @@
       <c r="F57" s="7"/>
       <c r="G57" s="7"/>
       <c r="H57" s="7" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="I57" s="1" t="s">
         <v>73</v>
@@ -3290,7 +3282,7 @@
         <v>0.2</v>
       </c>
       <c r="H58" s="7" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="I58" s="1" t="s">
         <v>73</v>
@@ -3326,7 +3318,7 @@
         <v>0.2</v>
       </c>
       <c r="H59" s="7" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I59" s="1" t="s">
         <v>73</v>
@@ -3352,17 +3344,15 @@
       <c r="D60" s="1">
         <v>70</v>
       </c>
-      <c r="E60" s="1">
-        <v>140</v>
-      </c>
+      <c r="E60" s="1"/>
       <c r="F60" s="7">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="G60" s="7">
         <v>100</v>
       </c>
       <c r="H60" s="7" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="I60" s="1" t="s">
         <v>73</v>
@@ -3398,7 +3388,7 @@
         <v>0.4</v>
       </c>
       <c r="H61" s="7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I61" s="1" t="s">
         <v>73</v>
@@ -3430,7 +3420,7 @@
       <c r="F62" s="7"/>
       <c r="G62" s="7"/>
       <c r="H62" s="7" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="I62" s="1" t="s">
         <v>73</v>
@@ -3466,7 +3456,7 @@
         <v>905.48</v>
       </c>
       <c r="H63" s="7" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I63" s="1" t="s">
         <v>73</v>
@@ -3498,7 +3488,7 @@
       <c r="F64" s="7"/>
       <c r="G64" s="7"/>
       <c r="H64" s="7" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I64" s="1" t="s">
         <v>73</v>
@@ -3522,9 +3512,7 @@
       <c r="D65" s="7">
         <v>7</v>
       </c>
-      <c r="E65" s="7">
-        <v>14</v>
-      </c>
+      <c r="E65" s="7"/>
       <c r="F65" s="7">
         <v>5</v>
       </c>
@@ -3532,7 +3520,7 @@
         <v>9</v>
       </c>
       <c r="H65" s="7" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I65" s="1" t="s">
         <v>73</v>
@@ -3568,7 +3556,7 @@
         <v>1450</v>
       </c>
       <c r="H66" s="7" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="I66" s="1" t="s">
         <v>73</v>
@@ -3604,7 +3592,7 @@
         <v>1.936006955E-3</v>
       </c>
       <c r="H67" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="I67" s="1" t="s">
         <v>73</v>
@@ -3637,7 +3625,7 @@
       <c r="F68" s="7"/>
       <c r="G68" s="7"/>
       <c r="H68" s="11" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="I68" s="1" t="s">
         <v>72</v>
@@ -3663,9 +3651,7 @@
       <c r="D69" s="1">
         <v>0.5</v>
       </c>
-      <c r="E69" s="7">
-        <v>0</v>
-      </c>
+      <c r="E69" s="7"/>
       <c r="F69" s="7">
         <v>0.5</v>
       </c>
@@ -3673,7 +3659,7 @@
         <v>0.5</v>
       </c>
       <c r="H69" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="I69" s="1" t="s">
         <v>71</v>
@@ -3697,9 +3683,7 @@
       <c r="D70" s="1">
         <v>0.37</v>
       </c>
-      <c r="E70" s="7">
-        <v>0</v>
-      </c>
+      <c r="E70" s="7"/>
       <c r="F70" s="7">
         <v>0.37</v>
       </c>
@@ -3707,7 +3691,7 @@
         <v>0.37</v>
       </c>
       <c r="H70" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="I70" s="1" t="s">
         <v>71</v>
@@ -3843,7 +3827,7 @@
         <v>6.45</v>
       </c>
       <c r="E2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F2" t="s">
         <v>59</v>
@@ -3864,7 +3848,7 @@
         <v>1.875</v>
       </c>
       <c r="E3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F3" t="s">
         <v>59</v>
@@ -3875,7 +3859,7 @@
         <v>78</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C4" t="s">
         <v>9</v>
@@ -4372,7 +4356,7 @@
         <v>5</v>
       </c>
       <c r="B14" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C14">
         <v>1</v>
@@ -4383,7 +4367,7 @@
         <v>6</v>
       </c>
       <c r="B15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C15">
         <v>1</v>
@@ -4394,7 +4378,7 @@
         <v>7</v>
       </c>
       <c r="B16" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C16">
         <v>0</v>
@@ -4405,7 +4389,7 @@
         <v>8</v>
       </c>
       <c r="B17" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C17">
         <v>0</v>
@@ -4416,7 +4400,7 @@
         <v>9</v>
       </c>
       <c r="B18" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C18">
         <v>1</v>
@@ -4427,7 +4411,7 @@
         <v>10</v>
       </c>
       <c r="B19" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C19">
         <v>0</v>

</xml_diff>

<commit_message>
Updated output for animal parameter uncertainty.
</commit_message>
<xml_diff>
--- a/Data/scenarios.xlsx
+++ b/Data/scenarios.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rober\Documents\GitHub Repos\merging_SFW_decomposition_models\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D625E2A7-BDE2-4E7B-B2AD-91C71BD8B5DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14DCFFA2-3AEC-484F-A928-7EDB61DA1BCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7C97690C-9E7B-4D0E-86C0-16835BCB4BB0}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{7C97690C-9E7B-4D0E-86C0-16835BCB4BB0}"/>
   </bookViews>
   <sheets>
     <sheet name="scenarios" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="609" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="611" uniqueCount="147">
   <si>
     <t>Parameter</t>
   </si>
@@ -473,6 +473,9 @@
   </si>
   <si>
     <t>Topp et al. 2006 SBB; min/max made up</t>
+  </si>
+  <si>
+    <t>Giovanni for NB</t>
   </si>
 </sst>
 </file>
@@ -1473,20 +1476,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD4418A0-EB93-4361-AE80-4D25DF544368}">
   <dimension ref="A1:L72"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="22.7109375" customWidth="1"/>
-    <col min="4" max="4" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="52.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="22.7265625" customWidth="1"/>
+    <col min="4" max="4" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="52.26953125" bestFit="1" customWidth="1"/>
     <col min="9" max="10" width="23" customWidth="1"/>
-    <col min="11" max="11" width="13.28515625" customWidth="1"/>
+    <col min="11" max="11" width="13.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1524,7 +1527,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
@@ -1558,7 +1561,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
@@ -1584,7 +1587,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>13</v>
       </c>
@@ -1595,16 +1598,20 @@
         <v>117</v>
       </c>
       <c r="D4" s="1">
-        <v>0.3</v>
-      </c>
-      <c r="E4" s="1"/>
+        <v>0.33</v>
+      </c>
+      <c r="E4" s="1">
+        <v>7.0000000000000007E-2</v>
+      </c>
       <c r="F4" s="1">
         <v>0</v>
       </c>
       <c r="G4" s="1">
         <v>1</v>
       </c>
-      <c r="H4" s="1"/>
+      <c r="H4" s="1" t="s">
+        <v>146</v>
+      </c>
       <c r="I4" s="1"/>
       <c r="J4" s="1" t="s">
         <v>61</v>
@@ -1614,7 +1621,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>14</v>
       </c>
@@ -1640,7 +1647,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
@@ -1672,7 +1679,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>16</v>
       </c>
@@ -1704,7 +1711,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>17</v>
       </c>
@@ -1738,7 +1745,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>18</v>
       </c>
@@ -1776,7 +1783,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>19</v>
       </c>
@@ -1814,7 +1821,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
@@ -1844,7 +1851,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>21</v>
       </c>
@@ -1878,7 +1885,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>22</v>
       </c>
@@ -1913,7 +1920,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>23</v>
       </c>
@@ -1947,7 +1954,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>25</v>
       </c>
@@ -1981,7 +1988,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>27</v>
       </c>
@@ -2015,7 +2022,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="17" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>29</v>
       </c>
@@ -2044,7 +2051,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="18" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>30</v>
       </c>
@@ -2073,7 +2080,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="19" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>31</v>
       </c>
@@ -2102,7 +2109,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="20" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>32</v>
       </c>
@@ -2134,7 +2141,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="21" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>33</v>
       </c>
@@ -2164,7 +2171,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>11</v>
       </c>
@@ -2196,7 +2203,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>12</v>
       </c>
@@ -2224,7 +2231,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>13</v>
       </c>
@@ -2235,16 +2242,20 @@
         <v>117</v>
       </c>
       <c r="D24" s="1">
-        <v>0.3</v>
-      </c>
-      <c r="E24" s="1"/>
+        <v>0.33</v>
+      </c>
+      <c r="E24" s="1">
+        <v>7.0000000000000007E-2</v>
+      </c>
       <c r="F24" s="1">
         <v>0</v>
       </c>
       <c r="G24" s="1">
-        <v>0.5</v>
-      </c>
-      <c r="H24" s="1"/>
+        <v>1</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>146</v>
+      </c>
       <c r="I24" s="1" t="s">
         <v>124</v>
       </c>
@@ -2256,7 +2267,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>14</v>
       </c>
@@ -2284,7 +2295,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>15</v>
       </c>
@@ -2316,7 +2327,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>16</v>
       </c>
@@ -2348,7 +2359,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>17</v>
       </c>
@@ -2380,7 +2391,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>18</v>
       </c>
@@ -2408,7 +2419,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>19</v>
       </c>
@@ -2436,7 +2447,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>20</v>
       </c>
@@ -2468,7 +2479,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>21</v>
       </c>
@@ -2496,7 +2507,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>36</v>
       </c>
@@ -2527,7 +2538,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>37</v>
       </c>
@@ -2555,7 +2566,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>38</v>
       </c>
@@ -2583,7 +2594,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>39</v>
       </c>
@@ -2611,7 +2622,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="37" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>41</v>
       </c>
@@ -2641,7 +2652,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="38" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>42</v>
       </c>
@@ -2671,7 +2682,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>11</v>
       </c>
@@ -2701,7 +2712,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
         <v>12</v>
       </c>
@@ -2731,7 +2742,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="41" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
         <v>13</v>
       </c>
@@ -2747,8 +2758,12 @@
       <c r="E41" s="1">
         <v>0.04</v>
       </c>
-      <c r="F41" s="1"/>
-      <c r="G41" s="1"/>
+      <c r="F41" s="1">
+        <v>0</v>
+      </c>
+      <c r="G41" s="1">
+        <v>1</v>
+      </c>
       <c r="H41" s="1" t="s">
         <v>44</v>
       </c>
@@ -2761,7 +2776,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="42" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
         <v>14</v>
       </c>
@@ -2791,7 +2806,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
         <v>15</v>
       </c>
@@ -2821,7 +2836,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
         <v>16</v>
       </c>
@@ -2851,7 +2866,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
         <v>17</v>
       </c>
@@ -2882,7 +2897,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
         <v>18</v>
       </c>
@@ -2916,7 +2931,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>19</v>
       </c>
@@ -2950,7 +2965,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
         <v>20</v>
       </c>
@@ -2978,7 +2993,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>21</v>
       </c>
@@ -3012,7 +3027,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="50" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
         <v>36</v>
       </c>
@@ -3043,7 +3058,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="51" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A51" s="1" t="s">
         <v>37</v>
       </c>
@@ -3073,7 +3088,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="52" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
         <v>38</v>
       </c>
@@ -3103,7 +3118,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="53" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A53" s="1" t="s">
         <v>39</v>
       </c>
@@ -3131,7 +3146,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="54" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
         <v>41</v>
       </c>
@@ -3161,7 +3176,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="55" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A55" s="1" t="s">
         <v>42</v>
       </c>
@@ -3193,7 +3208,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="56" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
         <v>11</v>
       </c>
@@ -3227,7 +3242,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="57" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
         <v>12</v>
       </c>
@@ -3259,7 +3274,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="58" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A58" s="1" t="s">
         <v>13</v>
       </c>
@@ -3270,11 +3285,9 @@
         <v>117</v>
       </c>
       <c r="D58" s="1">
-        <v>0.3</v>
-      </c>
-      <c r="E58" s="1">
-        <v>0.6</v>
-      </c>
+        <v>0.17</v>
+      </c>
+      <c r="E58" s="1"/>
       <c r="F58" s="7">
         <v>0.15</v>
       </c>
@@ -3295,7 +3308,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="59" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
         <v>14</v>
       </c>
@@ -3331,7 +3344,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="60" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:12" ht="58" x14ac:dyDescent="0.35">
       <c r="A60" s="1" t="s">
         <v>15</v>
       </c>
@@ -3365,7 +3378,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A61" s="1" t="s">
         <v>16</v>
       </c>
@@ -3401,7 +3414,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="62" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A62" s="1" t="s">
         <v>17</v>
       </c>
@@ -3433,7 +3446,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A63" s="1" t="s">
         <v>18</v>
       </c>
@@ -3469,7 +3482,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A64" s="1" t="s">
         <v>19</v>
       </c>
@@ -3501,7 +3514,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="65" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A65" s="1" t="s">
         <v>20</v>
       </c>
@@ -3533,7 +3546,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A66" s="1" t="s">
         <v>21</v>
       </c>
@@ -3569,7 +3582,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="67" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A67" s="1" t="s">
         <v>50</v>
       </c>
@@ -3605,7 +3618,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="68" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A68" s="1" t="s">
         <v>51</v>
       </c>
@@ -3638,7 +3651,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="69" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A69" s="1" t="s">
         <v>52</v>
       </c>
@@ -3672,7 +3685,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="70" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A70" s="1" t="s">
         <v>53</v>
       </c>
@@ -3704,7 +3717,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="71" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A71" s="1" t="s">
         <v>54</v>
       </c>
@@ -3736,7 +3749,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A72" s="1" t="s">
         <v>55</v>
       </c>
@@ -3783,16 +3796,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA0710C0-AB94-4FBF-AB29-E5085BC4F559}">
   <dimension ref="A1:F20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.7109375" customWidth="1"/>
+    <col min="1" max="1" width="11.7265625" customWidth="1"/>
     <col min="2" max="2" width="20" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.85546875" customWidth="1"/>
+    <col min="3" max="3" width="13.81640625" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="35.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="35.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>75</v>
       </c>
@@ -3812,7 +3825,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>78</v>
       </c>
@@ -3833,7 +3846,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>78</v>
       </c>
@@ -3854,7 +3867,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>78</v>
       </c>
@@ -3874,7 +3887,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>78</v>
       </c>
@@ -3894,7 +3907,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>78</v>
       </c>
@@ -3914,7 +3927,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>78</v>
       </c>
@@ -3934,7 +3947,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>78</v>
       </c>
@@ -3954,7 +3967,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>78</v>
       </c>
@@ -3974,7 +3987,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>78</v>
       </c>
@@ -3994,7 +4007,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>94</v>
       </c>
@@ -4014,7 +4027,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>94</v>
       </c>
@@ -4034,7 +4047,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>94</v>
       </c>
@@ -4054,7 +4067,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>94</v>
       </c>
@@ -4074,7 +4087,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>94</v>
       </c>
@@ -4094,7 +4107,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>94</v>
       </c>
@@ -4114,7 +4127,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>94</v>
       </c>
@@ -4134,7 +4147,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>94</v>
       </c>
@@ -4154,7 +4167,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>94</v>
       </c>
@@ -4174,7 +4187,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>94</v>
       </c>
@@ -4202,13 +4215,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC182590-26D0-4168-8E7C-B448CD67FE47}">
   <dimension ref="A1:C25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.7265625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>76</v>
       </c>
@@ -4219,7 +4232,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -4230,7 +4243,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -4241,7 +4254,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -4252,7 +4265,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -4263,7 +4276,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -4274,7 +4287,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -4285,7 +4298,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -4296,7 +4309,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>6</v>
       </c>
@@ -4307,7 +4320,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>7</v>
       </c>
@@ -4318,7 +4331,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -4329,7 +4342,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -4340,7 +4353,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>10</v>
       </c>
@@ -4351,7 +4364,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>5</v>
       </c>
@@ -4362,7 +4375,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>6</v>
       </c>
@@ -4373,7 +4386,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>7</v>
       </c>
@@ -4384,7 +4397,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>8</v>
       </c>
@@ -4395,7 +4408,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>9</v>
       </c>
@@ -4406,7 +4419,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>10</v>
       </c>
@@ -4417,7 +4430,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>5</v>
       </c>
@@ -4428,7 +4441,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>6</v>
       </c>
@@ -4439,7 +4452,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>7</v>
       </c>
@@ -4450,7 +4463,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>8</v>
       </c>
@@ -4461,7 +4474,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>9</v>
       </c>
@@ -4472,7 +4485,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Updated temperature for Root Herbivory scenario.
</commit_message>
<xml_diff>
--- a/Data/scenarios.xlsx
+++ b/Data/scenarios.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rober\Documents\GitHub Repos\merging_SFW_decomposition_models\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14DCFFA2-3AEC-484F-A928-7EDB61DA1BCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97B51A96-8F87-4558-A1F5-4A179A90BD63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{7C97690C-9E7B-4D0E-86C0-16835BCB4BB0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" xr2:uid="{7C97690C-9E7B-4D0E-86C0-16835BCB4BB0}"/>
   </bookViews>
   <sheets>
     <sheet name="scenarios" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="611" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="609" uniqueCount="145">
   <si>
     <t>Parameter</t>
   </si>
@@ -424,12 +424,6 @@
     <t>Buchkowski et al. 2024; Buchkowski and Schmitz 2022 for average weight from WE plots; 25% dry weight, 50% carbon</t>
   </si>
   <si>
-    <t>Konza Prarie LTER: https://kpbs.konza.k-state.edu provides range</t>
-  </si>
-  <si>
-    <t>unchanged from defaults- but can calculate from temp min/max (full temp range is 29.3C; tamp =14.65)</t>
-  </si>
-  <si>
     <t>unchanged from defaults; suggested min and max are from nelson et al 2004 (https://doi.org/10.1023/B:PLSO.0000020957.83641.62)</t>
   </si>
   <si>
@@ -469,13 +463,13 @@
     <t>Microarthropod</t>
   </si>
   <si>
-    <t>Need the SD of mean annual temperature, not temperature over the year.</t>
-  </si>
-  <si>
     <t>Topp et al. 2006 SBB; min/max made up</t>
   </si>
   <si>
     <t>Giovanni for NB</t>
+  </si>
+  <si>
+    <t>Nippert, J. 2023. APT02 Monthly temperature and precipitation records from Manhattan, KS ver 10. Environmental Data Initiative. https://doi.org/10.6073/pasta/d81b100b0737880b7950ec0d93625da9</t>
   </si>
 </sst>
 </file>
@@ -1024,9 +1018,6 @@
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" xfId="42" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1034,6 +1025,9 @@
     <xf numFmtId="0" fontId="19" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="42" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="43">
@@ -1476,20 +1470,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD4418A0-EB93-4361-AE80-4D25DF544368}">
   <dimension ref="A1:L72"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.26953125" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="22.7265625" customWidth="1"/>
-    <col min="4" max="4" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.54296875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="52.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="22.7109375" customWidth="1"/>
+    <col min="4" max="4" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="52.28515625" bestFit="1" customWidth="1"/>
     <col min="9" max="10" width="23" customWidth="1"/>
-    <col min="11" max="11" width="13.26953125" customWidth="1"/>
+    <col min="11" max="11" width="13.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1527,7 +1521,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
@@ -1561,7 +1555,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
@@ -1587,7 +1581,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>13</v>
       </c>
@@ -1610,7 +1604,7 @@
         <v>1</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="I4" s="1"/>
       <c r="J4" s="1" t="s">
@@ -1621,7 +1615,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>14</v>
       </c>
@@ -1647,7 +1641,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
@@ -1679,7 +1673,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>16</v>
       </c>
@@ -1711,7 +1705,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>17</v>
       </c>
@@ -1745,7 +1739,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>18</v>
       </c>
@@ -1783,7 +1777,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>19</v>
       </c>
@@ -1821,7 +1815,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
@@ -1851,7 +1845,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>21</v>
       </c>
@@ -1885,7 +1879,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>22</v>
       </c>
@@ -1920,7 +1914,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>23</v>
       </c>
@@ -1954,7 +1948,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>25</v>
       </c>
@@ -1988,7 +1982,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>27</v>
       </c>
@@ -2022,7 +2016,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="17" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>29</v>
       </c>
@@ -2051,7 +2045,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="18" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>30</v>
       </c>
@@ -2080,7 +2074,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="19" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>31</v>
       </c>
@@ -2109,7 +2103,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="20" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>32</v>
       </c>
@@ -2141,7 +2135,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="21" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>33</v>
       </c>
@@ -2171,7 +2165,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>11</v>
       </c>
@@ -2203,7 +2197,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>12</v>
       </c>
@@ -2231,7 +2225,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>13</v>
       </c>
@@ -2254,7 +2248,7 @@
         <v>1</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="I24" s="1" t="s">
         <v>124</v>
@@ -2267,7 +2261,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>14</v>
       </c>
@@ -2295,7 +2289,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>15</v>
       </c>
@@ -2327,7 +2321,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>16</v>
       </c>
@@ -2359,7 +2353,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>17</v>
       </c>
@@ -2391,7 +2385,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>18</v>
       </c>
@@ -2419,7 +2413,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>19</v>
       </c>
@@ -2447,7 +2441,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>20</v>
       </c>
@@ -2466,7 +2460,7 @@
         <v>10</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="I31" s="1" t="s">
         <v>124</v>
@@ -2479,7 +2473,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>21</v>
       </c>
@@ -2507,7 +2501,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>36</v>
       </c>
@@ -2538,7 +2532,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>37</v>
       </c>
@@ -2566,7 +2560,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>38</v>
       </c>
@@ -2594,7 +2588,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>39</v>
       </c>
@@ -2622,7 +2616,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="37" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>41</v>
       </c>
@@ -2652,7 +2646,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="38" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>42</v>
       </c>
@@ -2682,12 +2676,12 @@
         <v>59</v>
       </c>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>111</v>
@@ -2712,12 +2706,12 @@
         <v>59</v>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>111</v>
@@ -2742,12 +2736,12 @@
         <v>59</v>
       </c>
     </row>
-    <row r="41" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>117</v>
@@ -2776,12 +2770,12 @@
         <v>59</v>
       </c>
     </row>
-    <row r="42" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>117</v>
@@ -2806,12 +2800,12 @@
         <v>59</v>
       </c>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C43" s="1" t="s">
         <v>112</v>
@@ -2836,12 +2830,12 @@
         <v>59</v>
       </c>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C44" s="1" t="s">
         <v>113</v>
@@ -2866,12 +2860,12 @@
         <v>59</v>
       </c>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C45" s="1" t="s">
         <v>113</v>
@@ -2897,12 +2891,12 @@
         <v>59</v>
       </c>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>18</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C46" s="1" t="s">
         <v>114</v>
@@ -2931,12 +2925,12 @@
         <v>59</v>
       </c>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>19</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C47" s="1" t="s">
         <v>114</v>
@@ -2965,12 +2959,12 @@
         <v>59</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C48" s="1"/>
       <c r="D48" s="1">
@@ -2993,12 +2987,12 @@
         <v>59</v>
       </c>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>21</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C49" s="1" t="s">
         <v>115</v>
@@ -3027,12 +3021,12 @@
         <v>59</v>
       </c>
     </row>
-    <row r="50" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>36</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C50" s="1" t="s">
         <v>116</v>
@@ -3058,12 +3052,12 @@
         <v>59</v>
       </c>
     </row>
-    <row r="51" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>37</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>113</v>
@@ -3088,12 +3082,12 @@
         <v>59</v>
       </c>
     </row>
-    <row r="52" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>38</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C52" s="1" t="s">
         <v>113</v>
@@ -3118,12 +3112,12 @@
         <v>59</v>
       </c>
     </row>
-    <row r="53" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>39</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C53" s="1" t="s">
         <v>116</v>
@@ -3146,12 +3140,12 @@
         <v>59</v>
       </c>
     </row>
-    <row r="54" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>41</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C54" s="1" t="s">
         <v>113</v>
@@ -3176,12 +3170,12 @@
         <v>59</v>
       </c>
     </row>
-    <row r="55" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>42</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C55" s="1" t="s">
         <v>113</v>
@@ -3208,7 +3202,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="56" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>11</v>
       </c>
@@ -3219,21 +3213,17 @@
         <v>111</v>
       </c>
       <c r="D56" s="1">
-        <v>10</v>
-      </c>
-      <c r="E56" s="1"/>
-      <c r="F56" s="7">
-        <v>5</v>
-      </c>
-      <c r="G56" s="7">
-        <v>15</v>
-      </c>
-      <c r="H56" s="8" t="s">
-        <v>129</v>
-      </c>
-      <c r="I56" s="1" t="s">
+        <v>12.954660000000001</v>
+      </c>
+      <c r="E56" s="1">
+        <v>0.80562500000000004</v>
+      </c>
+      <c r="F56" s="7"/>
+      <c r="G56" s="7"/>
+      <c r="H56" s="12" t="s">
         <v>144</v>
       </c>
+      <c r="I56" s="1"/>
       <c r="J56" s="1" t="s">
         <v>61</v>
       </c>
@@ -3242,7 +3232,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="57" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>12</v>
       </c>
@@ -3252,20 +3242,18 @@
       <c r="C57" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D57" s="9">
-        <v>14.65</v>
-      </c>
-      <c r="E57" s="9">
-        <v>2</v>
+      <c r="D57" s="8">
+        <v>6.7212500000000004</v>
+      </c>
+      <c r="E57" s="8">
+        <v>0.63642900000000002</v>
       </c>
       <c r="F57" s="7"/>
       <c r="G57" s="7"/>
-      <c r="H57" s="7" t="s">
-        <v>130</v>
-      </c>
-      <c r="I57" s="1" t="s">
-        <v>73</v>
-      </c>
+      <c r="H57" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="I57" s="1"/>
       <c r="J57" s="1" t="s">
         <v>61</v>
       </c>
@@ -3274,7 +3262,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="58" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>13</v>
       </c>
@@ -3295,7 +3283,7 @@
         <v>0.2</v>
       </c>
       <c r="H58" s="7" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="I58" s="1" t="s">
         <v>73</v>
@@ -3308,7 +3296,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="59" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>14</v>
       </c>
@@ -3331,7 +3319,7 @@
         <v>0.2</v>
       </c>
       <c r="H59" s="7" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="I59" s="1" t="s">
         <v>73</v>
@@ -3344,7 +3332,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="60" spans="1:12" ht="58" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>15</v>
       </c>
@@ -3365,7 +3353,7 @@
         <v>100</v>
       </c>
       <c r="H60" s="7" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="I60" s="1" t="s">
         <v>73</v>
@@ -3378,7 +3366,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>16</v>
       </c>
@@ -3401,7 +3389,7 @@
         <v>0.4</v>
       </c>
       <c r="H61" s="7" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="I61" s="1" t="s">
         <v>73</v>
@@ -3414,7 +3402,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="62" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>17</v>
       </c>
@@ -3433,7 +3421,7 @@
       <c r="F62" s="7"/>
       <c r="G62" s="7"/>
       <c r="H62" s="7" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I62" s="1" t="s">
         <v>73</v>
@@ -3446,7 +3434,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>18</v>
       </c>
@@ -3469,7 +3457,7 @@
         <v>905.48</v>
       </c>
       <c r="H63" s="7" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I63" s="1" t="s">
         <v>73</v>
@@ -3482,7 +3470,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>19</v>
       </c>
@@ -3501,7 +3489,7 @@
       <c r="F64" s="7"/>
       <c r="G64" s="7"/>
       <c r="H64" s="7" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="I64" s="1" t="s">
         <v>73</v>
@@ -3514,7 +3502,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="65" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>20</v>
       </c>
@@ -3533,7 +3521,7 @@
         <v>9</v>
       </c>
       <c r="H65" s="7" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="I65" s="1" t="s">
         <v>73</v>
@@ -3546,7 +3534,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>21</v>
       </c>
@@ -3569,7 +3557,7 @@
         <v>1450</v>
       </c>
       <c r="H66" s="7" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="I66" s="1" t="s">
         <v>73</v>
@@ -3582,7 +3570,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="67" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>50</v>
       </c>
@@ -3592,20 +3580,20 @@
       <c r="C67" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D67" s="10">
+      <c r="D67" s="9">
         <v>1.384623481E-3</v>
       </c>
-      <c r="E67" s="10">
+      <c r="E67" s="9">
         <v>5.4402432010000005E-4</v>
       </c>
-      <c r="F67" s="10">
+      <c r="F67" s="9">
         <v>7.1040402530000003E-4</v>
       </c>
-      <c r="G67" s="10">
+      <c r="G67" s="9">
         <v>1.936006955E-3</v>
       </c>
       <c r="H67" s="7" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="I67" s="1" t="s">
         <v>73</v>
@@ -3618,7 +3606,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="68" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>51</v>
       </c>
@@ -3637,8 +3625,8 @@
       </c>
       <c r="F68" s="7"/>
       <c r="G68" s="7"/>
-      <c r="H68" s="11" t="s">
-        <v>141</v>
+      <c r="H68" s="10" t="s">
+        <v>139</v>
       </c>
       <c r="I68" s="1" t="s">
         <v>72</v>
@@ -3651,7 +3639,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>52</v>
       </c>
@@ -3672,7 +3660,7 @@
         <v>0.5</v>
       </c>
       <c r="H69" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="I69" s="1" t="s">
         <v>71</v>
@@ -3685,7 +3673,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>53</v>
       </c>
@@ -3704,7 +3692,7 @@
         <v>0.37</v>
       </c>
       <c r="H70" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="I70" s="1" t="s">
         <v>71</v>
@@ -3717,7 +3705,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="71" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>54</v>
       </c>
@@ -3749,7 +3737,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>55</v>
       </c>
@@ -3783,12 +3771,13 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="H56" r:id="rId1" display="https://kpbs.konza.k-state.edu/location/" xr:uid="{98608C20-26EF-4289-9EC6-968CD5323926}"/>
+    <hyperlink ref="H56" r:id="rId1" tooltip="https://doi.org/10.6073/pasta/d81b100b0737880b7950ec0d93625da9" display="https://doi.org/10.6073/pasta/d81b100b0737880b7950ec0d93625da9" xr:uid="{D2FB903B-7E32-4BBC-AD7C-E11D67A82484}"/>
+    <hyperlink ref="H57" r:id="rId2" tooltip="https://doi.org/10.6073/pasta/d81b100b0737880b7950ec0d93625da9" display="https://doi.org/10.6073/pasta/d81b100b0737880b7950ec0d93625da9" xr:uid="{F06A8F72-DA38-474C-B99F-04A053E543B4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId2"/>
+  <pageSetup orientation="portrait" r:id="rId3"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
   </tableParts>
 </worksheet>
 </file>
@@ -3796,16 +3785,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA0710C0-AB94-4FBF-AB29-E5085BC4F559}">
   <dimension ref="A1:F20"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.7265625" customWidth="1"/>
+    <col min="1" max="1" width="11.7109375" customWidth="1"/>
     <col min="2" max="2" width="20" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.81640625" customWidth="1"/>
+    <col min="3" max="3" width="13.85546875" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="35.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="35.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>75</v>
       </c>
@@ -3825,7 +3814,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>78</v>
       </c>
@@ -3846,7 +3835,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>78</v>
       </c>
@@ -3867,12 +3856,12 @@
         <v>59</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>78</v>
       </c>
-      <c r="B4" s="12" t="s">
-        <v>143</v>
+      <c r="B4" s="11" t="s">
+        <v>141</v>
       </c>
       <c r="C4" t="s">
         <v>9</v>
@@ -3887,7 +3876,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>78</v>
       </c>
@@ -3907,7 +3896,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>78</v>
       </c>
@@ -3927,7 +3916,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>78</v>
       </c>
@@ -3947,7 +3936,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>78</v>
       </c>
@@ -3967,7 +3956,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>78</v>
       </c>
@@ -3987,7 +3976,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>78</v>
       </c>
@@ -4007,7 +3996,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>94</v>
       </c>
@@ -4027,7 +4016,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>94</v>
       </c>
@@ -4047,7 +4036,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>94</v>
       </c>
@@ -4067,7 +4056,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>94</v>
       </c>
@@ -4087,7 +4076,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>94</v>
       </c>
@@ -4107,7 +4096,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>94</v>
       </c>
@@ -4127,7 +4116,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>94</v>
       </c>
@@ -4147,7 +4136,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>94</v>
       </c>
@@ -4167,7 +4156,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>94</v>
       </c>
@@ -4187,7 +4176,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>94</v>
       </c>
@@ -4215,13 +4204,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC182590-26D0-4168-8E7C-B448CD67FE47}">
   <dimension ref="A1:C25"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>76</v>
       </c>
@@ -4232,7 +4221,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -4243,7 +4232,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -4254,7 +4243,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -4265,7 +4254,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -4276,7 +4265,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -4287,7 +4276,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -4298,7 +4287,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -4309,7 +4298,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>6</v>
       </c>
@@ -4320,7 +4309,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>7</v>
       </c>
@@ -4331,7 +4320,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -4342,7 +4331,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -4353,7 +4342,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>10</v>
       </c>
@@ -4364,73 +4353,73 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>5</v>
       </c>
       <c r="B14" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C14">
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>6</v>
       </c>
       <c r="B15" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C15">
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>7</v>
       </c>
       <c r="B16" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C16">
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>8</v>
       </c>
       <c r="B17" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C17">
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>9</v>
       </c>
       <c r="B18" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C18">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>10</v>
       </c>
       <c r="B19" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C19">
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>5</v>
       </c>
@@ -4441,7 +4430,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>6</v>
       </c>
@@ -4452,7 +4441,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>7</v>
       </c>
@@ -4463,7 +4452,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>8</v>
       </c>
@@ -4474,7 +4463,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>9</v>
       </c>
@@ -4485,7 +4474,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>10</v>
       </c>

</xml_diff>